<commit_message>
Updated inventory - including new projectors
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/SystemDocumentation/github/uactechdoc/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AB8B916-AEBB-D640-BF2E-D82BF5D262FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD39B844-699B-9F40-8853-B611888D7FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3620" yWindow="3800" windowWidth="26620" windowHeight="15840" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
+    <workbookView xWindow="6620" yWindow="3800" windowWidth="23620" windowHeight="15840" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
   <sheets>
     <sheet name="network" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="279">
   <si>
     <t>NSCU-A004</t>
   </si>
@@ -906,6 +906,33 @@
   </si>
   <si>
     <t>KB0034</t>
+  </si>
+  <si>
+    <t>2604-2401</t>
+  </si>
+  <si>
+    <t>80-99-E7-4D-A8-5E</t>
+  </si>
+  <si>
+    <t>2604-2402</t>
+  </si>
+  <si>
+    <t>2604-2403</t>
+  </si>
+  <si>
+    <t>58-18-62-6B-1D-2B</t>
+  </si>
+  <si>
+    <t>192.168.201.20</t>
+  </si>
+  <si>
+    <t>192.168.201.21</t>
+  </si>
+  <si>
+    <t>192.168.201.22</t>
+  </si>
+  <si>
+    <t>58-18-62-6B-1D-2C</t>
   </si>
 </sst>
 </file>
@@ -1078,30 +1105,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="49" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="49" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1109,44 +1133,16 @@
     <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="10"/>
-        <name val="Calibri Light"/>
-        <family val="2"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri Light"/>
-        <family val="2"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -1232,6 +1228,24 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -1304,6 +1318,18 @@
         <scheme val="major"/>
       </font>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -1394,24 +1420,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}" name="Table1" displayName="Table1" ref="A1:K79" totalsRowShown="0" headerRowDxfId="12" dataDxfId="1">
-  <autoFilter ref="A1:K79" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}" name="Table1" displayName="Table1" ref="A1:K82" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A1:K82" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K74">
     <sortCondition ref="A2:A74"/>
     <sortCondition ref="B2:B74"/>
   </sortState>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{EF2C341F-E5C1-604C-942C-FB7E9F76F1CD}" name="AssetTag" dataDxfId="11"/>
-    <tableColumn id="13" xr3:uid="{41250547-1480-7146-952C-14798A4748DA}" name="NIC" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{5FD75CC6-F089-3C49-9E51-1565A7A8B99A}" name="MAC" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{2045B636-E35D-274F-BBD3-3FF47E121094}" name="Static-Reserved" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{10F05B30-ACC5-4444-9BCB-C4F83EBE82E8}" name="IP" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{D8CE5014-251A-FD49-B36C-92F7DAE750CB}" name="URL" dataDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{51987960-7E23-714D-8524-EE3E88D77DA5}" name="Services" dataDxfId="0" dataCellStyle="Hyperlink"/>
-    <tableColumn id="15" xr3:uid="{16C691FB-14A7-3342-ACEE-B45625DAF5F5}" name="Monitor" dataDxfId="5"/>
-    <tableColumn id="16" xr3:uid="{D6182358-29F5-9D47-8228-7124B0F8D7E0}" name="RelatedIssueId" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{6C62EAB0-EF42-3142-95A8-47F7C21989EE}" name="Usage" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{890B1E64-D13A-3548-8BF0-C28FFF87E38B}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{EF2C341F-E5C1-604C-942C-FB7E9F76F1CD}" name="AssetTag" dataDxfId="10"/>
+    <tableColumn id="13" xr3:uid="{41250547-1480-7146-952C-14798A4748DA}" name="NIC" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{5FD75CC6-F089-3C49-9E51-1565A7A8B99A}" name="MAC" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{2045B636-E35D-274F-BBD3-3FF47E121094}" name="Static-Reserved" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{10F05B30-ACC5-4444-9BCB-C4F83EBE82E8}" name="IP" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{D8CE5014-251A-FD49-B36C-92F7DAE750CB}" name="URL" dataDxfId="5"/>
+    <tableColumn id="17" xr3:uid="{51987960-7E23-714D-8524-EE3E88D77DA5}" name="Services" dataDxfId="4" dataCellStyle="Hyperlink"/>
+    <tableColumn id="15" xr3:uid="{16C691FB-14A7-3342-ACEE-B45625DAF5F5}" name="Monitor" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{D6182358-29F5-9D47-8228-7124B0F8D7E0}" name="RelatedIssueId" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{6C62EAB0-EF42-3142-95A8-47F7C21989EE}" name="Usage" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{890B1E64-D13A-3548-8BF0-C28FFF87E38B}" name="Notes" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1800,29 +1826,29 @@
       <c r="B3" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12" t="s">
+      <c r="D3" s="6"/>
+      <c r="E3" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
       <c r="H3" s="8" t="s">
         <v>178</v>
       </c>
       <c r="I3" s="9"/>
-      <c r="J3" s="11" t="s">
+      <c r="J3" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="K3" s="12"/>
+      <c r="K3" s="6"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="B4" s="11"/>
+      <c r="B4" s="5"/>
       <c r="C4" s="6" t="s">
         <v>166</v>
       </c>
@@ -1842,73 +1868,73 @@
       <c r="K4" s="6"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="5" t="s">
         <v>202</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12" t="s">
+      <c r="D5" s="6"/>
+      <c r="E5" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
       <c r="H5" s="8" t="s">
         <v>178</v>
       </c>
       <c r="I5" s="9"/>
-      <c r="J5" s="12" t="s">
+      <c r="J5" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="K5" s="12"/>
+      <c r="K5" s="6"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
       <c r="H6" s="8" t="s">
         <v>179</v>
       </c>
       <c r="I6" s="9"/>
-      <c r="J6" s="12" t="s">
+      <c r="J6" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="K6" s="12"/>
+      <c r="K6" s="6"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11" t="s">
+      <c r="B7" s="5"/>
+      <c r="C7" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12" t="s">
+      <c r="D7" s="6"/>
+      <c r="E7" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
       <c r="H7" s="8" t="s">
         <v>178</v>
       </c>
       <c r="I7" s="9"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
@@ -1955,46 +1981,46 @@
       <c r="B10" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12" t="s">
+      <c r="D10" s="6"/>
+      <c r="E10" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
       <c r="H10" s="8" t="s">
         <v>178</v>
       </c>
       <c r="I10" s="9"/>
-      <c r="J10" s="12" t="s">
+      <c r="J10" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="K10" s="12"/>
+      <c r="K10" s="6"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
       <c r="H11" s="8" t="s">
         <v>179</v>
       </c>
       <c r="I11" s="9"/>
-      <c r="J11" s="12" t="s">
+      <c r="J11" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="K11" s="12"/>
+      <c r="K11" s="6"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
@@ -2003,101 +2029,101 @@
       <c r="B12" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12" t="s">
+      <c r="D12" s="6"/>
+      <c r="E12" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
       <c r="H12" s="8" t="s">
         <v>178</v>
       </c>
       <c r="I12" s="9"/>
-      <c r="J12" s="12" t="s">
+      <c r="J12" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="K12" s="12"/>
+      <c r="K12" s="6"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
       <c r="H13" s="8" t="s">
         <v>179</v>
       </c>
       <c r="I13" s="9"/>
-      <c r="J13" s="12" t="s">
+      <c r="J13" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="K13" s="12"/>
+      <c r="K13" s="6"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="5" t="s">
         <v>229</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>203</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12" t="s">
+      <c r="D14" s="6"/>
+      <c r="E14" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
       <c r="H14" s="8" t="s">
         <v>178</v>
       </c>
       <c r="I14" s="9"/>
-      <c r="J14" s="12" t="s">
+      <c r="J14" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="K14" s="12"/>
+      <c r="K14" s="6"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
       <c r="H15" s="8" t="s">
         <v>179</v>
       </c>
       <c r="I15" s="9"/>
-      <c r="J15" s="12" t="s">
+      <c r="J15" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="K15" s="12"/>
+      <c r="K15" s="6"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
         <v>148</v>
       </c>
       <c r="B16" s="6"/>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="11" t="s">
         <v>146</v>
       </c>
       <c r="D16" s="6" t="s">
@@ -2115,15 +2141,15 @@
       <c r="J16" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="K16" s="14" t="s">
+      <c r="K16" s="12" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="15"/>
+      <c r="B17" s="13"/>
       <c r="C17" s="6" t="s">
         <v>21</v>
       </c>
@@ -2143,27 +2169,27 @@
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="B18" s="16"/>
-      <c r="C18" s="11" t="s">
+      <c r="B18" s="14"/>
+      <c r="C18" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12" t="s">
+      <c r="D18" s="6"/>
+      <c r="E18" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12" t="s">
+      <c r="F18" s="6"/>
+      <c r="G18" s="6" t="s">
         <v>245</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>178</v>
       </c>
       <c r="I18" s="9"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
@@ -2172,7 +2198,7 @@
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="15" t="s">
         <v>192</v>
       </c>
       <c r="F19" s="6"/>
@@ -2258,7 +2284,7 @@
         <v>7</v>
       </c>
       <c r="B23" s="5"/>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="16" t="s">
         <v>5</v>
       </c>
       <c r="D23" s="6"/>
@@ -2285,11 +2311,11 @@
       <c r="B24" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="15" t="s">
         <v>159</v>
       </c>
       <c r="D24" s="6"/>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="15" t="s">
         <v>183</v>
       </c>
       <c r="F24" s="6"/>
@@ -2312,7 +2338,7 @@
       <c r="B25" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="C25" s="17" t="s">
         <v>174</v>
       </c>
       <c r="D25" s="6"/>
@@ -2339,11 +2365,11 @@
       <c r="B26" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="15" t="s">
         <v>184</v>
       </c>
       <c r="D26" s="6"/>
-      <c r="E26" s="17" t="s">
+      <c r="E26" s="15" t="s">
         <v>185</v>
       </c>
       <c r="F26" s="6"/>
@@ -2453,7 +2479,7 @@
       <c r="J30" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="K30" s="14"/>
+      <c r="K30" s="12"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
@@ -2656,7 +2682,7 @@
       <c r="J40" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="K40" s="14"/>
+      <c r="K40" s="12"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" s="6" t="s">
@@ -2686,7 +2712,7 @@
       <c r="J41" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="K41" s="14"/>
+      <c r="K41" s="12"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" s="6" t="s">
@@ -2716,7 +2742,7 @@
       <c r="J42" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="K42" s="14"/>
+      <c r="K42" s="12"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" s="6" t="s">
@@ -2729,7 +2755,7 @@
       <c r="D43" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="E43" s="17" t="s">
+      <c r="E43" s="15" t="s">
         <v>135</v>
       </c>
       <c r="F43" s="7" t="str">
@@ -2776,7 +2802,7 @@
       <c r="J44" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="K44" s="14"/>
+      <c r="K44" s="12"/>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" s="6" t="s">
@@ -2898,27 +2924,27 @@
       <c r="K49" s="6"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A50" s="11" t="s">
+      <c r="A50" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B50" s="11"/>
-      <c r="C50" s="11" t="s">
+      <c r="B50" s="5"/>
+      <c r="C50" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D50" s="12"/>
-      <c r="E50" s="12" t="s">
+      <c r="D50" s="6"/>
+      <c r="E50" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="F50" s="12"/>
-      <c r="G50" s="12"/>
+      <c r="F50" s="6"/>
+      <c r="G50" s="6"/>
       <c r="H50" s="8" t="s">
         <v>178</v>
       </c>
       <c r="I50" s="9"/>
-      <c r="J50" s="12" t="s">
+      <c r="J50" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="K50" s="12"/>
+      <c r="K50" s="6"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
@@ -2943,7 +2969,7 @@
       <c r="J51" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="K51" s="14" t="s">
+      <c r="K51" s="12" t="s">
         <v>79</v>
       </c>
     </row>
@@ -2952,7 +2978,7 @@
         <v>60</v>
       </c>
       <c r="B52" s="6"/>
-      <c r="C52" s="27" t="s">
+      <c r="C52" s="23" t="s">
         <v>59</v>
       </c>
       <c r="D52" s="6" t="s">
@@ -2979,7 +3005,7 @@
         <v>54</v>
       </c>
       <c r="B53" s="6"/>
-      <c r="C53" s="27" t="s">
+      <c r="C53" s="23" t="s">
         <v>53</v>
       </c>
       <c r="D53" s="6" t="s">
@@ -3006,7 +3032,7 @@
         <v>52</v>
       </c>
       <c r="B54" s="6"/>
-      <c r="C54" s="27" t="s">
+      <c r="C54" s="23" t="s">
         <v>51</v>
       </c>
       <c r="D54" s="6" t="s">
@@ -3033,7 +3059,7 @@
         <v>50</v>
       </c>
       <c r="B55" s="6"/>
-      <c r="C55" s="27" t="s">
+      <c r="C55" s="23" t="s">
         <v>48</v>
       </c>
       <c r="D55" s="6" t="s">
@@ -3056,10 +3082,10 @@
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A56" s="20" t="s">
+      <c r="A56" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B56" s="20"/>
+      <c r="B56" s="10"/>
       <c r="C56" s="6" t="s">
         <v>56</v>
       </c>
@@ -3120,7 +3146,7 @@
         <v>122</v>
       </c>
       <c r="B58" s="6"/>
-      <c r="C58" s="21" t="s">
+      <c r="C58" s="18" t="s">
         <v>120</v>
       </c>
       <c r="D58" s="6" t="s">
@@ -3176,7 +3202,7 @@
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A60" s="22" t="s">
+      <c r="A60" s="19" t="s">
         <v>114</v>
       </c>
       <c r="B60" s="6"/>
@@ -3236,7 +3262,7 @@
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A62" s="23" t="s">
+      <c r="A62" s="20" t="s">
         <v>240</v>
       </c>
       <c r="B62" s="5"/>
@@ -3272,7 +3298,7 @@
       </c>
       <c r="F63" s="6"/>
       <c r="G63" s="6"/>
-      <c r="H63" s="24" t="s">
+      <c r="H63" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I63" s="9"/>
@@ -3300,14 +3326,14 @@
         <v>http://192.168.206.7</v>
       </c>
       <c r="G64" s="7"/>
-      <c r="H64" s="24" t="s">
+      <c r="H64" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I64" s="9"/>
       <c r="J64" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="K64" s="14" t="s">
+      <c r="K64" s="12" t="s">
         <v>87</v>
       </c>
     </row>
@@ -3330,14 +3356,14 @@
         <v>http://192.168.0.192</v>
       </c>
       <c r="G65" s="7"/>
-      <c r="H65" s="24" t="s">
+      <c r="H65" s="21" t="s">
         <v>179</v>
       </c>
       <c r="I65" s="9"/>
       <c r="J65" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="K65" s="14" t="s">
+      <c r="K65" s="12" t="s">
         <v>87</v>
       </c>
     </row>
@@ -3357,7 +3383,7 @@
       </c>
       <c r="F66" s="6"/>
       <c r="G66" s="6"/>
-      <c r="H66" s="24" t="s">
+      <c r="H66" s="21" t="s">
         <v>179</v>
       </c>
       <c r="I66" s="9"/>
@@ -3384,14 +3410,14 @@
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6"/>
-      <c r="H67" s="24" t="s">
+      <c r="H67" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I67" s="9"/>
       <c r="J67" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="K67" s="14" t="s">
+      <c r="K67" s="12" t="s">
         <v>79</v>
       </c>
     </row>
@@ -3414,14 +3440,14 @@
         <v>ftp://192.168.0.189</v>
       </c>
       <c r="G68" s="7"/>
-      <c r="H68" s="24" t="s">
+      <c r="H68" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I68" s="9"/>
       <c r="J68" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="K68" s="14" t="s">
+      <c r="K68" s="12" t="s">
         <v>79</v>
       </c>
     </row>
@@ -3444,14 +3470,14 @@
         <v>ftp://192.168.0.190</v>
       </c>
       <c r="G69" s="7"/>
-      <c r="H69" s="24" t="s">
+      <c r="H69" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I69" s="9"/>
       <c r="J69" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="K69" s="14" t="s">
+      <c r="K69" s="12" t="s">
         <v>79</v>
       </c>
     </row>
@@ -3476,7 +3502,7 @@
       <c r="G70" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="H70" s="24" t="s">
+      <c r="H70" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I70" s="9"/>
@@ -3508,7 +3534,7 @@
       <c r="G71" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="H71" s="24" t="s">
+      <c r="H71" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I71" s="9"/>
@@ -3540,7 +3566,7 @@
       <c r="G72" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="H72" s="24" t="s">
+      <c r="H72" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I72" s="9"/>
@@ -3572,7 +3598,7 @@
       <c r="G73" s="7" t="s">
         <v>242</v>
       </c>
-      <c r="H73" s="24" t="s">
+      <c r="H73" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I73" s="9"/>
@@ -3595,7 +3621,7 @@
       <c r="E74" s="6"/>
       <c r="F74" s="6"/>
       <c r="G74" s="6"/>
-      <c r="H74" s="24" t="s">
+      <c r="H74" s="21" t="s">
         <v>179</v>
       </c>
       <c r="I74" s="9"/>
@@ -3607,175 +3633,244 @@
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A75" s="11" t="s">
+      <c r="A75" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="B75" s="11"/>
+      <c r="B75" s="5"/>
       <c r="C75" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="D75" s="12"/>
-      <c r="E75" s="12" t="s">
+      <c r="D75" s="6"/>
+      <c r="E75" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="F75" s="12"/>
-      <c r="G75" s="25" t="s">
+      <c r="F75" s="6"/>
+      <c r="G75" s="22" t="s">
         <v>245</v>
       </c>
-      <c r="H75" s="24" t="s">
+      <c r="H75" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I75" s="9"/>
-      <c r="J75" s="12" t="s">
+      <c r="J75" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="K75" s="12"/>
+      <c r="K75" s="6"/>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A76" s="11" t="s">
+      <c r="A76" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="B76" s="11"/>
-      <c r="C76" s="11"/>
-      <c r="D76" s="12"/>
-      <c r="E76" s="12"/>
-      <c r="F76" s="12"/>
-      <c r="G76" s="25"/>
-      <c r="H76" s="24" t="s">
+      <c r="B76" s="5"/>
+      <c r="C76" s="5"/>
+      <c r="D76" s="6"/>
+      <c r="E76" s="6"/>
+      <c r="F76" s="6"/>
+      <c r="G76" s="22"/>
+      <c r="H76" s="21" t="s">
         <v>179</v>
       </c>
       <c r="I76" s="9"/>
-      <c r="J76" s="12"/>
-      <c r="K76" s="12"/>
+      <c r="J76" s="6"/>
+      <c r="K76" s="6"/>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A77" s="11" t="s">
+      <c r="A77" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="B77" s="11"/>
-      <c r="C77" s="11"/>
-      <c r="D77" s="12"/>
-      <c r="E77" s="12" t="s">
+      <c r="B77" s="5"/>
+      <c r="C77" s="5"/>
+      <c r="D77" s="6"/>
+      <c r="E77" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="F77" s="12"/>
-      <c r="G77" s="25"/>
-      <c r="H77" s="24"/>
+      <c r="F77" s="6"/>
+      <c r="G77" s="22"/>
+      <c r="H77" s="21"/>
       <c r="I77" s="9"/>
-      <c r="J77" s="12"/>
-      <c r="K77" s="12"/>
+      <c r="J77" s="6"/>
+      <c r="K77" s="6"/>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A78" s="11" t="s">
+      <c r="A78" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="B78" s="11"/>
-      <c r="C78" s="11"/>
-      <c r="D78" s="12"/>
-      <c r="E78" s="12" t="s">
+      <c r="B78" s="5"/>
+      <c r="C78" s="5"/>
+      <c r="D78" s="6"/>
+      <c r="E78" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="F78" s="12"/>
-      <c r="G78" s="25" t="s">
+      <c r="F78" s="6"/>
+      <c r="G78" s="22" t="s">
         <v>261</v>
       </c>
-      <c r="H78" s="24" t="s">
+      <c r="H78" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I78" s="9"/>
-      <c r="J78" s="12" t="s">
+      <c r="J78" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="K78" s="12"/>
+      <c r="K78" s="6"/>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A79" s="11" t="s">
+      <c r="A79" s="5" t="s">
         <v>262</v>
       </c>
-      <c r="B79" s="11"/>
-      <c r="C79" s="11"/>
-      <c r="D79" s="12"/>
-      <c r="E79" s="26" t="s">
+      <c r="B79" s="5"/>
+      <c r="C79" s="5"/>
+      <c r="D79" s="6"/>
+      <c r="E79" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="F79" s="12"/>
-      <c r="G79" s="25" t="s">
+      <c r="F79" s="6"/>
+      <c r="G79" s="22" t="s">
         <v>260</v>
       </c>
-      <c r="H79" s="24" t="s">
+      <c r="H79" s="21" t="s">
         <v>178</v>
       </c>
       <c r="I79" s="9"/>
-      <c r="J79" s="12" t="s">
+      <c r="J79" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="K79" s="12"/>
+      <c r="K79" s="6"/>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="H80"/>
-      <c r="I80"/>
-    </row>
-    <row r="81" spans="8:9" x14ac:dyDescent="0.2">
-      <c r="H81"/>
-      <c r="I81"/>
-    </row>
-    <row r="82" spans="8:9" x14ac:dyDescent="0.2">
-      <c r="H82"/>
-      <c r="I82"/>
-    </row>
-    <row r="83" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="A80" s="24" t="s">
+        <v>270</v>
+      </c>
+      <c r="B80" s="24"/>
+      <c r="C80" s="24" t="s">
+        <v>271</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E80" s="25" t="s">
+        <v>275</v>
+      </c>
+      <c r="F80" s="25"/>
+      <c r="G80" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="H80" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="I80" s="26"/>
+      <c r="J80" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="K80" s="25"/>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A81" s="24" t="s">
+        <v>272</v>
+      </c>
+      <c r="B81" s="24"/>
+      <c r="C81" s="24" t="s">
+        <v>274</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E81" s="25" t="s">
+        <v>276</v>
+      </c>
+      <c r="F81" s="25"/>
+      <c r="G81" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="H81" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="I81" s="26"/>
+      <c r="J81" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="K81" s="25"/>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A82" s="24" t="s">
+        <v>273</v>
+      </c>
+      <c r="B82" s="24"/>
+      <c r="C82" s="24" t="s">
+        <v>278</v>
+      </c>
+      <c r="D82" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E82" s="25" t="s">
+        <v>277</v>
+      </c>
+      <c r="F82" s="25"/>
+      <c r="G82" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="H82" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="I82" s="26"/>
+      <c r="J82" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="K82" s="25"/>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H83"/>
       <c r="I83"/>
     </row>
-    <row r="84" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H84"/>
       <c r="I84"/>
     </row>
-    <row r="85" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H85"/>
       <c r="I85"/>
     </row>
-    <row r="86" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H86"/>
       <c r="I86"/>
     </row>
-    <row r="87" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H87"/>
       <c r="I87"/>
     </row>
-    <row r="88" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H88"/>
       <c r="I88"/>
     </row>
-    <row r="89" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H89"/>
       <c r="I89"/>
     </row>
-    <row r="90" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H90"/>
       <c r="I90"/>
     </row>
-    <row r="91" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H91"/>
       <c r="I91"/>
     </row>
-    <row r="92" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H92"/>
       <c r="I92"/>
     </row>
-    <row r="93" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H93"/>
       <c r="I93"/>
     </row>
-    <row r="94" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H94"/>
       <c r="I94"/>
     </row>
-    <row r="95" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H95"/>
       <c r="I95"/>
     </row>
-    <row r="96" spans="8:9" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H96"/>
       <c r="I96"/>
     </row>

</xml_diff>

<commit_message>
removed old projectors from monitor list
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD39B844-699B-9F40-8853-B611888D7FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4914360D-6D87-EA46-BF16-BB4B328DCC53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6620" yWindow="3800" windowWidth="23620" windowHeight="15840" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
@@ -1105,7 +1105,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1134,9 +1134,6 @@
     <xf numFmtId="49" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3535,7 +3532,7 @@
         <v>242</v>
       </c>
       <c r="H71" s="21" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I71" s="9"/>
       <c r="J71" s="6" t="s">
@@ -3567,7 +3564,7 @@
         <v>242</v>
       </c>
       <c r="H72" s="21" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I72" s="9"/>
       <c r="J72" s="6" t="s">
@@ -3599,7 +3596,7 @@
         <v>242</v>
       </c>
       <c r="H73" s="21" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I73" s="9"/>
       <c r="J73" s="6" t="s">
@@ -3738,85 +3735,85 @@
       <c r="K79" s="6"/>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A80" s="24" t="s">
+      <c r="A80" s="5" t="s">
         <v>270</v>
       </c>
-      <c r="B80" s="24"/>
-      <c r="C80" s="24" t="s">
+      <c r="B80" s="5"/>
+      <c r="C80" s="5" t="s">
         <v>271</v>
       </c>
       <c r="D80" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E80" s="25" t="s">
+      <c r="E80" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="F80" s="25"/>
+      <c r="F80" s="6"/>
       <c r="G80" s="7" t="s">
         <v>242</v>
       </c>
       <c r="H80" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="I80" s="26"/>
+      <c r="I80" s="9"/>
       <c r="J80" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="K80" s="25"/>
+      <c r="K80" s="6"/>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A81" s="24" t="s">
+      <c r="A81" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="B81" s="24"/>
-      <c r="C81" s="24" t="s">
+      <c r="B81" s="5"/>
+      <c r="C81" s="5" t="s">
         <v>274</v>
       </c>
       <c r="D81" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E81" s="25" t="s">
+      <c r="E81" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="F81" s="25"/>
+      <c r="F81" s="6"/>
       <c r="G81" s="7" t="s">
         <v>242</v>
       </c>
       <c r="H81" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="I81" s="26"/>
+      <c r="I81" s="9"/>
       <c r="J81" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="K81" s="25"/>
+      <c r="K81" s="6"/>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A82" s="24" t="s">
+      <c r="A82" s="5" t="s">
         <v>273</v>
       </c>
-      <c r="B82" s="24"/>
-      <c r="C82" s="24" t="s">
+      <c r="B82" s="5"/>
+      <c r="C82" s="5" t="s">
         <v>278</v>
       </c>
       <c r="D82" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E82" s="25" t="s">
+      <c r="E82" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="F82" s="25"/>
+      <c r="F82" s="6"/>
       <c r="G82" s="7" t="s">
         <v>242</v>
       </c>
       <c r="H82" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="I82" s="26"/>
+      <c r="I82" s="9"/>
       <c r="J82" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="K82" s="25"/>
+      <c r="K82" s="6"/>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H83"/>

</xml_diff>

<commit_message>
Added configuration for NDI routes
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA31CF37-BC5D-744B-9006-89A0AE02ED27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B885147-4BDA-A94C-B58B-86DCE4AA399D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8320" yWindow="1460" windowWidth="21920" windowHeight="18180" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="294">
   <si>
     <t>NSCU-A004</t>
   </si>
@@ -389,9 +389,6 @@
     <t>ZVKU-A003</t>
   </si>
   <si>
-    <t>00:1d:56:03:81:45</t>
-  </si>
-  <si>
     <t>Matrix Switch</t>
   </si>
   <si>
@@ -653,9 +650,6 @@
     <t>USB Nic</t>
   </si>
   <si>
-    <t>192.168.206.7</t>
-  </si>
-  <si>
     <t>192.168.0.210</t>
   </si>
   <si>
@@ -933,6 +927,57 @@
   </si>
   <si>
     <t>KB0041</t>
+  </si>
+  <si>
+    <t>2603-1203</t>
+  </si>
+  <si>
+    <t>98-BA-5F-91-07-6A</t>
+  </si>
+  <si>
+    <t>Omada</t>
+  </si>
+  <si>
+    <t>192.168.201.105</t>
+  </si>
+  <si>
+    <t>7C-2E-0D-A8-52-4F</t>
+  </si>
+  <si>
+    <t>7C-2E-0D-20-68-69</t>
+  </si>
+  <si>
+    <t>00-1D-56-04-CC-E3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00:1d:56:03:81:45 </t>
+  </si>
+  <si>
+    <t>Unknown Mac</t>
+  </si>
+  <si>
+    <t>192.168.201.110</t>
+  </si>
+  <si>
+    <t>2411-1330</t>
+  </si>
+  <si>
+    <t>2507-1000</t>
+  </si>
+  <si>
+    <t>D0-C8-57-81-F2-19</t>
+  </si>
+  <si>
+    <t>NDI</t>
+  </si>
+  <si>
+    <t>D0-C8-57-82-74-B9</t>
+  </si>
+  <si>
+    <t>192.168.204.32</t>
+  </si>
+  <si>
+    <t>192.168.204.31</t>
   </si>
 </sst>
 </file>
@@ -1105,7 +1150,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1134,6 +1179,10 @@
     <xf numFmtId="49" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1417,8 +1466,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}" name="Table1" displayName="Table1" ref="A1:K82" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:K82" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}" name="Table1" displayName="Table1" ref="A1:K86" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A1:K86" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K73">
     <sortCondition ref="A2:A73"/>
     <sortCondition ref="B2:B73"/>
@@ -1757,50 +1806,50 @@
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>149</v>
-      </c>
       <c r="K1" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F2" s="7" t="str">
         <f>CONCATENATE("http://", E2)</f>
@@ -1808,126 +1857,126 @@
       </c>
       <c r="G2" s="7"/>
       <c r="H2" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I2" s="9"/>
       <c r="J2" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="6" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I3" s="9"/>
       <c r="J3" s="5" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="K3" s="6"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I4" s="9"/>
       <c r="J4" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K4" s="6"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>197</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>199</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I5" s="9"/>
       <c r="J5" s="6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K5" s="6"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I6" s="9"/>
       <c r="J6" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="K6" s="6"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
       <c r="H7" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I7" s="9"/>
       <c r="J7" s="6"/>
@@ -1935,18 +1984,20 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B8" s="5"/>
-      <c r="C8" s="6"/>
+      <c r="C8" s="6" t="s">
+        <v>281</v>
+      </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
       <c r="H8" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I8" s="9"/>
       <c r="J8" s="6"/>
@@ -1954,18 +2005,20 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B9" s="5"/>
-      <c r="C9" s="6"/>
+      <c r="C9" s="6" t="s">
+        <v>282</v>
+      </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
       <c r="H9" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="6"/>
@@ -1973,170 +2026,170 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
       <c r="H10" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I10" s="9"/>
       <c r="J10" s="6" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="K10" s="6"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
       <c r="H11" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I11" s="9"/>
       <c r="J11" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
       <c r="H12" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I12" s="9"/>
       <c r="J12" s="6" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="K12" s="6"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
       <c r="H13" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I13" s="9"/>
       <c r="J13" s="6" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="K13" s="6"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="6"/>
       <c r="H14" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I14" s="9"/>
       <c r="J14" s="6" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="K14" s="6"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
       <c r="H15" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I15" s="9"/>
       <c r="J15" s="6" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="K15" s="6"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6"/>
       <c r="H16" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I16" s="9"/>
       <c r="J16" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K16" s="12" t="s">
         <v>79</v>
@@ -2155,7 +2208,7 @@
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I17" s="9"/>
       <c r="J17" s="6" t="s">
@@ -2167,22 +2220,22 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B18" s="14"/>
       <c r="C18" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="6" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I18" s="9"/>
       <c r="J18" s="6"/>
@@ -2196,12 +2249,12 @@
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="15" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="6"/>
       <c r="H19" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I19" s="9"/>
       <c r="J19" s="6" t="s">
@@ -2214,21 +2267,21 @@
         <v>7</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F20" s="7"/>
       <c r="G20" s="7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I20" s="9"/>
       <c r="J20" s="6"/>
@@ -2239,21 +2292,21 @@
         <v>7</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C21" s="5"/>
       <c r="D21" s="6"/>
       <c r="E21" s="6" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
       <c r="H21" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I21" s="9"/>
       <c r="J21" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="K21" s="6"/>
     </row>
@@ -2262,7 +2315,7 @@
         <v>7</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C22" s="5"/>
       <c r="D22" s="6"/>
@@ -2270,7 +2323,7 @@
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
       <c r="H22" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I22" s="9"/>
       <c r="J22" s="6"/>
@@ -2293,7 +2346,7 @@
       </c>
       <c r="G23" s="6"/>
       <c r="H23" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I23" s="9"/>
       <c r="J23" s="6" t="s">
@@ -2306,25 +2359,25 @@
         <v>1</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I24" s="9"/>
       <c r="J24" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K24" s="6"/>
     </row>
@@ -2333,25 +2386,25 @@
         <v>1</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I25" s="9"/>
       <c r="J25" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K25" s="6"/>
     </row>
@@ -2360,83 +2413,83 @@
         <v>1</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="15" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I26" s="9"/>
       <c r="J26" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="K26" s="6"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
       <c r="H27" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I27" s="9"/>
       <c r="J27" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K27" s="6"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D28" s="6"/>
       <c r="E28" s="6" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F28" s="7"/>
       <c r="G28" s="7" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I28" s="9"/>
       <c r="J28" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K28" s="6"/>
     </row>
     <row r="29" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -2445,36 +2498,36 @@
       <c r="F29" s="7"/>
       <c r="G29" s="7"/>
       <c r="H29" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="K29" s="6"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E30" s="6"/>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
       <c r="H30" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I30" s="9"/>
       <c r="J30" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K30" s="12"/>
     </row>
@@ -2489,7 +2542,7 @@
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
       <c r="H31" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I31" s="9"/>
       <c r="J31" s="6" t="s">
@@ -2508,7 +2561,7 @@
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
       <c r="H32" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I32" s="9"/>
       <c r="J32" s="6" t="s">
@@ -2527,7 +2580,7 @@
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
       <c r="H33" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I33" s="9"/>
       <c r="J33" s="6" t="s">
@@ -2546,7 +2599,7 @@
       <c r="F34" s="6"/>
       <c r="G34" s="6"/>
       <c r="H34" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I34" s="9"/>
       <c r="J34" s="6" t="s">
@@ -2565,7 +2618,7 @@
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
       <c r="H35" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I35" s="9"/>
       <c r="J35" s="6" t="s">
@@ -2586,7 +2639,7 @@
       <c r="F36" s="6"/>
       <c r="G36" s="6"/>
       <c r="H36" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I36" s="9"/>
       <c r="J36" s="6" t="s">
@@ -2605,7 +2658,7 @@
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
       <c r="H37" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I37" s="9"/>
       <c r="J37" s="6" t="s">
@@ -2624,7 +2677,7 @@
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
       <c r="H38" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I38" s="9"/>
       <c r="J38" s="6" t="s">
@@ -2643,7 +2696,7 @@
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
       <c r="H39" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I39" s="9"/>
       <c r="J39" s="6" t="s">
@@ -2657,27 +2710,27 @@
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F40" s="7" t="str">
         <f>CONCATENATE("http://", E40)</f>
         <v>http://192.168.0.22</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I40" s="9"/>
       <c r="J40" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K40" s="12"/>
     </row>
@@ -2687,27 +2740,27 @@
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F41" s="7" t="str">
         <f>CONCATENATE("http://", E41)</f>
         <v>http://192.168.0.23</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I41" s="9"/>
       <c r="J41" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K41" s="12"/>
     </row>
@@ -2717,27 +2770,27 @@
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F42" s="7" t="str">
         <f>CONCATENATE("http://", E42)</f>
         <v>http://192.168.0.24</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I42" s="9"/>
       <c r="J42" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K42" s="12"/>
     </row>
@@ -2747,27 +2800,27 @@
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E43" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F43" s="7" t="str">
         <f>CONCATENATE("http://", E43)</f>
         <v>http://192.168.0.25</v>
       </c>
       <c r="G43" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I43" s="9"/>
       <c r="J43" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K43" s="6"/>
     </row>
@@ -2777,27 +2830,27 @@
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F44" s="7" t="str">
         <f>CONCATENATE("http://", E44)</f>
         <v>http://192.168.0.26</v>
       </c>
       <c r="G44" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I44" s="9"/>
       <c r="J44" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K44" s="12"/>
     </row>
@@ -2806,7 +2859,7 @@
         <v>46</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>45</v>
@@ -2820,14 +2873,14 @@
       <c r="F45" s="6"/>
       <c r="G45" s="6"/>
       <c r="H45" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I45" s="9"/>
       <c r="J45" s="6" t="s">
         <v>42</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
@@ -2835,7 +2888,7 @@
         <v>46</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="6"/>
@@ -2843,11 +2896,11 @@
       <c r="F46" s="6"/>
       <c r="G46" s="7"/>
       <c r="H46" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I46" s="9"/>
       <c r="J46" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="K46" s="6"/>
     </row>
@@ -2856,7 +2909,7 @@
         <v>43</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>41</v>
@@ -2870,14 +2923,14 @@
       <c r="F47" s="6"/>
       <c r="G47" s="6"/>
       <c r="H47" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I47" s="9"/>
       <c r="J47" s="6" t="s">
         <v>42</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
@@ -2885,7 +2938,7 @@
         <v>43</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="6"/>
@@ -2893,11 +2946,11 @@
       <c r="F48" s="6"/>
       <c r="G48" s="7"/>
       <c r="H48" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I48" s="9"/>
       <c r="J48" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="K48" s="6"/>
     </row>
@@ -2930,16 +2983,16 @@
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="6"/>
       <c r="H50" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I50" s="9"/>
       <c r="J50" s="6" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="K50" s="6"/>
     </row>
@@ -2955,15 +3008,15 @@
         <v>40</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="F51" s="6"/>
       <c r="G51" s="6"/>
       <c r="H51" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I51" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J51" s="6" t="s">
         <v>49</v>
@@ -2984,15 +3037,15 @@
         <v>40</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
       <c r="H52" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I52" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J52" s="6" t="s">
         <v>49</v>
@@ -3013,15 +3066,15 @@
         <v>40</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="F53" s="6"/>
       <c r="G53" s="6"/>
       <c r="H53" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I53" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J53" s="6" t="s">
         <v>49</v>
@@ -3042,15 +3095,15 @@
         <v>40</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="F54" s="6"/>
       <c r="G54" s="6"/>
       <c r="H54" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I54" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J54" s="6" t="s">
         <v>49</v>
@@ -3078,10 +3131,10 @@
         <v>http://192.168.0.197:8080</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="H55" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I55" s="9"/>
       <c r="J55" s="6" t="s">
@@ -3091,17 +3144,17 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D56" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F56" s="7" t="str">
         <f>CONCATENATE("http://", E56)</f>
@@ -3109,11 +3162,11 @@
       </c>
       <c r="G56" s="7"/>
       <c r="H56" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I56" s="9"/>
       <c r="J56" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K56" s="6" t="s">
         <v>75</v>
@@ -3121,17 +3174,17 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="18" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D57" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F57" s="7" t="str">
         <f>CONCATENATE("http://", E57)</f>
@@ -3139,11 +3192,11 @@
       </c>
       <c r="G57" s="7"/>
       <c r="H57" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I57" s="9"/>
       <c r="J57" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K57" s="6" t="s">
         <v>71</v>
@@ -3151,17 +3204,17 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D58" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F58" s="7" t="str">
         <f>CONCATENATE("http://", E58)</f>
@@ -3169,13 +3222,13 @@
       </c>
       <c r="G58" s="7"/>
       <c r="H58" s="8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I58" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K58" s="6" t="s">
         <v>66</v>
@@ -3183,17 +3236,17 @@
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" s="19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B59" s="6"/>
       <c r="C59" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F59" s="7" t="str">
         <f>CONCATENATE("http://", E59)</f>
@@ -3201,29 +3254,29 @@
       </c>
       <c r="G59" s="7"/>
       <c r="H59" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I59" s="9"/>
       <c r="J59" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F60" s="7" t="str">
         <f>CONCATENATE("http://", E60)</f>
@@ -3231,19 +3284,19 @@
       </c>
       <c r="G60" s="7"/>
       <c r="H60" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I60" s="9"/>
       <c r="J60" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K60" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" s="20" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B61" s="5"/>
       <c r="C61" s="6" t="s">
@@ -3251,12 +3304,12 @@
       </c>
       <c r="D61" s="6"/>
       <c r="E61" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F61" s="6"/>
       <c r="G61" s="6"/>
       <c r="H61" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I61" s="9"/>
       <c r="J61" s="6" t="s">
@@ -3266,52 +3319,54 @@
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B62" s="5"/>
       <c r="C62" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F62" s="6"/>
       <c r="G62" s="6"/>
       <c r="H62" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I62" s="9"/>
       <c r="J62" s="6" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K62" s="6"/>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B63" s="6"/>
       <c r="C63" s="6" t="s">
-        <v>97</v>
+        <v>283</v>
       </c>
       <c r="D63" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>185</v>
+        <v>286</v>
       </c>
       <c r="F63" s="7" t="str">
         <f>CONCATENATE("http://", E63)</f>
-        <v>http://192.168.206.7</v>
-      </c>
-      <c r="G63" s="7"/>
+        <v>http://192.168.201.110</v>
+      </c>
+      <c r="G63" s="27" t="s">
+        <v>238</v>
+      </c>
       <c r="H63" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I63" s="9"/>
       <c r="J63" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K63" s="12" t="s">
         <v>87</v>
@@ -3337,7 +3392,7 @@
       </c>
       <c r="G64" s="7"/>
       <c r="H64" s="21" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I64" s="9"/>
       <c r="J64" s="6" t="s">
@@ -3364,7 +3419,7 @@
       <c r="F65" s="6"/>
       <c r="G65" s="6"/>
       <c r="H65" s="21" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I65" s="9"/>
       <c r="J65" s="6" t="s">
@@ -3376,28 +3431,28 @@
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B66" s="6"/>
       <c r="C66" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D66" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F66" s="6"/>
       <c r="G66" s="6"/>
       <c r="H66" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I66" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J66" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K66" s="12" t="s">
         <v>79</v>
@@ -3423,10 +3478,10 @@
       </c>
       <c r="G67" s="7"/>
       <c r="H67" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I67" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J67" s="6" t="s">
         <v>82</v>
@@ -3455,10 +3510,10 @@
       </c>
       <c r="G68" s="7"/>
       <c r="H68" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I68" s="9" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J68" s="6" t="s">
         <v>82</v>
@@ -3486,13 +3541,13 @@
         <v>http://192.168.0.183</v>
       </c>
       <c r="G69" s="7" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H69" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I69" s="9" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="J69" s="6" t="s">
         <v>64</v>
@@ -3520,10 +3575,10 @@
         <v>http://192.168.0.193</v>
       </c>
       <c r="G70" s="7" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H70" s="21" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I70" s="9"/>
       <c r="J70" s="6" t="s">
@@ -3552,10 +3607,10 @@
         <v>http://192.168.0.194</v>
       </c>
       <c r="G71" s="7" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H71" s="21" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I71" s="9"/>
       <c r="J71" s="6" t="s">
@@ -3584,10 +3639,10 @@
         <v>http://192.168.0.195</v>
       </c>
       <c r="G72" s="7" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H72" s="21" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I72" s="9"/>
       <c r="J72" s="6" t="s">
@@ -3610,7 +3665,7 @@
       <c r="F73" s="6"/>
       <c r="G73" s="6"/>
       <c r="H73" s="21" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I73" s="9"/>
       <c r="J73" s="6" t="s">
@@ -3622,32 +3677,32 @@
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B74" s="5"/>
       <c r="C74" s="6" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D74" s="6"/>
       <c r="E74" s="6" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="F74" s="6"/>
       <c r="G74" s="22" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H74" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I74" s="9"/>
       <c r="J74" s="6" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="K74" s="6"/>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A75" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B75" s="5"/>
       <c r="C75" s="5"/>
@@ -3656,7 +3711,7 @@
       <c r="F75" s="6"/>
       <c r="G75" s="22"/>
       <c r="H75" s="21" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I75" s="9"/>
       <c r="J75" s="6"/>
@@ -3664,13 +3719,13 @@
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A76" s="5" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B76" s="5"/>
       <c r="C76" s="5"/>
       <c r="D76" s="6"/>
       <c r="E76" s="6" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="F76" s="6"/>
       <c r="G76" s="22"/>
@@ -3681,70 +3736,70 @@
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B77" s="5"/>
       <c r="C77" s="5"/>
       <c r="D77" s="6"/>
       <c r="E77" s="6" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="F77" s="6"/>
       <c r="G77" s="22" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H77" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I77" s="9"/>
       <c r="J77" s="6" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="K77" s="6"/>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78" s="5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B78" s="5"/>
       <c r="C78" s="5"/>
       <c r="D78" s="6"/>
       <c r="E78" s="15" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="F78" s="6"/>
       <c r="G78" s="22" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H78" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I78" s="9"/>
       <c r="J78" s="6" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="K78" s="6"/>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B79" s="5"/>
       <c r="C79" s="5" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D79" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="F79" s="6"/>
       <c r="G79" s="7" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H79" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I79" s="9"/>
       <c r="J79" s="6" t="s">
@@ -3754,24 +3809,24 @@
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80" s="5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B80" s="5"/>
       <c r="C80" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D80" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="F80" s="6"/>
       <c r="G80" s="7" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H80" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I80" s="9"/>
       <c r="J80" s="6" t="s">
@@ -3781,24 +3836,24 @@
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B81" s="5"/>
       <c r="C81" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D81" s="6" t="s">
         <v>40</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F81" s="6"/>
       <c r="G81" s="7" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H81" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I81" s="9"/>
       <c r="J81" s="6" t="s">
@@ -3808,42 +3863,116 @@
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" s="5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B82" s="5"/>
       <c r="C82" s="5"/>
       <c r="D82" s="6"/>
       <c r="E82" s="6" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F82" s="6"/>
       <c r="G82" s="22" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H82" s="21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I82" s="9"/>
       <c r="J82" s="6" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="K82" s="6"/>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="H83"/>
-      <c r="I83"/>
+      <c r="A83" s="24" t="s">
+        <v>277</v>
+      </c>
+      <c r="B83" s="24"/>
+      <c r="C83" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="D83" s="25"/>
+      <c r="E83" s="25" t="s">
+        <v>280</v>
+      </c>
+      <c r="F83" s="25"/>
+      <c r="G83" s="22"/>
+      <c r="H83" s="21" t="s">
+        <v>173</v>
+      </c>
+      <c r="I83" s="26"/>
+      <c r="J83" s="25" t="s">
+        <v>279</v>
+      </c>
+      <c r="K83" s="25"/>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="H84"/>
-      <c r="I84"/>
+      <c r="A84" s="24"/>
+      <c r="B84" s="24"/>
+      <c r="C84" s="24" t="s">
+        <v>284</v>
+      </c>
+      <c r="D84" s="25"/>
+      <c r="E84" s="25"/>
+      <c r="F84" s="25"/>
+      <c r="G84" s="22"/>
+      <c r="H84" s="21"/>
+      <c r="I84" s="26"/>
+      <c r="J84" s="25"/>
+      <c r="K84" s="25" t="s">
+        <v>285</v>
+      </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="H85"/>
-      <c r="I85"/>
+      <c r="A85" s="24" t="s">
+        <v>287</v>
+      </c>
+      <c r="B85" s="24"/>
+      <c r="C85" s="24" t="s">
+        <v>289</v>
+      </c>
+      <c r="D85" s="25"/>
+      <c r="E85" s="25" t="s">
+        <v>292</v>
+      </c>
+      <c r="F85" s="25"/>
+      <c r="G85" s="22" t="s">
+        <v>238</v>
+      </c>
+      <c r="H85" s="21" t="s">
+        <v>172</v>
+      </c>
+      <c r="I85" s="26"/>
+      <c r="J85" s="25" t="s">
+        <v>290</v>
+      </c>
+      <c r="K85" s="25"/>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="H86"/>
-      <c r="I86"/>
+      <c r="A86" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="B86" s="24"/>
+      <c r="C86" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D86" s="25"/>
+      <c r="E86" s="25" t="s">
+        <v>293</v>
+      </c>
+      <c r="F86" s="25"/>
+      <c r="G86" s="22" t="s">
+        <v>238</v>
+      </c>
+      <c r="H86" s="21" t="s">
+        <v>172</v>
+      </c>
+      <c r="I86" s="26"/>
+      <c r="J86" s="25" t="s">
+        <v>290</v>
+      </c>
+      <c r="K86" s="25"/>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H87"/>

</xml_diff>

<commit_message>
corrected Lobby Tv details
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B885147-4BDA-A94C-B58B-86DCE4AA399D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26EE30E-47C6-0C48-BFD4-6BD8600B8406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8320" yWindow="1460" windowWidth="21920" windowHeight="18180" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="298">
   <si>
     <t>NSCU-A004</t>
   </si>
@@ -978,6 +978,18 @@
   </si>
   <si>
     <t>192.168.204.31</t>
+  </si>
+  <si>
+    <t>14-3F-A6-B8-EA-5D</t>
+  </si>
+  <si>
+    <t>192.168.207.100</t>
+  </si>
+  <si>
+    <t>2310-1700</t>
+  </si>
+  <si>
+    <t>Lobby TV</t>
   </si>
 </sst>
 </file>
@@ -1179,10 +1191,10 @@
     <xf numFmtId="49" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1466,8 +1478,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}" name="Table1" displayName="Table1" ref="A1:K86" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:K86" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}" name="Table1" displayName="Table1" ref="A1:K87" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A1:K87" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K73">
     <sortCondition ref="A2:A73"/>
     <sortCondition ref="B2:B73"/>
@@ -3358,7 +3370,7 @@
         <f>CONCATENATE("http://", E63)</f>
         <v>http://192.168.201.110</v>
       </c>
-      <c r="G63" s="27" t="s">
+      <c r="G63" s="24" t="s">
         <v>238</v>
       </c>
       <c r="H63" s="21" t="s">
@@ -3885,98 +3897,117 @@
       <c r="K82" s="6"/>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A83" s="24" t="s">
+      <c r="A83" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="B83" s="24"/>
+      <c r="B83" s="5"/>
       <c r="C83" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="D83" s="25"/>
-      <c r="E83" s="25" t="s">
+      <c r="D83" s="6"/>
+      <c r="E83" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="F83" s="25"/>
+      <c r="F83" s="6"/>
       <c r="G83" s="22"/>
       <c r="H83" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="I83" s="26"/>
-      <c r="J83" s="25" t="s">
+      <c r="I83" s="9"/>
+      <c r="J83" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="K83" s="25"/>
+      <c r="K83" s="6"/>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A84" s="24"/>
-      <c r="B84" s="24"/>
-      <c r="C84" s="24" t="s">
+      <c r="A84" s="5"/>
+      <c r="B84" s="5"/>
+      <c r="C84" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="D84" s="25"/>
-      <c r="E84" s="25"/>
-      <c r="F84" s="25"/>
+      <c r="D84" s="6"/>
+      <c r="E84" s="6"/>
+      <c r="F84" s="6"/>
       <c r="G84" s="22"/>
       <c r="H84" s="21"/>
-      <c r="I84" s="26"/>
-      <c r="J84" s="25"/>
-      <c r="K84" s="25" t="s">
+      <c r="I84" s="9"/>
+      <c r="J84" s="6"/>
+      <c r="K84" s="6" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A85" s="24" t="s">
+      <c r="A85" s="5" t="s">
         <v>287</v>
       </c>
-      <c r="B85" s="24"/>
-      <c r="C85" s="24" t="s">
+      <c r="B85" s="5"/>
+      <c r="C85" s="5" t="s">
         <v>289</v>
       </c>
-      <c r="D85" s="25"/>
-      <c r="E85" s="25" t="s">
+      <c r="D85" s="6"/>
+      <c r="E85" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="F85" s="25"/>
+      <c r="F85" s="6"/>
       <c r="G85" s="22" t="s">
         <v>238</v>
       </c>
       <c r="H85" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="I85" s="26"/>
-      <c r="J85" s="25" t="s">
+      <c r="I85" s="9"/>
+      <c r="J85" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="K85" s="25"/>
+      <c r="K85" s="6"/>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A86" s="24" t="s">
+      <c r="A86" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="B86" s="24"/>
-      <c r="C86" s="24" t="s">
+      <c r="B86" s="5"/>
+      <c r="C86" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="D86" s="25"/>
-      <c r="E86" s="25" t="s">
+      <c r="D86" s="6"/>
+      <c r="E86" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="F86" s="25"/>
+      <c r="F86" s="6"/>
       <c r="G86" s="22" t="s">
         <v>238</v>
       </c>
       <c r="H86" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="I86" s="26"/>
-      <c r="J86" s="25" t="s">
+      <c r="I86" s="9"/>
+      <c r="J86" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="K86" s="25"/>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="H87"/>
-      <c r="I87"/>
+      <c r="K86" s="6"/>
+    </row>
+    <row r="87" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="A87" s="25" t="s">
+        <v>296</v>
+      </c>
+      <c r="B87" s="25"/>
+      <c r="C87" s="25" t="s">
+        <v>294</v>
+      </c>
+      <c r="D87" s="26"/>
+      <c r="E87" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="F87" s="26"/>
+      <c r="G87" s="22"/>
+      <c r="H87" s="21" t="s">
+        <v>172</v>
+      </c>
+      <c r="I87" s="27"/>
+      <c r="J87" s="26" t="s">
+        <v>297</v>
+      </c>
+      <c r="K87" s="26"/>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H88"/>

</xml_diff>

<commit_message>
update switch port connections
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26EE30E-47C6-0C48-BFD4-6BD8600B8406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8866A086-482F-7046-9EAE-D859752DDC87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8320" yWindow="1460" windowWidth="21920" windowHeight="18180" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="300">
   <si>
     <t>NSCU-A004</t>
   </si>
@@ -990,6 +990,12 @@
   </si>
   <si>
     <t>Lobby TV</t>
+  </si>
+  <si>
+    <t>2603-1206</t>
+  </si>
+  <si>
+    <t>192.168.201.103</t>
   </si>
 </sst>
 </file>
@@ -1110,7 +1116,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -1157,12 +1163,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="double">
+        <color theme="4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1195,6 +1210,7 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1478,8 +1494,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}" name="Table1" displayName="Table1" ref="A1:K87" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:K87" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}" name="Table1" displayName="Table1" ref="A1:K88" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A1:K88" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K73">
     <sortCondition ref="A2:A73"/>
     <sortCondition ref="B2:B73"/>
@@ -3986,7 +4002,7 @@
       </c>
       <c r="K86" s="6"/>
     </row>
-    <row r="87" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:11" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A87" s="25" t="s">
         <v>296</v>
       </c>
@@ -4009,9 +4025,24 @@
       </c>
       <c r="K87" s="26"/>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="H88"/>
-      <c r="I88"/>
+    <row r="88" spans="1:11" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="28" t="s">
+        <v>298</v>
+      </c>
+      <c r="B88" s="25"/>
+      <c r="C88" s="25"/>
+      <c r="D88" s="26"/>
+      <c r="E88" s="26" t="s">
+        <v>299</v>
+      </c>
+      <c r="F88" s="26"/>
+      <c r="G88" s="22"/>
+      <c r="H88" s="21" t="s">
+        <v>172</v>
+      </c>
+      <c r="I88" s="27"/>
+      <c r="J88" s="26"/>
+      <c r="K88" s="26"/>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H89"/>

</xml_diff>

<commit_message>
updated ip address type
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649F0B39-7306-054C-A7F6-A2FDF5FD2C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BA37C41-0AE7-BB40-AD36-3D15171DB6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1880" yWindow="2960" windowWidth="28360" windowHeight="16680" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="373">
   <si>
     <t>NSCU-A004</t>
   </si>
@@ -1187,9 +1187,6 @@
     <t>2603-1300</t>
   </si>
   <si>
-    <t>CueCommander is port 1880, Companion is port 8000, media_arts_home is port 80.</t>
-  </si>
-  <si>
     <t>osc:9110</t>
   </si>
   <si>
@@ -1215,6 +1212,9 @@
   </si>
   <si>
     <t>Amplifier</t>
+  </si>
+  <si>
+    <t>cuecommander:1880, companion:8000, media_arts_home:80</t>
   </si>
 </sst>
 </file>
@@ -1491,7 +1491,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1586,6 +1586,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2250,7 +2251,9 @@
       <c r="C2" s="22" t="s">
         <v>320</v>
       </c>
-      <c r="D2" s="6"/>
+      <c r="D2" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E2" s="23" t="s">
         <v>239</v>
       </c>
@@ -2277,7 +2280,9 @@
       <c r="C3" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="D3" s="6"/>
+      <c r="D3" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E3" s="6" t="s">
         <v>192</v>
       </c>
@@ -2302,7 +2307,9 @@
       <c r="C4" s="22" t="s">
         <v>195</v>
       </c>
-      <c r="D4" s="6"/>
+      <c r="D4" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E4" s="23"/>
       <c r="F4" s="23"/>
       <c r="G4" s="6"/>
@@ -2325,7 +2332,9 @@
       <c r="C5" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="D5" s="6"/>
+      <c r="D5" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E5" s="6" t="s">
         <v>202</v>
       </c>
@@ -2350,7 +2359,9 @@
       <c r="C6" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="D6" s="6"/>
+      <c r="D6" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E6" s="23"/>
       <c r="F6" s="23"/>
       <c r="G6" s="6"/>
@@ -2373,7 +2384,9 @@
       <c r="C7" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D7" s="6"/>
+      <c r="D7" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E7" s="6" t="s">
         <v>218</v>
       </c>
@@ -2400,7 +2413,9 @@
       <c r="C8" s="22" t="s">
         <v>220</v>
       </c>
-      <c r="D8" s="6"/>
+      <c r="D8" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E8" s="23"/>
       <c r="F8" s="23"/>
       <c r="G8" s="6"/>
@@ -2423,7 +2438,9 @@
       <c r="C9" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="D9" s="6"/>
+      <c r="D9" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E9" s="6" t="s">
         <v>205</v>
       </c>
@@ -2448,7 +2465,9 @@
       <c r="C10" s="22" t="s">
         <v>207</v>
       </c>
-      <c r="D10" s="6"/>
+      <c r="D10" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E10" s="23"/>
       <c r="F10" s="23"/>
       <c r="G10" s="6"/>
@@ -2469,7 +2488,9 @@
       <c r="C11" s="32" t="s">
         <v>321</v>
       </c>
-      <c r="D11" s="6"/>
+      <c r="D11" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E11" s="32" t="s">
         <v>309</v>
       </c>
@@ -2496,7 +2517,9 @@
       <c r="C12" s="22" t="s">
         <v>322</v>
       </c>
-      <c r="D12" s="6"/>
+      <c r="D12" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E12" s="22" t="s">
         <v>319</v>
       </c>
@@ -2523,7 +2546,9 @@
       <c r="C13" s="22" t="s">
         <v>323</v>
       </c>
-      <c r="D13" s="6"/>
+      <c r="D13" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E13" s="22" t="s">
         <v>315</v>
       </c>
@@ -2550,7 +2575,9 @@
       <c r="C14" s="22" t="s">
         <v>324</v>
       </c>
-      <c r="D14" s="6"/>
+      <c r="D14" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E14" s="22" t="s">
         <v>303</v>
       </c>
@@ -2577,7 +2604,9 @@
       <c r="C15" s="22" t="s">
         <v>325</v>
       </c>
-      <c r="D15" s="6"/>
+      <c r="D15" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E15" s="22" t="s">
         <v>307</v>
       </c>
@@ -2604,7 +2633,9 @@
       <c r="C16" s="32" t="s">
         <v>326</v>
       </c>
-      <c r="D16" s="6"/>
+      <c r="D16" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E16" s="32" t="s">
         <v>313</v>
       </c>
@@ -2631,7 +2662,9 @@
       <c r="C17" s="32" t="s">
         <v>327</v>
       </c>
-      <c r="D17" s="6"/>
+      <c r="D17" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E17" s="32" t="s">
         <v>317</v>
       </c>
@@ -2658,7 +2691,9 @@
       <c r="C18" s="22" t="s">
         <v>328</v>
       </c>
-      <c r="D18" s="6"/>
+      <c r="D18" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E18" s="22" t="s">
         <v>311</v>
       </c>
@@ -2685,7 +2720,9 @@
       <c r="C19" s="32" t="s">
         <v>329</v>
       </c>
-      <c r="D19" s="6"/>
+      <c r="D19" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E19" s="32" t="s">
         <v>305</v>
       </c>
@@ -2710,7 +2747,9 @@
       <c r="C20" s="32" t="s">
         <v>330</v>
       </c>
-      <c r="D20" s="6"/>
+      <c r="D20" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E20" s="32" t="s">
         <v>293</v>
       </c>
@@ -2872,7 +2911,9 @@
       <c r="C26" s="22" t="s">
         <v>268</v>
       </c>
-      <c r="D26" s="6"/>
+      <c r="D26" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E26" s="23"/>
       <c r="F26" s="23"/>
       <c r="G26" s="19"/>
@@ -2981,7 +3022,9 @@
       <c r="C30" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D30" s="6"/>
+      <c r="D30" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E30" s="6" t="s">
         <v>224</v>
       </c>
@@ -2992,7 +3035,7 @@
       </c>
       <c r="I30" s="9"/>
       <c r="J30" s="6" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="K30" s="44"/>
     </row>
@@ -3006,7 +3049,9 @@
       <c r="C31" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="D31" s="6"/>
+      <c r="D31" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E31" s="6" t="s">
         <v>196</v>
       </c>
@@ -3017,7 +3062,7 @@
       </c>
       <c r="I31" s="9"/>
       <c r="J31" s="5" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="K31" s="44"/>
     </row>
@@ -3029,7 +3074,9 @@
       <c r="C32" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="D32" s="6"/>
+      <c r="D32" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E32" s="6" t="s">
         <v>222</v>
       </c>
@@ -3050,7 +3097,9 @@
       <c r="C33" s="22" t="s">
         <v>332</v>
       </c>
-      <c r="D33" s="6"/>
+      <c r="D33" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E33" s="22" t="s">
         <v>288</v>
       </c>
@@ -3069,7 +3118,9 @@
       <c r="C34" s="32" t="s">
         <v>333</v>
       </c>
-      <c r="D34" s="23"/>
+      <c r="D34" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E34" s="32" t="s">
         <v>290</v>
       </c>
@@ -3088,7 +3139,9 @@
       <c r="C35" s="32" t="s">
         <v>334</v>
       </c>
-      <c r="D35" s="6"/>
+      <c r="D35" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E35" s="32" t="s">
         <v>287</v>
       </c>
@@ -3103,13 +3156,15 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B36" s="32"/>
       <c r="C36" s="32" t="s">
         <v>335</v>
       </c>
-      <c r="D36" s="6"/>
+      <c r="D36" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E36" s="32" t="s">
         <v>284</v>
       </c>
@@ -3128,7 +3183,9 @@
       <c r="C37" s="32" t="s">
         <v>336</v>
       </c>
-      <c r="D37" s="6"/>
+      <c r="D37" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E37" s="32" t="s">
         <v>291</v>
       </c>
@@ -3140,7 +3197,7 @@
       <c r="I37" s="9"/>
       <c r="J37" s="6"/>
       <c r="K37" s="44" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
@@ -3149,7 +3206,9 @@
       <c r="C38" s="32" t="s">
         <v>337</v>
       </c>
-      <c r="D38" s="6"/>
+      <c r="D38" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E38" s="32" t="s">
         <v>289</v>
       </c>
@@ -3161,7 +3220,7 @@
       <c r="I38" s="9"/>
       <c r="J38" s="6"/>
       <c r="K38" s="44" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
@@ -3170,7 +3229,9 @@
       <c r="C39" s="32" t="s">
         <v>338</v>
       </c>
-      <c r="D39" s="6"/>
+      <c r="D39" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E39" s="32" t="s">
         <v>296</v>
       </c>
@@ -3182,7 +3243,7 @@
       <c r="I39" s="9"/>
       <c r="J39" s="6"/>
       <c r="K39" s="44" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
@@ -3191,7 +3252,9 @@
       <c r="C40" s="22" t="s">
         <v>339</v>
       </c>
-      <c r="D40" s="6"/>
+      <c r="D40" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E40" s="22" t="s">
         <v>292</v>
       </c>
@@ -3203,7 +3266,7 @@
       <c r="I40" s="9"/>
       <c r="J40" s="6"/>
       <c r="K40" s="44" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
@@ -3212,7 +3275,9 @@
       <c r="C41" s="22" t="s">
         <v>340</v>
       </c>
-      <c r="D41" s="6"/>
+      <c r="D41" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E41" s="22" t="s">
         <v>295</v>
       </c>
@@ -3224,7 +3289,7 @@
       <c r="I41" s="9"/>
       <c r="J41" s="6"/>
       <c r="K41" s="44" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
@@ -3233,7 +3298,9 @@
       <c r="C42" s="22" t="s">
         <v>341</v>
       </c>
-      <c r="D42" s="6"/>
+      <c r="D42" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E42" s="22" t="s">
         <v>286</v>
       </c>
@@ -3245,7 +3312,7 @@
       <c r="I42" s="9"/>
       <c r="J42" s="6"/>
       <c r="K42" s="44" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
@@ -3254,7 +3321,9 @@
       <c r="C43" s="22" t="s">
         <v>342</v>
       </c>
-      <c r="D43" s="6"/>
+      <c r="D43" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E43" s="22" t="s">
         <v>297</v>
       </c>
@@ -3266,7 +3335,7 @@
       <c r="I43" s="9"/>
       <c r="J43" s="6"/>
       <c r="K43" s="44" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
@@ -3275,7 +3344,9 @@
       <c r="C44" s="32" t="s">
         <v>343</v>
       </c>
-      <c r="D44" s="6"/>
+      <c r="D44" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E44" s="32" t="s">
         <v>285</v>
       </c>
@@ -3287,7 +3358,7 @@
       <c r="I44" s="9"/>
       <c r="J44" s="6"/>
       <c r="K44" s="44" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
@@ -3296,7 +3367,9 @@
       <c r="C45" s="32" t="s">
         <v>344</v>
       </c>
-      <c r="D45" s="23"/>
+      <c r="D45" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E45" s="32" t="s">
         <v>281</v>
       </c>
@@ -3308,7 +3381,7 @@
       <c r="I45" s="24"/>
       <c r="J45" s="23"/>
       <c r="K45" s="44" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
@@ -3409,7 +3482,9 @@
       <c r="C49" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="D49" s="6"/>
+      <c r="D49" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E49" s="6" t="s">
         <v>231</v>
       </c>
@@ -3436,7 +3511,9 @@
       <c r="C50" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="D50" s="6"/>
+      <c r="D50" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E50" s="6" t="s">
         <v>200</v>
       </c>
@@ -3756,7 +3833,9 @@
       <c r="C61" s="22" t="s">
         <v>345</v>
       </c>
-      <c r="D61" s="23"/>
+      <c r="D61" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E61" s="58" t="s">
         <v>276</v>
       </c>
@@ -3783,7 +3862,9 @@
       <c r="C62" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="D62" s="6"/>
+      <c r="D62" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="E62" s="6" t="s">
         <v>181</v>
       </c>
@@ -3808,7 +3889,9 @@
       <c r="C63" s="6" t="s">
         <v>346</v>
       </c>
-      <c r="D63" s="6"/>
+      <c r="D63" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E63" s="6" t="s">
         <v>150</v>
       </c>
@@ -3831,7 +3914,9 @@
       <c r="C64" s="23" t="s">
         <v>347</v>
       </c>
-      <c r="D64" s="6"/>
+      <c r="D64" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E64" s="23" t="s">
         <v>188</v>
       </c>
@@ -3856,7 +3941,9 @@
       <c r="C65" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="D65" s="6"/>
+      <c r="D65" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E65" s="6" t="s">
         <v>149</v>
       </c>
@@ -3884,13 +3971,15 @@
       <c r="C66" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="D66" s="6"/>
+      <c r="D66" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E66" s="6" t="s">
         <v>176</v>
       </c>
       <c r="F66" s="6"/>
       <c r="G66" s="6" t="s">
-        <v>241</v>
+        <v>372</v>
       </c>
       <c r="H66" s="18" t="s">
         <v>166</v>
@@ -3899,9 +3988,7 @@
       <c r="J66" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="K66" s="44" t="s">
-        <v>363</v>
-      </c>
+      <c r="K66" s="44"/>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" s="5" t="s">
@@ -3913,13 +4000,15 @@
       <c r="C67" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="D67" s="6"/>
+      <c r="D67" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="E67" s="14" t="s">
         <v>171</v>
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6" t="s">
-        <v>241</v>
+        <v>372</v>
       </c>
       <c r="H67" s="18" t="s">
         <v>166</v>
@@ -3938,7 +4027,9 @@
       <c r="C68" s="57" t="s">
         <v>348</v>
       </c>
-      <c r="D68" s="6"/>
+      <c r="D68" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="E68" s="23" t="s">
         <v>301</v>
       </c>
@@ -3954,7 +4045,7 @@
         <v>361</v>
       </c>
       <c r="K68" s="48" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.2">
@@ -3965,7 +4056,9 @@
       <c r="C69" s="57" t="s">
         <v>349</v>
       </c>
-      <c r="D69" s="6"/>
+      <c r="D69" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E69" s="23" t="s">
         <v>299</v>
       </c>
@@ -3981,7 +4074,7 @@
         <v>361</v>
       </c>
       <c r="K69" s="47" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.2">
@@ -4173,7 +4266,9 @@
       <c r="C76" s="36" t="s">
         <v>352</v>
       </c>
-      <c r="D76" s="6"/>
+      <c r="D76" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E76" s="36" t="s">
         <v>157</v>
       </c>
@@ -4184,7 +4279,7 @@
       </c>
       <c r="I76" s="9"/>
       <c r="J76" s="6" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K76" s="44">
         <v>18</v>
@@ -4225,7 +4320,9 @@
       <c r="C78" s="29" t="s">
         <v>353</v>
       </c>
-      <c r="D78" s="6"/>
+      <c r="D78" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E78" s="29" t="s">
         <v>156</v>
       </c>
@@ -4236,7 +4333,7 @@
       <c r="H78" s="8"/>
       <c r="I78" s="9"/>
       <c r="J78" s="32" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="K78" s="47">
         <v>14</v>
@@ -4252,7 +4349,9 @@
       <c r="C79" s="37" t="s">
         <v>172</v>
       </c>
-      <c r="D79" s="6"/>
+      <c r="D79" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E79" s="37" t="s">
         <v>173</v>
       </c>
@@ -4304,7 +4403,9 @@
       <c r="C81" s="29" t="s">
         <v>355</v>
       </c>
-      <c r="D81" s="6"/>
+      <c r="D81" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E81" s="36" t="s">
         <v>267</v>
       </c>
@@ -4329,7 +4430,9 @@
       <c r="C82" s="29" t="s">
         <v>185</v>
       </c>
-      <c r="D82" s="6"/>
+      <c r="D82" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E82" s="36" t="s">
         <v>186</v>
       </c>
@@ -4356,7 +4459,9 @@
       <c r="C83" s="29" t="s">
         <v>184</v>
       </c>
-      <c r="D83" s="6"/>
+      <c r="D83" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="E83" s="36" t="s">
         <v>178</v>
       </c>
@@ -4381,7 +4486,9 @@
       <c r="C84" s="26" t="s">
         <v>356</v>
       </c>
-      <c r="D84" s="6"/>
+      <c r="D84" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E84" s="36" t="s">
         <v>260</v>
       </c>
@@ -4472,7 +4579,9 @@
       <c r="C87" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="D87" s="6"/>
+      <c r="D87" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E87" s="36"/>
       <c r="F87" s="36"/>
       <c r="G87" s="6"/>
@@ -4517,7 +4626,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="89" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" s="22" t="s">
         <v>271</v>
       </c>
@@ -4525,7 +4634,9 @@
       <c r="C89" s="29" t="s">
         <v>357</v>
       </c>
-      <c r="D89" s="6"/>
+      <c r="D89" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="E89" s="36" t="s">
         <v>274</v>
       </c>
@@ -4550,7 +4661,9 @@
       <c r="C90" s="29" t="s">
         <v>358</v>
       </c>
-      <c r="D90" s="6"/>
+      <c r="D90" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="E90" s="36" t="s">
         <v>275</v>
       </c>
@@ -4577,7 +4690,9 @@
       <c r="C91" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="D91" s="6"/>
+      <c r="D91" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E91" s="36"/>
       <c r="F91" s="36"/>
       <c r="G91" s="6"/>
@@ -4600,7 +4715,9 @@
       <c r="C92" s="36" t="s">
         <v>154</v>
       </c>
-      <c r="D92" s="6"/>
+      <c r="D92" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E92" s="36" t="s">
         <v>155</v>
       </c>
@@ -4623,7 +4740,9 @@
         <v>183</v>
       </c>
       <c r="C93" s="29"/>
-      <c r="D93" s="6"/>
+      <c r="D93" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E93" s="36" t="s">
         <v>182</v>
       </c>
@@ -4644,7 +4763,9 @@
       </c>
       <c r="B94" s="33"/>
       <c r="C94" s="36"/>
-      <c r="D94" s="6"/>
+      <c r="D94" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E94" s="37" t="s">
         <v>179</v>
       </c>
@@ -4665,13 +4786,15 @@
       </c>
       <c r="B95" s="5"/>
       <c r="C95" s="29"/>
-      <c r="D95" s="6"/>
+      <c r="D95" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E95" s="37" t="s">
         <v>243</v>
       </c>
       <c r="F95" s="36"/>
       <c r="G95" s="19" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="H95" s="8" t="s">
         <v>166</v>
@@ -4688,7 +4811,9 @@
       </c>
       <c r="B96" s="22"/>
       <c r="C96" s="29"/>
-      <c r="D96" s="6"/>
+      <c r="D96" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E96" s="36" t="s">
         <v>238</v>
       </c>
@@ -4705,7 +4830,9 @@
       </c>
       <c r="B97" s="22"/>
       <c r="C97" s="29"/>
-      <c r="D97" s="23"/>
+      <c r="D97" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E97" s="36" t="s">
         <v>280</v>
       </c>
@@ -4718,13 +4845,15 @@
       <c r="J97" s="36"/>
       <c r="K97" s="51"/>
     </row>
-    <row r="98" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" s="30" t="s">
         <v>9</v>
       </c>
       <c r="B98" s="5"/>
       <c r="C98" s="38"/>
-      <c r="D98" s="6"/>
+      <c r="D98" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E98" s="38" t="s">
         <v>4</v>
       </c>
@@ -4743,7 +4872,9 @@
       </c>
       <c r="B99" s="5"/>
       <c r="C99" s="29"/>
-      <c r="D99" s="6"/>
+      <c r="D99" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E99" s="36"/>
       <c r="F99" s="36"/>
       <c r="G99" s="19"/>
@@ -4762,7 +4893,9 @@
         <v>161</v>
       </c>
       <c r="C100" s="29"/>
-      <c r="D100" s="6"/>
+      <c r="D100" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E100" s="36"/>
       <c r="F100" s="39"/>
       <c r="G100" s="7"/>
@@ -4773,13 +4906,15 @@
       <c r="J100" s="36"/>
       <c r="K100" s="51"/>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A101" s="22" t="s">
         <v>168</v>
       </c>
       <c r="B101" s="28"/>
       <c r="C101" s="29"/>
-      <c r="D101" s="6"/>
+      <c r="D101" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E101" s="36"/>
       <c r="F101" s="39"/>
       <c r="G101" s="7"/>
@@ -4800,7 +4935,9 @@
       </c>
       <c r="B102" s="6"/>
       <c r="C102" s="36"/>
-      <c r="D102" s="6"/>
+      <c r="D102" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E102" s="36"/>
       <c r="F102" s="36"/>
       <c r="G102" s="6"/>
@@ -4819,7 +4956,9 @@
       </c>
       <c r="B103" s="23"/>
       <c r="C103" s="36"/>
-      <c r="D103" s="6"/>
+      <c r="D103" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E103" s="36"/>
       <c r="F103" s="36"/>
       <c r="G103" s="6"/>
@@ -4838,7 +4977,9 @@
       </c>
       <c r="B104" s="23"/>
       <c r="C104" s="36"/>
-      <c r="D104" s="6"/>
+      <c r="D104" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E104" s="36"/>
       <c r="F104" s="36"/>
       <c r="G104" s="6"/>
@@ -4857,7 +4998,9 @@
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="36"/>
-      <c r="D105" s="6"/>
+      <c r="D105" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E105" s="36"/>
       <c r="F105" s="36"/>
       <c r="G105" s="6"/>
@@ -4876,7 +5019,9 @@
       </c>
       <c r="B106" s="6"/>
       <c r="C106" s="36"/>
-      <c r="D106" s="6"/>
+      <c r="D106" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E106" s="36"/>
       <c r="F106" s="36"/>
       <c r="G106" s="6"/>
@@ -4897,7 +5042,9 @@
       </c>
       <c r="B107" s="6"/>
       <c r="C107" s="36"/>
-      <c r="D107" s="6"/>
+      <c r="D107" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E107" s="36"/>
       <c r="F107" s="36"/>
       <c r="G107" s="6"/>
@@ -4916,7 +5063,9 @@
       </c>
       <c r="B108" s="6"/>
       <c r="C108" s="36"/>
-      <c r="D108" s="6"/>
+      <c r="D108" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E108" s="36"/>
       <c r="F108" s="36"/>
       <c r="G108" s="6"/>
@@ -4935,7 +5084,9 @@
       </c>
       <c r="B109" s="6"/>
       <c r="C109" s="36"/>
-      <c r="D109" s="6"/>
+      <c r="D109" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E109" s="36"/>
       <c r="F109" s="36"/>
       <c r="G109" s="6"/>
@@ -4954,7 +5105,9 @@
       </c>
       <c r="B110" s="6"/>
       <c r="C110" s="36"/>
-      <c r="D110" s="6"/>
+      <c r="D110" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E110" s="36"/>
       <c r="F110" s="36"/>
       <c r="G110" s="6"/>
@@ -4975,7 +5128,9 @@
         <v>194</v>
       </c>
       <c r="C111" s="22"/>
-      <c r="D111" s="6"/>
+      <c r="D111" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E111" s="23"/>
       <c r="F111" s="23"/>
       <c r="G111" s="7"/>
@@ -4996,7 +5151,9 @@
         <v>194</v>
       </c>
       <c r="C112" s="22"/>
-      <c r="D112" s="6"/>
+      <c r="D112" s="60" t="s">
+        <v>100</v>
+      </c>
       <c r="E112" s="23"/>
       <c r="F112" s="23"/>
       <c r="G112" s="7"/>

</xml_diff>

<commit_message>
updated some DHCP types
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BA37C41-0AE7-BB40-AD36-3D15171DB6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9C1C04-0C35-2340-B8FA-73CABF26C156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1880" yWindow="2960" windowWidth="28360" windowHeight="16680" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
@@ -1491,7 +1491,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1518,9 +1518,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="5" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1528,7 +1525,7 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1537,7 +1534,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1545,16 +1542,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1579,13 +1573,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -1872,7 +1860,43 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}" name="Table1" displayName="Table1" ref="A1:K131" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:K131" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}"/>
+  <autoFilter ref="A1:K131" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="192.168.0.103"/>
+        <filter val="192.168.0.122"/>
+        <filter val="192.168.0.130"/>
+        <filter val="192.168.0.145"/>
+        <filter val="192.168.0.180"/>
+        <filter val="192.168.0.181"/>
+        <filter val="192.168.0.183"/>
+        <filter val="192.168.0.185"/>
+        <filter val="192.168.0.186"/>
+        <filter val="192.168.0.187"/>
+        <filter val="192.168.0.188"/>
+        <filter val="192.168.0.189"/>
+        <filter val="192.168.0.190"/>
+        <filter val="192.168.0.191"/>
+        <filter val="192.168.0.192"/>
+        <filter val="192.168.0.193"/>
+        <filter val="192.168.0.194"/>
+        <filter val="192.168.0.195"/>
+        <filter val="192.168.0.197"/>
+        <filter val="192.168.0.201"/>
+        <filter val="192.168.0.202"/>
+        <filter val="192.168.0.207"/>
+        <filter val="192.168.0.208"/>
+        <filter val="192.168.0.210"/>
+        <filter val="192.168.0.22"/>
+        <filter val="192.168.0.23"/>
+        <filter val="192.168.0.239"/>
+        <filter val="192.168.0.24"/>
+        <filter val="192.168.0.25"/>
+        <filter val="192.168.0.26"/>
+        <filter val="192.168.0.53"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K131">
     <sortCondition ref="C2:C131"/>
   </sortState>
@@ -2203,7 +2227,7 @@
     <col min="8" max="8" width="10.1640625" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.1640625" style="4" customWidth="1"/>
     <col min="10" max="10" width="29.1640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="44.6640625" style="55" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="44.6640625" style="51" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="19.1640625" customWidth="1"/>
     <col min="13" max="13" width="19.33203125" bestFit="1" customWidth="1"/>
   </cols>
@@ -2239,25 +2263,25 @@
       <c r="J1" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="K1" s="43" t="s">
+      <c r="K1" s="40" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="22" t="s">
+    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
         <v>237</v>
       </c>
       <c r="B2" s="5"/>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="5" t="s">
         <v>320</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E2" s="23" t="s">
+      <c r="E2" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="F2" s="23"/>
+      <c r="F2" s="6"/>
       <c r="G2" s="19" t="s">
         <v>245</v>
       </c>
@@ -2265,12 +2289,12 @@
         <v>166</v>
       </c>
       <c r="I2" s="9"/>
-      <c r="J2" s="23" t="s">
+      <c r="J2" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="K2" s="45"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K2" s="41"/>
+    </row>
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>189</v>
       </c>
@@ -2295,34 +2319,34 @@
       <c r="J3" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="K3" s="44"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K3" s="41"/>
+    </row>
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="5" t="s">
         <v>195</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I4" s="9"/>
-      <c r="J4" s="23" t="s">
+      <c r="J4" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="K4" s="45"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K4" s="41"/>
+    </row>
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>208</v>
       </c>
@@ -2347,34 +2371,34 @@
       <c r="J5" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="K5" s="44"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" s="23" t="s">
+      <c r="K5" s="41"/>
+    </row>
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
         <v>208</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="5" t="s">
         <v>204</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I6" s="9"/>
-      <c r="J6" s="23" t="s">
+      <c r="J6" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="K6" s="45"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K6" s="41"/>
+    </row>
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>215</v>
       </c>
@@ -2401,34 +2425,34 @@
       <c r="J7" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="K7" s="44"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K7" s="41"/>
+    </row>
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="5" t="s">
         <v>220</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
       <c r="G8" s="6"/>
       <c r="H8" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I8" s="9"/>
-      <c r="J8" s="23" t="s">
+      <c r="J8" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="K8" s="45"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K8" s="41"/>
+    </row>
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>214</v>
       </c>
@@ -2453,48 +2477,48 @@
       <c r="J9" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="K9" s="44"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K9" s="41"/>
+    </row>
+    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="5" t="s">
         <v>207</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
       <c r="G10" s="6"/>
       <c r="H10" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I10" s="9"/>
-      <c r="J10" s="23" t="s">
+      <c r="J10" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="K10" s="45"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="32" t="s">
+      <c r="K10" s="41"/>
+    </row>
+    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="29" t="s">
         <v>308</v>
       </c>
       <c r="B11" s="5"/>
-      <c r="C11" s="32" t="s">
+      <c r="C11" s="29" t="s">
         <v>321</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E11" s="32" t="s">
+      <c r="E11" s="29" t="s">
         <v>309</v>
       </c>
-      <c r="F11" s="32" t="s">
+      <c r="F11" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G11" s="7" t="s">
@@ -2502,28 +2526,28 @@
       </c>
       <c r="H11" s="8"/>
       <c r="I11" s="9"/>
-      <c r="J11" s="22" t="s">
+      <c r="J11" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="K11" s="48">
+      <c r="K11" s="44">
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" s="22" t="s">
+    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
         <v>318</v>
       </c>
       <c r="B12" s="5"/>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="5" t="s">
         <v>322</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E12" s="22" t="s">
+      <c r="E12" s="5" t="s">
         <v>319</v>
       </c>
-      <c r="F12" s="22" t="s">
+      <c r="F12" s="5" t="s">
         <v>282</v>
       </c>
       <c r="G12" s="7" t="s">
@@ -2531,28 +2555,28 @@
       </c>
       <c r="H12" s="8"/>
       <c r="I12" s="9"/>
-      <c r="J12" s="32" t="s">
+      <c r="J12" s="29" t="s">
         <v>300</v>
       </c>
-      <c r="K12" s="47">
+      <c r="K12" s="43">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="22" t="s">
+    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
         <v>314</v>
       </c>
       <c r="B13" s="5"/>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="5" t="s">
         <v>323</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E13" s="22" t="s">
+      <c r="E13" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="F13" s="22" t="s">
+      <c r="F13" s="5" t="s">
         <v>282</v>
       </c>
       <c r="G13" s="7" t="s">
@@ -2560,28 +2584,28 @@
       </c>
       <c r="H13" s="8"/>
       <c r="I13" s="9"/>
-      <c r="J13" s="32" t="s">
+      <c r="J13" s="29" t="s">
         <v>283</v>
       </c>
-      <c r="K13" s="47">
+      <c r="K13" s="43">
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="22" t="s">
+    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="5" t="s">
         <v>302</v>
       </c>
       <c r="B14" s="5"/>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="5" t="s">
         <v>324</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E14" s="22" t="s">
+      <c r="E14" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="F14" s="22" t="s">
+      <c r="F14" s="5" t="s">
         <v>282</v>
       </c>
       <c r="G14" s="7" t="s">
@@ -2589,28 +2613,28 @@
       </c>
       <c r="H14" s="8"/>
       <c r="I14" s="9"/>
-      <c r="J14" s="32" t="s">
+      <c r="J14" s="29" t="s">
         <v>283</v>
       </c>
-      <c r="K14" s="47">
+      <c r="K14" s="43">
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="22" t="s">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="5" t="s">
         <v>306</v>
       </c>
       <c r="B15" s="5"/>
-      <c r="C15" s="22" t="s">
+      <c r="C15" s="5" t="s">
         <v>325</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E15" s="22" t="s">
+      <c r="E15" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="F15" s="22" t="s">
+      <c r="F15" s="5" t="s">
         <v>282</v>
       </c>
       <c r="G15" s="7" t="s">
@@ -2618,28 +2642,28 @@
       </c>
       <c r="H15" s="8"/>
       <c r="I15" s="9"/>
-      <c r="J15" s="32" t="s">
+      <c r="J15" s="29" t="s">
         <v>283</v>
       </c>
-      <c r="K15" s="47">
+      <c r="K15" s="43">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="32" t="s">
+    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="29" t="s">
         <v>312</v>
       </c>
       <c r="B16" s="5"/>
-      <c r="C16" s="32" t="s">
+      <c r="C16" s="29" t="s">
         <v>326</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E16" s="32" t="s">
+      <c r="E16" s="29" t="s">
         <v>313</v>
       </c>
-      <c r="F16" s="32" t="s">
+      <c r="F16" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G16" s="7" t="s">
@@ -2647,28 +2671,28 @@
       </c>
       <c r="H16" s="8"/>
       <c r="I16" s="9"/>
-      <c r="J16" s="22" t="s">
+      <c r="J16" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="K16" s="48">
+      <c r="K16" s="44">
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A17" s="32" t="s">
+    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="29" t="s">
         <v>316</v>
       </c>
       <c r="B17" s="5"/>
-      <c r="C17" s="32" t="s">
+      <c r="C17" s="29" t="s">
         <v>327</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E17" s="32" t="s">
+      <c r="E17" s="29" t="s">
         <v>317</v>
       </c>
-      <c r="F17" s="32" t="s">
+      <c r="F17" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G17" s="7" t="s">
@@ -2676,28 +2700,28 @@
       </c>
       <c r="H17" s="8"/>
       <c r="I17" s="9"/>
-      <c r="J17" s="22" t="s">
+      <c r="J17" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="K17" s="48">
+      <c r="K17" s="44">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="22" t="s">
+    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
         <v>310</v>
       </c>
       <c r="B18" s="5"/>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="5" t="s">
         <v>328</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="5" t="s">
         <v>311</v>
       </c>
-      <c r="F18" s="22" t="s">
+      <c r="F18" s="5" t="s">
         <v>282</v>
       </c>
       <c r="G18" s="7" t="s">
@@ -2705,28 +2729,28 @@
       </c>
       <c r="H18" s="8"/>
       <c r="I18" s="9"/>
-      <c r="J18" s="32" t="s">
+      <c r="J18" s="29" t="s">
         <v>283</v>
       </c>
-      <c r="K18" s="47">
+      <c r="K18" s="43">
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="32" t="s">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="29" t="s">
         <v>304</v>
       </c>
       <c r="B19" s="5"/>
-      <c r="C19" s="32" t="s">
+      <c r="C19" s="29" t="s">
         <v>329</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E19" s="32" t="s">
+      <c r="E19" s="29" t="s">
         <v>305</v>
       </c>
-      <c r="F19" s="32" t="s">
+      <c r="F19" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G19" s="7" t="s">
@@ -2734,36 +2758,36 @@
       </c>
       <c r="H19" s="8"/>
       <c r="I19" s="9"/>
-      <c r="J19" s="22" t="s">
+      <c r="J19" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="K19" s="48">
+      <c r="K19" s="44">
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="5"/>
-      <c r="B20" s="32"/>
-      <c r="C20" s="32" t="s">
+      <c r="B20" s="29"/>
+      <c r="C20" s="29" t="s">
         <v>330</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E20" s="32" t="s">
+      <c r="E20" s="29" t="s">
         <v>293</v>
       </c>
-      <c r="F20" s="32" t="s">
+      <c r="F20" s="29" t="s">
         <v>294</v>
       </c>
       <c r="G20" s="7"/>
       <c r="H20" s="8"/>
       <c r="I20" s="9"/>
-      <c r="J20" s="23"/>
-      <c r="K20" s="45"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="23" t="s">
+      <c r="J20" s="6"/>
+      <c r="K20" s="41"/>
+    </row>
+    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
         <v>55</v>
       </c>
       <c r="B21" s="6"/>
@@ -2787,11 +2811,11 @@
       <c r="J21" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="K21" s="44" t="s">
+      <c r="K21" s="41" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
         <v>45</v>
       </c>
@@ -2816,11 +2840,11 @@
       <c r="J22" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="K22" s="44" t="s">
+      <c r="K22" s="41" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
         <v>47</v>
       </c>
@@ -2845,11 +2869,11 @@
       <c r="J23" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="K23" s="44" t="s">
+      <c r="K23" s="41" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
         <v>49</v>
       </c>
@@ -2874,7 +2898,7 @@
       <c r="J24" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="K24" s="44" t="s">
+      <c r="K24" s="41" t="s">
         <v>42</v>
       </c>
     </row>
@@ -2901,41 +2925,41 @@
       <c r="J25" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="K25" s="46" t="s">
+      <c r="K25" s="42" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A26" s="22"/>
+    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="5"/>
       <c r="B26" s="5"/>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="5" t="s">
         <v>268</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E26" s="23"/>
-      <c r="F26" s="23"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
       <c r="G26" s="19"/>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
-      <c r="J26" s="23"/>
-      <c r="K26" s="45" t="s">
+      <c r="J26" s="6"/>
+      <c r="K26" s="41" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23" t="s">
+      <c r="B27" s="6"/>
+      <c r="C27" s="6" t="s">
         <v>331</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E27" s="23" t="s">
+      <c r="E27" s="6" t="s">
         <v>270</v>
       </c>
       <c r="F27" s="19" t="str">
@@ -2952,7 +2976,7 @@
       <c r="J27" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="K27" s="46">
+      <c r="K27" s="42">
         <v>4</v>
       </c>
     </row>
@@ -2981,7 +3005,7 @@
       <c r="J28" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K28" s="44" t="s">
+      <c r="K28" s="41" t="s">
         <v>248</v>
       </c>
     </row>
@@ -3010,11 +3034,11 @@
       <c r="J29" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K29" s="44" t="s">
+      <c r="K29" s="41" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>6</v>
       </c>
@@ -3037,9 +3061,9 @@
       <c r="J30" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="K30" s="44"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K30" s="41"/>
+    </row>
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
         <v>198</v>
       </c>
@@ -3064,9 +3088,9 @@
       <c r="J31" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="K31" s="44"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K31" s="41"/>
+    </row>
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
         <v>221</v>
       </c>
@@ -3089,303 +3113,303 @@
       <c r="J32" s="6">
         <v>30</v>
       </c>
-      <c r="K32" s="44"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K32" s="41"/>
+    </row>
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="5"/>
-      <c r="B33" s="22"/>
-      <c r="C33" s="22" t="s">
+      <c r="B33" s="5"/>
+      <c r="C33" s="5" t="s">
         <v>332</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E33" s="22" t="s">
+      <c r="E33" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="F33" s="22" t="s">
+      <c r="F33" s="5" t="s">
         <v>282</v>
       </c>
       <c r="G33" s="7"/>
       <c r="H33" s="8"/>
       <c r="I33" s="9"/>
       <c r="J33" s="6"/>
-      <c r="K33" s="44"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A34" s="22"/>
-      <c r="B34" s="32"/>
-      <c r="C34" s="32" t="s">
+      <c r="K33" s="41"/>
+    </row>
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="5"/>
+      <c r="B34" s="29"/>
+      <c r="C34" s="29" t="s">
         <v>333</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E34" s="32" t="s">
+      <c r="E34" s="29" t="s">
         <v>290</v>
       </c>
-      <c r="F34" s="32" t="s">
+      <c r="F34" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G34" s="19"/>
       <c r="H34" s="8"/>
-      <c r="I34" s="24"/>
-      <c r="J34" s="23"/>
-      <c r="K34" s="45"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I34" s="9"/>
+      <c r="J34" s="6"/>
+      <c r="K34" s="41"/>
+    </row>
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="5"/>
-      <c r="B35" s="32"/>
-      <c r="C35" s="32" t="s">
+      <c r="B35" s="29"/>
+      <c r="C35" s="29" t="s">
         <v>334</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E35" s="32" t="s">
+      <c r="E35" s="29" t="s">
         <v>287</v>
       </c>
-      <c r="F35" s="32" t="s">
+      <c r="F35" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G35" s="7"/>
       <c r="H35" s="8"/>
       <c r="I35" s="9"/>
       <c r="J35" s="6"/>
-      <c r="K35" s="44"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K35" s="41"/>
+    </row>
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32" t="s">
+      <c r="B36" s="29"/>
+      <c r="C36" s="29" t="s">
         <v>335</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E36" s="32" t="s">
+      <c r="E36" s="29" t="s">
         <v>284</v>
       </c>
-      <c r="F36" s="32" t="s">
+      <c r="F36" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G36" s="7"/>
       <c r="H36" s="8"/>
       <c r="I36" s="9"/>
       <c r="J36" s="6"/>
-      <c r="K36" s="44"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K36" s="41"/>
+    </row>
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="5"/>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32" t="s">
+      <c r="B37" s="29"/>
+      <c r="C37" s="29" t="s">
         <v>336</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E37" s="32" t="s">
+      <c r="E37" s="29" t="s">
         <v>291</v>
       </c>
-      <c r="F37" s="32" t="s">
+      <c r="F37" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G37" s="7"/>
       <c r="H37" s="8"/>
       <c r="I37" s="9"/>
       <c r="J37" s="6"/>
-      <c r="K37" s="44" t="s">
+      <c r="K37" s="41" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="5"/>
-      <c r="B38" s="32"/>
-      <c r="C38" s="32" t="s">
+      <c r="B38" s="29"/>
+      <c r="C38" s="29" t="s">
         <v>337</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E38" s="32" t="s">
+      <c r="E38" s="29" t="s">
         <v>289</v>
       </c>
-      <c r="F38" s="32" t="s">
+      <c r="F38" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G38" s="7"/>
       <c r="H38" s="8"/>
       <c r="I38" s="9"/>
       <c r="J38" s="6"/>
-      <c r="K38" s="44" t="s">
+      <c r="K38" s="41" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="5"/>
-      <c r="B39" s="32"/>
-      <c r="C39" s="32" t="s">
+      <c r="B39" s="29"/>
+      <c r="C39" s="29" t="s">
         <v>338</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E39" s="32" t="s">
+      <c r="E39" s="29" t="s">
         <v>296</v>
       </c>
-      <c r="F39" s="32" t="s">
+      <c r="F39" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G39" s="7"/>
       <c r="H39" s="8"/>
       <c r="I39" s="9"/>
       <c r="J39" s="6"/>
-      <c r="K39" s="44" t="s">
+      <c r="K39" s="41" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="5"/>
-      <c r="B40" s="22"/>
-      <c r="C40" s="22" t="s">
+      <c r="B40" s="5"/>
+      <c r="C40" s="5" t="s">
         <v>339</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E40" s="22" t="s">
+      <c r="E40" s="5" t="s">
         <v>292</v>
       </c>
-      <c r="F40" s="22" t="s">
+      <c r="F40" s="5" t="s">
         <v>282</v>
       </c>
       <c r="G40" s="7"/>
       <c r="H40" s="8"/>
       <c r="I40" s="9"/>
       <c r="J40" s="6"/>
-      <c r="K40" s="44" t="s">
+      <c r="K40" s="41" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="5"/>
-      <c r="B41" s="22"/>
-      <c r="C41" s="22" t="s">
+      <c r="B41" s="5"/>
+      <c r="C41" s="5" t="s">
         <v>340</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E41" s="22" t="s">
+      <c r="E41" s="5" t="s">
         <v>295</v>
       </c>
-      <c r="F41" s="22" t="s">
+      <c r="F41" s="5" t="s">
         <v>282</v>
       </c>
       <c r="G41" s="7"/>
       <c r="H41" s="8"/>
       <c r="I41" s="9"/>
       <c r="J41" s="6"/>
-      <c r="K41" s="44" t="s">
+      <c r="K41" s="41" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="5"/>
-      <c r="B42" s="22"/>
-      <c r="C42" s="22" t="s">
+      <c r="B42" s="5"/>
+      <c r="C42" s="5" t="s">
         <v>341</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E42" s="22" t="s">
+      <c r="E42" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="F42" s="22" t="s">
+      <c r="F42" s="5" t="s">
         <v>282</v>
       </c>
       <c r="G42" s="7"/>
       <c r="H42" s="8"/>
       <c r="I42" s="9"/>
       <c r="J42" s="6"/>
-      <c r="K42" s="44" t="s">
+      <c r="K42" s="41" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="5"/>
-      <c r="B43" s="22"/>
-      <c r="C43" s="22" t="s">
+      <c r="B43" s="5"/>
+      <c r="C43" s="5" t="s">
         <v>342</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E43" s="22" t="s">
+      <c r="E43" s="5" t="s">
         <v>297</v>
       </c>
-      <c r="F43" s="22" t="s">
+      <c r="F43" s="5" t="s">
         <v>282</v>
       </c>
       <c r="G43" s="7"/>
       <c r="H43" s="8"/>
       <c r="I43" s="9"/>
       <c r="J43" s="6"/>
-      <c r="K43" s="44" t="s">
+      <c r="K43" s="41" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="5"/>
-      <c r="B44" s="32"/>
-      <c r="C44" s="32" t="s">
+      <c r="B44" s="29"/>
+      <c r="C44" s="29" t="s">
         <v>343</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E44" s="32" t="s">
+      <c r="E44" s="29" t="s">
         <v>285</v>
       </c>
-      <c r="F44" s="32" t="s">
+      <c r="F44" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G44" s="7"/>
       <c r="H44" s="8"/>
       <c r="I44" s="9"/>
       <c r="J44" s="6"/>
-      <c r="K44" s="44" t="s">
+      <c r="K44" s="41" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A45" s="22"/>
-      <c r="B45" s="32"/>
-      <c r="C45" s="32" t="s">
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="5"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="29" t="s">
         <v>344</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E45" s="32" t="s">
+      <c r="E45" s="29" t="s">
         <v>281</v>
       </c>
-      <c r="F45" s="32" t="s">
+      <c r="F45" s="29" t="s">
         <v>282</v>
       </c>
       <c r="G45" s="19"/>
       <c r="H45" s="8"/>
-      <c r="I45" s="24"/>
-      <c r="J45" s="23"/>
-      <c r="K45" s="44" t="s">
+      <c r="I45" s="9"/>
+      <c r="J45" s="6"/>
+      <c r="K45" s="41" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A46" s="23" t="s">
+      <c r="A46" s="6" t="s">
         <v>108</v>
       </c>
       <c r="B46" s="6"/>
@@ -3410,7 +3434,7 @@
       <c r="J46" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="K46" s="44" t="s">
+      <c r="K46" s="41" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3440,7 +3464,7 @@
       <c r="J47" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="K47" s="44" t="s">
+      <c r="K47" s="41" t="s">
         <v>98</v>
       </c>
     </row>
@@ -3470,12 +3494,12 @@
       <c r="J48" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="K48" s="46" t="s">
+      <c r="K48" s="42" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A49" s="22" t="s">
+    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="5" t="s">
         <v>233</v>
       </c>
       <c r="B49" s="5"/>
@@ -3499,12 +3523,12 @@
       <c r="J49" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="K49" s="44">
+      <c r="K49" s="41">
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A50" s="34" t="s">
+    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="31" t="s">
         <v>199</v>
       </c>
       <c r="B50" s="13"/>
@@ -3526,7 +3550,7 @@
       </c>
       <c r="I50" s="9"/>
       <c r="J50" s="6"/>
-      <c r="K50" s="44"/>
+      <c r="K50" s="41"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
@@ -3537,7 +3561,7 @@
         <v>129</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>128</v>
@@ -3556,7 +3580,7 @@
       <c r="J51" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="K51" s="46"/>
+      <c r="K51" s="42"/>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
@@ -3567,7 +3591,7 @@
         <v>132</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>131</v>
@@ -3586,30 +3610,30 @@
       <c r="J52" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="K52" s="46"/>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A53" s="23" t="s">
+      <c r="K52" s="42"/>
+    </row>
+    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="6" t="s">
         <v>130</v>
       </c>
       <c r="B53" s="6"/>
-      <c r="C53" s="23" t="s">
+      <c r="C53" s="6" t="s">
         <v>132</v>
       </c>
       <c r="D53" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E53" s="23"/>
+      <c r="E53" s="6"/>
       <c r="F53" s="19"/>
       <c r="G53" s="7"/>
       <c r="H53" s="18" t="s">
         <v>167</v>
       </c>
       <c r="I53" s="9"/>
-      <c r="J53" s="23" t="s">
+      <c r="J53" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="K53" s="59"/>
+      <c r="K53" s="42"/>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" s="6" t="s">
@@ -3620,7 +3644,7 @@
         <v>127</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>126</v>
@@ -3639,7 +3663,7 @@
       <c r="J54" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="K54" s="46"/>
+      <c r="K54" s="42"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" s="6" t="s">
@@ -3650,7 +3674,7 @@
         <v>125</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="E55" s="14" t="s">
         <v>124</v>
@@ -3669,7 +3693,7 @@
       <c r="J55" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="K55" s="44"/>
+      <c r="K55" s="41"/>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
@@ -3680,7 +3704,7 @@
         <v>122</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>121</v>
@@ -3699,7 +3723,7 @@
       <c r="J56" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="K56" s="46"/>
+      <c r="K56" s="42"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" s="10" t="s">
@@ -3729,7 +3753,7 @@
       <c r="J57" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="K57" s="44"/>
+      <c r="K57" s="41"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" s="6" t="s">
@@ -3759,7 +3783,7 @@
       <c r="J58" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="K58" s="44" t="s">
+      <c r="K58" s="41" t="s">
         <v>70</v>
       </c>
     </row>
@@ -3789,7 +3813,7 @@
       <c r="J59" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="K59" s="44" t="s">
+      <c r="K59" s="41" t="s">
         <v>66</v>
       </c>
     </row>
@@ -3821,38 +3845,38 @@
       <c r="J60" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="K60" s="44" t="s">
+      <c r="K60" s="41" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A61" s="22" t="s">
+    <row r="61" spans="1:11" ht="17" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="B61" s="22"/>
-      <c r="C61" s="22" t="s">
+      <c r="B61" s="5"/>
+      <c r="C61" s="5" t="s">
         <v>345</v>
       </c>
       <c r="D61" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E61" s="58" t="s">
+      <c r="E61" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="F61" s="23"/>
+      <c r="F61" s="6"/>
       <c r="G61" s="19"/>
       <c r="H61" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="I61" s="24"/>
-      <c r="J61" s="23" t="s">
+      <c r="I61" s="9"/>
+      <c r="J61" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="K61" s="45">
+      <c r="K61" s="41">
         <v>12</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="5" t="s">
         <v>3</v>
       </c>
@@ -3877,7 +3901,7 @@
       </c>
       <c r="I62" s="9"/>
       <c r="J62" s="6"/>
-      <c r="K62" s="44">
+      <c r="K62" s="41">
         <v>3</v>
       </c>
     </row>
@@ -3904,23 +3928,23 @@
       <c r="J63" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="K63" s="44"/>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K63" s="41"/>
+    </row>
+    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B64" s="22"/>
-      <c r="C64" s="23" t="s">
+      <c r="B64" s="5"/>
+      <c r="C64" s="6" t="s">
         <v>347</v>
       </c>
       <c r="D64" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E64" s="23" t="s">
+      <c r="E64" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="F64" s="23"/>
+      <c r="F64" s="6"/>
       <c r="G64" s="6"/>
       <c r="H64" s="18" t="s">
         <v>166</v>
@@ -3929,7 +3953,7 @@
       <c r="J64" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="K64" s="44">
+      <c r="K64" s="41">
         <v>6</v>
       </c>
     </row>
@@ -3959,7 +3983,7 @@
       <c r="J65" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="K65" s="44"/>
+      <c r="K65" s="41"/>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" s="5" t="s">
@@ -3972,7 +3996,7 @@
         <v>162</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>176</v>
@@ -3988,9 +4012,9 @@
       <c r="J66" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="K66" s="44"/>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K66" s="41"/>
+    </row>
+    <row r="67" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="5" t="s">
         <v>1</v>
       </c>
@@ -4017,63 +4041,63 @@
       <c r="J67" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="K67" s="44"/>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A68" s="22" t="s">
+      <c r="K67" s="41"/>
+    </row>
+    <row r="68" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="B68" s="22"/>
-      <c r="C68" s="57" t="s">
+      <c r="B68" s="5"/>
+      <c r="C68" s="53" t="s">
         <v>348</v>
       </c>
       <c r="D68" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E68" s="23" t="s">
+      <c r="E68" s="6" t="s">
         <v>301</v>
       </c>
-      <c r="F68" s="23"/>
+      <c r="F68" s="6"/>
       <c r="G68" s="19" t="s">
         <v>230</v>
       </c>
       <c r="H68" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="I68" s="24"/>
-      <c r="J68" s="22" t="s">
+      <c r="I68" s="9"/>
+      <c r="J68" s="5" t="s">
         <v>361</v>
       </c>
-      <c r="K68" s="48" t="s">
+      <c r="K68" s="44" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" s="5" t="s">
         <v>360</v>
       </c>
-      <c r="B69" s="22"/>
-      <c r="C69" s="57" t="s">
+      <c r="B69" s="5"/>
+      <c r="C69" s="53" t="s">
         <v>349</v>
       </c>
-      <c r="D69" s="60" t="s">
+      <c r="D69" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E69" s="23" t="s">
+      <c r="E69" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="F69" s="23"/>
+      <c r="F69" s="6"/>
       <c r="G69" s="19" t="s">
         <v>230</v>
       </c>
       <c r="H69" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="I69" s="24"/>
-      <c r="J69" s="41" t="s">
+      <c r="I69" s="9"/>
+      <c r="J69" s="38" t="s">
         <v>361</v>
       </c>
-      <c r="K69" s="47" t="s">
+      <c r="K69" s="43" t="s">
         <v>367</v>
       </c>
     </row>
@@ -4102,7 +4126,7 @@
       <c r="J70" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="K70" s="46" t="s">
+      <c r="K70" s="42" t="s">
         <v>74</v>
       </c>
     </row>
@@ -4136,25 +4160,25 @@
       <c r="J71" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="K71" s="44" t="s">
+      <c r="K71" s="41" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="B72" s="22"/>
-      <c r="C72" s="22" t="s">
+      <c r="B72" s="5"/>
+      <c r="C72" s="5" t="s">
         <v>350</v>
       </c>
       <c r="D72" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E72" s="23" t="s">
+      <c r="E72" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="F72" s="23"/>
+      <c r="F72" s="6"/>
       <c r="G72" s="7" t="s">
         <v>227</v>
       </c>
@@ -4165,23 +4189,23 @@
       <c r="J72" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="K72" s="44"/>
-    </row>
-    <row r="73" spans="1:11" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="25" t="s">
+      <c r="K72" s="41"/>
+    </row>
+    <row r="73" spans="1:11" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="22" t="s">
         <v>256</v>
       </c>
-      <c r="B73" s="22"/>
-      <c r="C73" s="22" t="s">
+      <c r="B73" s="5"/>
+      <c r="C73" s="5" t="s">
         <v>351</v>
       </c>
       <c r="D73" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E73" s="23" t="s">
+      <c r="E73" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="F73" s="23"/>
+      <c r="F73" s="6"/>
       <c r="G73" s="7" t="s">
         <v>227</v>
       </c>
@@ -4192,23 +4216,23 @@
       <c r="J73" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="K73" s="44"/>
+      <c r="K73" s="41"/>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A74" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B74" s="33"/>
-      <c r="C74" s="36" t="s">
+      <c r="B74" s="30"/>
+      <c r="C74" s="33" t="s">
         <v>80</v>
       </c>
       <c r="D74" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E74" s="36" t="s">
+      <c r="E74" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="F74" s="39" t="str">
+      <c r="F74" s="36" t="str">
         <f>CONCATENATE("ftp://", E74)</f>
         <v>ftp://192.168.0.189</v>
       </c>
@@ -4222,7 +4246,7 @@
       <c r="J74" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="K74" s="46" t="s">
+      <c r="K74" s="42" t="s">
         <v>74</v>
       </c>
     </row>
@@ -4230,17 +4254,17 @@
       <c r="A75" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B75" s="33"/>
-      <c r="C75" s="36" t="s">
+      <c r="B75" s="30"/>
+      <c r="C75" s="33" t="s">
         <v>76</v>
       </c>
       <c r="D75" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E75" s="36" t="s">
+      <c r="E75" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="F75" s="39" t="str">
+      <c r="F75" s="36" t="str">
         <f>CONCATENATE("ftp://", E75)</f>
         <v>ftp://192.168.0.190</v>
       </c>
@@ -4254,25 +4278,25 @@
       <c r="J75" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="K75" s="46" t="s">
+      <c r="K75" s="42" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="B76" s="28"/>
-      <c r="C76" s="36" t="s">
+      <c r="B76" s="25"/>
+      <c r="C76" s="33" t="s">
         <v>352</v>
       </c>
-      <c r="D76" s="60" t="s">
+      <c r="D76" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E76" s="36" t="s">
+      <c r="E76" s="33" t="s">
         <v>157</v>
       </c>
-      <c r="F76" s="36"/>
+      <c r="F76" s="33"/>
       <c r="G76" s="6"/>
       <c r="H76" s="8" t="s">
         <v>166</v>
@@ -4281,7 +4305,7 @@
       <c r="J76" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="K76" s="44">
+      <c r="K76" s="41">
         <v>18</v>
       </c>
     </row>
@@ -4289,17 +4313,17 @@
       <c r="A77" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B77" s="33"/>
-      <c r="C77" s="36" t="s">
+      <c r="B77" s="30"/>
+      <c r="C77" s="33" t="s">
         <v>89</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E77" s="36" t="s">
+      <c r="E77" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="F77" s="36"/>
+      <c r="F77" s="33"/>
       <c r="G77" s="6"/>
       <c r="H77" s="8" t="s">
         <v>167</v>
@@ -4308,34 +4332,34 @@
       <c r="J77" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="K77" s="44" t="s">
+      <c r="K77" s="41" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A78" s="22" t="s">
+    <row r="78" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="B78" s="28"/>
-      <c r="C78" s="29" t="s">
+      <c r="B78" s="25"/>
+      <c r="C78" s="26" t="s">
         <v>353</v>
       </c>
-      <c r="D78" s="60" t="s">
+      <c r="D78" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E78" s="29" t="s">
+      <c r="E78" s="26" t="s">
         <v>156</v>
       </c>
-      <c r="F78" s="29" t="s">
+      <c r="F78" s="26" t="s">
         <v>298</v>
       </c>
       <c r="G78" s="7"/>
       <c r="H78" s="8"/>
       <c r="I78" s="9"/>
-      <c r="J78" s="32" t="s">
+      <c r="J78" s="29" t="s">
         <v>369</v>
       </c>
-      <c r="K78" s="47">
+      <c r="K78" s="43">
         <v>14</v>
       </c>
     </row>
@@ -4343,19 +4367,19 @@
       <c r="A79" s="5" t="s">
         <v>362</v>
       </c>
-      <c r="B79" s="28" t="s">
+      <c r="B79" s="25" t="s">
         <v>174</v>
       </c>
-      <c r="C79" s="37" t="s">
+      <c r="C79" s="34" t="s">
         <v>172</v>
       </c>
-      <c r="D79" s="60" t="s">
+      <c r="D79" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E79" s="37" t="s">
+      <c r="E79" s="34" t="s">
         <v>173</v>
       </c>
-      <c r="F79" s="36"/>
+      <c r="F79" s="33"/>
       <c r="G79" s="6" t="s">
         <v>241</v>
       </c>
@@ -4366,23 +4390,23 @@
       <c r="J79" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="K79" s="44"/>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K79" s="41"/>
+    </row>
+    <row r="80" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="B80" s="30"/>
-      <c r="C80" s="31" t="s">
+      <c r="B80" s="27"/>
+      <c r="C80" s="28" t="s">
         <v>354</v>
       </c>
       <c r="D80" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E80" s="38" t="s">
+      <c r="E80" s="35" t="s">
         <v>257</v>
       </c>
-      <c r="F80" s="38"/>
+      <c r="F80" s="35"/>
       <c r="G80" s="7" t="s">
         <v>227</v>
       </c>
@@ -4393,23 +4417,23 @@
       <c r="J80" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="K80" s="44"/>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K80" s="41"/>
+    </row>
+    <row r="81" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="B81" s="28"/>
-      <c r="C81" s="29" t="s">
+      <c r="B81" s="25"/>
+      <c r="C81" s="26" t="s">
         <v>355</v>
       </c>
-      <c r="D81" s="60" t="s">
+      <c r="D81" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E81" s="36" t="s">
+      <c r="E81" s="33" t="s">
         <v>267</v>
       </c>
-      <c r="F81" s="36"/>
+      <c r="F81" s="33"/>
       <c r="G81" s="19"/>
       <c r="H81" s="8" t="s">
         <v>167</v>
@@ -4418,25 +4442,25 @@
       <c r="J81" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="K81" s="44"/>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K81" s="41"/>
+    </row>
+    <row r="82" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="B82" s="28" t="s">
+      <c r="B82" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="C82" s="29" t="s">
+      <c r="C82" s="26" t="s">
         <v>185</v>
       </c>
-      <c r="D82" s="60" t="s">
+      <c r="D82" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E82" s="36" t="s">
+      <c r="E82" s="33" t="s">
         <v>186</v>
       </c>
-      <c r="F82" s="39"/>
+      <c r="F82" s="36"/>
       <c r="G82" s="7"/>
       <c r="H82" s="8" t="s">
         <v>166</v>
@@ -4445,7 +4469,7 @@
       <c r="J82" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="K82" s="44">
+      <c r="K82" s="41">
         <v>10</v>
       </c>
     </row>
@@ -4453,19 +4477,19 @@
       <c r="A83" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="B83" s="28" t="s">
+      <c r="B83" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="C83" s="29" t="s">
+      <c r="C83" s="26" t="s">
         <v>184</v>
       </c>
       <c r="D83" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E83" s="36" t="s">
+      <c r="E83" s="33" t="s">
         <v>178</v>
       </c>
-      <c r="F83" s="39"/>
+      <c r="F83" s="36"/>
       <c r="G83" s="7" t="s">
         <v>228</v>
       </c>
@@ -4476,23 +4500,23 @@
       <c r="J83" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="K83" s="44"/>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K83" s="41"/>
+    </row>
+    <row r="84" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="B84" s="28"/>
-      <c r="C84" s="26" t="s">
+      <c r="B84" s="25"/>
+      <c r="C84" s="23" t="s">
         <v>356</v>
       </c>
-      <c r="D84" s="60" t="s">
+      <c r="D84" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E84" s="36" t="s">
+      <c r="E84" s="33" t="s">
         <v>260</v>
       </c>
-      <c r="F84" s="36"/>
+      <c r="F84" s="33"/>
       <c r="G84" s="19" t="s">
         <v>230</v>
       </c>
@@ -4500,28 +4524,28 @@
         <v>166</v>
       </c>
       <c r="I84" s="9"/>
-      <c r="J84" s="23" t="s">
+      <c r="J84" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="K84" s="48">
+      <c r="K84" s="44">
         <v>4</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A85" s="33" t="s">
+      <c r="A85" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="B85" s="23"/>
-      <c r="C85" s="36" t="s">
+      <c r="B85" s="6"/>
+      <c r="C85" s="33" t="s">
         <v>63</v>
       </c>
       <c r="D85" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E85" s="36" t="s">
+      <c r="E85" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="F85" s="39" t="str">
+      <c r="F85" s="36" t="str">
         <f>CONCATENATE("http://", E85)</f>
         <v>http://192.168.0.195</v>
       </c>
@@ -4535,25 +4559,25 @@
       <c r="J85" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="K85" s="44" t="s">
+      <c r="K85" s="41" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A86" s="56" t="s">
+      <c r="A86" s="52" t="s">
         <v>69</v>
       </c>
-      <c r="B86" s="23"/>
-      <c r="C86" s="38" t="s">
+      <c r="B86" s="6"/>
+      <c r="C86" s="35" t="s">
         <v>68</v>
       </c>
       <c r="D86" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E86" s="38" t="s">
+      <c r="E86" s="35" t="s">
         <v>67</v>
       </c>
-      <c r="F86" s="40" t="str">
+      <c r="F86" s="37" t="str">
         <f>CONCATENATE("http://", E86)</f>
         <v>http://192.168.0.194</v>
       </c>
@@ -4564,53 +4588,53 @@
         <v>167</v>
       </c>
       <c r="I86" s="9"/>
-      <c r="J86" s="38" t="s">
+      <c r="J86" s="35" t="s">
         <v>64</v>
       </c>
-      <c r="K86" s="49" t="s">
+      <c r="K86" s="45" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A87" s="35" t="s">
+    <row r="87" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="32" t="s">
         <v>18</v>
       </c>
       <c r="B87" s="12"/>
-      <c r="C87" s="36" t="s">
+      <c r="C87" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="D87" s="60" t="s">
+      <c r="D87" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E87" s="36"/>
-      <c r="F87" s="36"/>
+      <c r="E87" s="33"/>
+      <c r="F87" s="33"/>
       <c r="G87" s="6"/>
       <c r="H87" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I87" s="9"/>
-      <c r="J87" s="36" t="s">
+      <c r="J87" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="K87" s="51" t="s">
+      <c r="K87" s="47" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A88" s="23" t="s">
+      <c r="A88" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="B88" s="33"/>
-      <c r="C88" s="36" t="s">
+      <c r="B88" s="30"/>
+      <c r="C88" s="33" t="s">
         <v>118</v>
       </c>
       <c r="D88" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E88" s="36" t="s">
+      <c r="E88" s="33" t="s">
         <v>117</v>
       </c>
-      <c r="F88" s="39" t="str">
+      <c r="F88" s="36" t="str">
         <f>CONCATENATE("http://", E88)</f>
         <v>http://192.168.0.186</v>
       </c>
@@ -4619,28 +4643,28 @@
         <v>166</v>
       </c>
       <c r="I88" s="9"/>
-      <c r="J88" s="36" t="s">
+      <c r="J88" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="K88" s="51" t="s">
+      <c r="K88" s="47" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A89" s="22" t="s">
+    <row r="89" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="B89" s="28"/>
-      <c r="C89" s="29" t="s">
+      <c r="B89" s="25"/>
+      <c r="C89" s="26" t="s">
         <v>357</v>
       </c>
       <c r="D89" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E89" s="36" t="s">
+      <c r="E89" s="33" t="s">
         <v>274</v>
       </c>
-      <c r="F89" s="36"/>
+      <c r="F89" s="33"/>
       <c r="G89" s="19" t="s">
         <v>230</v>
       </c>
@@ -4648,26 +4672,26 @@
         <v>166</v>
       </c>
       <c r="I89" s="9"/>
-      <c r="J89" s="36" t="s">
+      <c r="J89" s="33" t="s">
         <v>273</v>
       </c>
-      <c r="K89" s="51"/>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A90" s="28" t="s">
+      <c r="K89" s="47"/>
+    </row>
+    <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="25" t="s">
         <v>272</v>
       </c>
       <c r="B90" s="5"/>
-      <c r="C90" s="29" t="s">
+      <c r="C90" s="26" t="s">
         <v>358</v>
       </c>
       <c r="D90" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E90" s="36" t="s">
+      <c r="E90" s="33" t="s">
         <v>275</v>
       </c>
-      <c r="F90" s="36"/>
+      <c r="F90" s="33"/>
       <c r="G90" s="19" t="s">
         <v>230</v>
       </c>
@@ -4675,124 +4699,124 @@
         <v>166</v>
       </c>
       <c r="I90" s="9"/>
-      <c r="J90" s="36" t="s">
+      <c r="J90" s="33" t="s">
         <v>273</v>
       </c>
-      <c r="K90" s="51">
+      <c r="K90" s="47">
         <v>13</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A91" s="22" t="s">
+    <row r="91" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B91" s="28"/>
-      <c r="C91" s="36" t="s">
+      <c r="B91" s="25"/>
+      <c r="C91" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="D91" s="60" t="s">
+      <c r="D91" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E91" s="36"/>
-      <c r="F91" s="36"/>
+      <c r="E91" s="33"/>
+      <c r="F91" s="33"/>
       <c r="G91" s="6"/>
       <c r="H91" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I91" s="9"/>
-      <c r="J91" s="36" t="s">
+      <c r="J91" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="K91" s="51" t="s">
+      <c r="K91" s="47" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A92" s="28" t="s">
+      <c r="A92" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="B92" s="22"/>
-      <c r="C92" s="36" t="s">
+      <c r="B92" s="5"/>
+      <c r="C92" s="33" t="s">
         <v>154</v>
       </c>
-      <c r="D92" s="60" t="s">
+      <c r="D92" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E92" s="36" t="s">
+      <c r="E92" s="33" t="s">
         <v>155</v>
       </c>
-      <c r="F92" s="36"/>
+      <c r="F92" s="33"/>
       <c r="G92" s="6"/>
       <c r="H92" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I92" s="9"/>
-      <c r="J92" s="36" t="s">
+      <c r="J92" s="33" t="s">
         <v>153</v>
       </c>
-      <c r="K92" s="51"/>
+      <c r="K92" s="47"/>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A93" s="22" t="s">
+      <c r="A93" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B93" s="28" t="s">
+      <c r="B93" s="25" t="s">
         <v>183</v>
       </c>
-      <c r="C93" s="29"/>
-      <c r="D93" s="60" t="s">
+      <c r="C93" s="26"/>
+      <c r="D93" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E93" s="36" t="s">
+      <c r="E93" s="33" t="s">
         <v>182</v>
       </c>
-      <c r="F93" s="39"/>
+      <c r="F93" s="36"/>
       <c r="G93" s="7"/>
       <c r="H93" s="8" t="s">
         <v>166</v>
       </c>
       <c r="I93" s="9"/>
-      <c r="J93" s="29" t="s">
+      <c r="J93" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="K93" s="51"/>
+      <c r="K93" s="47"/>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A94" s="23" t="s">
+      <c r="A94" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B94" s="33"/>
-      <c r="C94" s="36"/>
-      <c r="D94" s="60" t="s">
+      <c r="B94" s="30"/>
+      <c r="C94" s="33"/>
+      <c r="D94" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E94" s="37" t="s">
+      <c r="E94" s="34" t="s">
         <v>179</v>
       </c>
-      <c r="F94" s="36"/>
+      <c r="F94" s="33"/>
       <c r="G94" s="6"/>
       <c r="H94" s="8" t="s">
         <v>166</v>
       </c>
       <c r="I94" s="9"/>
-      <c r="J94" s="36" t="s">
+      <c r="J94" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="K94" s="51"/>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A95" s="28" t="s">
+      <c r="K94" s="47"/>
+    </row>
+    <row r="95" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A95" s="25" t="s">
         <v>246</v>
       </c>
       <c r="B95" s="5"/>
-      <c r="C95" s="29"/>
-      <c r="D95" s="60" t="s">
+      <c r="C95" s="26"/>
+      <c r="D95" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E95" s="37" t="s">
+      <c r="E95" s="34" t="s">
         <v>243</v>
       </c>
-      <c r="F95" s="36"/>
+      <c r="F95" s="33"/>
       <c r="G95" s="19" t="s">
         <v>363</v>
       </c>
@@ -4800,123 +4824,123 @@
         <v>166</v>
       </c>
       <c r="I95" s="9"/>
-      <c r="J95" s="36" t="s">
+      <c r="J95" s="33" t="s">
         <v>244</v>
       </c>
-      <c r="K95" s="51"/>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A96" s="28" t="s">
+      <c r="K95" s="47"/>
+    </row>
+    <row r="96" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A96" s="25" t="s">
         <v>236</v>
       </c>
-      <c r="B96" s="22"/>
-      <c r="C96" s="29"/>
-      <c r="D96" s="60" t="s">
+      <c r="B96" s="5"/>
+      <c r="C96" s="26"/>
+      <c r="D96" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E96" s="36" t="s">
+      <c r="E96" s="33" t="s">
         <v>238</v>
       </c>
-      <c r="F96" s="36"/>
+      <c r="F96" s="33"/>
       <c r="G96" s="19"/>
       <c r="H96" s="8"/>
       <c r="I96" s="9"/>
-      <c r="J96" s="36"/>
-      <c r="K96" s="51"/>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A97" s="28" t="s">
+      <c r="J96" s="33"/>
+      <c r="K96" s="47"/>
+    </row>
+    <row r="97" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A97" s="25" t="s">
         <v>279</v>
       </c>
-      <c r="B97" s="22"/>
-      <c r="C97" s="29"/>
-      <c r="D97" s="60" t="s">
+      <c r="B97" s="5"/>
+      <c r="C97" s="26"/>
+      <c r="D97" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E97" s="36" t="s">
+      <c r="E97" s="33" t="s">
         <v>280</v>
       </c>
-      <c r="F97" s="36"/>
+      <c r="F97" s="33"/>
       <c r="G97" s="19"/>
       <c r="H97" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="I97" s="24"/>
-      <c r="J97" s="36"/>
-      <c r="K97" s="51"/>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A98" s="30" t="s">
+      <c r="I97" s="9"/>
+      <c r="J97" s="33"/>
+      <c r="K97" s="47"/>
+    </row>
+    <row r="98" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A98" s="27" t="s">
         <v>9</v>
       </c>
       <c r="B98" s="5"/>
-      <c r="C98" s="38"/>
-      <c r="D98" s="60" t="s">
+      <c r="C98" s="35"/>
+      <c r="D98" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E98" s="38" t="s">
+      <c r="E98" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="F98" s="38"/>
+      <c r="F98" s="35"/>
       <c r="G98" s="6"/>
       <c r="H98" s="18"/>
       <c r="I98" s="9"/>
-      <c r="J98" s="38" t="s">
+      <c r="J98" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="K98" s="49"/>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A99" s="28" t="s">
+      <c r="K98" s="45"/>
+    </row>
+    <row r="99" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A99" s="25" t="s">
         <v>235</v>
       </c>
       <c r="B99" s="5"/>
-      <c r="C99" s="29"/>
-      <c r="D99" s="60" t="s">
+      <c r="C99" s="26"/>
+      <c r="D99" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E99" s="36"/>
-      <c r="F99" s="36"/>
+      <c r="E99" s="33"/>
+      <c r="F99" s="33"/>
       <c r="G99" s="19"/>
       <c r="H99" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I99" s="9"/>
-      <c r="J99" s="36"/>
-      <c r="K99" s="51"/>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A100" s="22" t="s">
+      <c r="J99" s="33"/>
+      <c r="K99" s="47"/>
+    </row>
+    <row r="100" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A100" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B100" s="28" t="s">
+      <c r="B100" s="25" t="s">
         <v>161</v>
       </c>
-      <c r="C100" s="29"/>
-      <c r="D100" s="60" t="s">
+      <c r="C100" s="26"/>
+      <c r="D100" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E100" s="36"/>
-      <c r="F100" s="39"/>
+      <c r="E100" s="33"/>
+      <c r="F100" s="36"/>
       <c r="G100" s="7"/>
       <c r="H100" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I100" s="9"/>
-      <c r="J100" s="36"/>
-      <c r="K100" s="51"/>
-    </row>
-    <row r="101" spans="1:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="A101" s="22" t="s">
+      <c r="J100" s="33"/>
+      <c r="K100" s="47"/>
+    </row>
+    <row r="101" spans="1:11" ht="17" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A101" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="B101" s="28"/>
-      <c r="C101" s="29"/>
-      <c r="D101" s="60" t="s">
+      <c r="B101" s="25"/>
+      <c r="C101" s="26"/>
+      <c r="D101" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E101" s="36"/>
-      <c r="F101" s="39"/>
+      <c r="E101" s="33"/>
+      <c r="F101" s="36"/>
       <c r="G101" s="7"/>
       <c r="H101" s="8" t="s">
         <v>166</v>
@@ -4924,249 +4948,249 @@
       <c r="I101" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="J101" s="36" t="s">
+      <c r="J101" s="33" t="s">
         <v>247</v>
       </c>
-      <c r="K101" s="51"/>
-    </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A102" s="33" t="s">
+      <c r="K101" s="47"/>
+    </row>
+    <row r="102" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A102" s="30" t="s">
         <v>33</v>
       </c>
       <c r="B102" s="6"/>
-      <c r="C102" s="36"/>
-      <c r="D102" s="60" t="s">
+      <c r="C102" s="33"/>
+      <c r="D102" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E102" s="36"/>
-      <c r="F102" s="36"/>
+      <c r="E102" s="33"/>
+      <c r="F102" s="33"/>
       <c r="G102" s="6"/>
       <c r="H102" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I102" s="9"/>
-      <c r="J102" s="36" t="s">
+      <c r="J102" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="K102" s="51"/>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A103" s="33" t="s">
+      <c r="K102" s="47"/>
+    </row>
+    <row r="103" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A103" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="B103" s="23"/>
-      <c r="C103" s="36"/>
-      <c r="D103" s="60" t="s">
+      <c r="B103" s="6"/>
+      <c r="C103" s="33"/>
+      <c r="D103" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E103" s="36"/>
-      <c r="F103" s="36"/>
+      <c r="E103" s="33"/>
+      <c r="F103" s="33"/>
       <c r="G103" s="6"/>
       <c r="H103" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I103" s="9"/>
-      <c r="J103" s="36" t="s">
+      <c r="J103" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="K103" s="51"/>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A104" s="33" t="s">
+      <c r="K103" s="47"/>
+    </row>
+    <row r="104" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A104" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="B104" s="23"/>
-      <c r="C104" s="36"/>
-      <c r="D104" s="60" t="s">
+      <c r="B104" s="6"/>
+      <c r="C104" s="33"/>
+      <c r="D104" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E104" s="36"/>
-      <c r="F104" s="36"/>
+      <c r="E104" s="33"/>
+      <c r="F104" s="33"/>
       <c r="G104" s="6"/>
       <c r="H104" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I104" s="9"/>
-      <c r="J104" s="36" t="s">
+      <c r="J104" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="K104" s="51"/>
-    </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A105" s="33" t="s">
+      <c r="K104" s="47"/>
+    </row>
+    <row r="105" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A105" s="30" t="s">
         <v>28</v>
       </c>
       <c r="B105" s="6"/>
-      <c r="C105" s="36"/>
-      <c r="D105" s="60" t="s">
+      <c r="C105" s="33"/>
+      <c r="D105" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E105" s="36"/>
-      <c r="F105" s="36"/>
+      <c r="E105" s="33"/>
+      <c r="F105" s="33"/>
       <c r="G105" s="6"/>
       <c r="H105" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I105" s="9"/>
-      <c r="J105" s="36" t="s">
+      <c r="J105" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="K105" s="51"/>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A106" s="33" t="s">
+      <c r="K105" s="47"/>
+    </row>
+    <row r="106" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A106" s="30" t="s">
         <v>23</v>
       </c>
       <c r="B106" s="6"/>
-      <c r="C106" s="36"/>
-      <c r="D106" s="60" t="s">
+      <c r="C106" s="33"/>
+      <c r="D106" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E106" s="36"/>
-      <c r="F106" s="36"/>
+      <c r="E106" s="33"/>
+      <c r="F106" s="33"/>
       <c r="G106" s="6"/>
       <c r="H106" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I106" s="9"/>
-      <c r="J106" s="36" t="s">
+      <c r="J106" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="K106" s="51" t="s">
+      <c r="K106" s="47" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A107" s="33" t="s">
+    <row r="107" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A107" s="30" t="s">
         <v>31</v>
       </c>
       <c r="B107" s="6"/>
-      <c r="C107" s="36"/>
-      <c r="D107" s="60" t="s">
+      <c r="C107" s="33"/>
+      <c r="D107" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E107" s="36"/>
-      <c r="F107" s="36"/>
+      <c r="E107" s="33"/>
+      <c r="F107" s="33"/>
       <c r="G107" s="6"/>
       <c r="H107" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I107" s="9"/>
-      <c r="J107" s="36" t="s">
+      <c r="J107" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="K107" s="51"/>
-    </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A108" s="33" t="s">
+      <c r="K107" s="47"/>
+    </row>
+    <row r="108" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A108" s="30" t="s">
         <v>25</v>
       </c>
       <c r="B108" s="6"/>
-      <c r="C108" s="36"/>
-      <c r="D108" s="60" t="s">
+      <c r="C108" s="33"/>
+      <c r="D108" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E108" s="36"/>
-      <c r="F108" s="36"/>
+      <c r="E108" s="33"/>
+      <c r="F108" s="33"/>
       <c r="G108" s="6"/>
       <c r="H108" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I108" s="9"/>
-      <c r="J108" s="36" t="s">
+      <c r="J108" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="K108" s="51"/>
-    </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A109" s="33" t="s">
+      <c r="K108" s="47"/>
+    </row>
+    <row r="109" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A109" s="30" t="s">
         <v>30</v>
       </c>
       <c r="B109" s="6"/>
-      <c r="C109" s="36"/>
-      <c r="D109" s="60" t="s">
+      <c r="C109" s="33"/>
+      <c r="D109" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E109" s="36"/>
-      <c r="F109" s="36"/>
+      <c r="E109" s="33"/>
+      <c r="F109" s="33"/>
       <c r="G109" s="6"/>
       <c r="H109" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I109" s="9"/>
-      <c r="J109" s="36" t="s">
+      <c r="J109" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="K109" s="51"/>
-    </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A110" s="33" t="s">
+      <c r="K109" s="47"/>
+    </row>
+    <row r="110" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A110" s="30" t="s">
         <v>26</v>
       </c>
       <c r="B110" s="6"/>
-      <c r="C110" s="36"/>
-      <c r="D110" s="60" t="s">
+      <c r="C110" s="33"/>
+      <c r="D110" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E110" s="36"/>
-      <c r="F110" s="36"/>
+      <c r="E110" s="33"/>
+      <c r="F110" s="33"/>
       <c r="G110" s="6"/>
       <c r="H110" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I110" s="9"/>
-      <c r="J110" s="36" t="s">
+      <c r="J110" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="K110" s="51"/>
-    </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A111" s="23" t="s">
+      <c r="K110" s="47"/>
+    </row>
+    <row r="111" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A111" s="6" t="s">
         <v>41</v>
       </c>
       <c r="B111" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C111" s="22"/>
-      <c r="D111" s="60" t="s">
+      <c r="C111" s="5"/>
+      <c r="D111" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E111" s="23"/>
-      <c r="F111" s="23"/>
+      <c r="E111" s="6"/>
+      <c r="F111" s="6"/>
       <c r="G111" s="7"/>
       <c r="H111" s="18" t="s">
         <v>167</v>
       </c>
       <c r="I111" s="9"/>
-      <c r="J111" s="38" t="s">
+      <c r="J111" s="35" t="s">
         <v>213</v>
       </c>
-      <c r="K111" s="49"/>
-    </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A112" s="23" t="s">
+      <c r="K111" s="45"/>
+    </row>
+    <row r="112" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A112" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B112" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="C112" s="22"/>
-      <c r="D112" s="60" t="s">
+      <c r="C112" s="5"/>
+      <c r="D112" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E112" s="23"/>
-      <c r="F112" s="23"/>
+      <c r="E112" s="6"/>
+      <c r="F112" s="6"/>
       <c r="G112" s="7"/>
       <c r="H112" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I112" s="9"/>
-      <c r="J112" s="42" t="s">
+      <c r="J112" s="39" t="s">
         <v>213</v>
       </c>
-      <c r="K112" s="51"/>
-    </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K112" s="47"/>
+    </row>
+    <row r="113" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" s="5"/>
       <c r="B113" s="5"/>
       <c r="C113" s="5"/>
@@ -5176,10 +5200,10 @@
       <c r="G113" s="7"/>
       <c r="H113" s="8"/>
       <c r="I113" s="9"/>
-      <c r="J113" s="29"/>
-      <c r="K113" s="50"/>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J113" s="26"/>
+      <c r="K113" s="46"/>
+    </row>
+    <row r="114" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" s="5"/>
       <c r="B114" s="5"/>
       <c r="C114" s="5"/>
@@ -5189,10 +5213,10 @@
       <c r="G114" s="7"/>
       <c r="H114" s="8"/>
       <c r="I114" s="9"/>
-      <c r="J114" s="26"/>
-      <c r="K114" s="52"/>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J114" s="23"/>
+      <c r="K114" s="48"/>
+    </row>
+    <row r="115" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" s="5"/>
       <c r="B115" s="5"/>
       <c r="C115" s="5"/>
@@ -5202,10 +5226,10 @@
       <c r="G115" s="7"/>
       <c r="H115" s="8"/>
       <c r="I115" s="9"/>
-      <c r="J115" s="29"/>
-      <c r="K115" s="50"/>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J115" s="26"/>
+      <c r="K115" s="46"/>
+    </row>
+    <row r="116" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116" s="5"/>
       <c r="B116" s="5"/>
       <c r="C116" s="5"/>
@@ -5215,10 +5239,10 @@
       <c r="G116" s="7"/>
       <c r="H116" s="8"/>
       <c r="I116" s="9"/>
-      <c r="J116" s="26"/>
-      <c r="K116" s="52"/>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J116" s="23"/>
+      <c r="K116" s="48"/>
+    </row>
+    <row r="117" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117" s="5"/>
       <c r="B117" s="5"/>
       <c r="C117" s="5"/>
@@ -5228,10 +5252,10 @@
       <c r="G117" s="7"/>
       <c r="H117" s="8"/>
       <c r="I117" s="9"/>
-      <c r="J117" s="29"/>
-      <c r="K117" s="50"/>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J117" s="26"/>
+      <c r="K117" s="46"/>
+    </row>
+    <row r="118" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118" s="5"/>
       <c r="B118" s="5"/>
       <c r="C118" s="5"/>
@@ -5241,10 +5265,10 @@
       <c r="G118" s="7"/>
       <c r="H118" s="8"/>
       <c r="I118" s="9"/>
-      <c r="J118" s="26"/>
-      <c r="K118" s="52"/>
-    </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J118" s="23"/>
+      <c r="K118" s="48"/>
+    </row>
+    <row r="119" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" s="5"/>
       <c r="B119" s="5"/>
       <c r="C119" s="5"/>
@@ -5254,23 +5278,23 @@
       <c r="G119" s="7"/>
       <c r="H119" s="8"/>
       <c r="I119" s="9"/>
-      <c r="J119" s="29"/>
-      <c r="K119" s="50"/>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A120" s="22"/>
-      <c r="B120" s="22"/>
-      <c r="C120" s="22"/>
-      <c r="D120" s="23"/>
-      <c r="E120" s="23"/>
-      <c r="F120" s="23"/>
+      <c r="J119" s="26"/>
+      <c r="K119" s="46"/>
+    </row>
+    <row r="120" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A120" s="5"/>
+      <c r="B120" s="5"/>
+      <c r="C120" s="5"/>
+      <c r="D120" s="6"/>
+      <c r="E120" s="6"/>
+      <c r="F120" s="6"/>
       <c r="G120" s="19"/>
       <c r="H120" s="18"/>
-      <c r="I120" s="24"/>
-      <c r="J120" s="27"/>
-      <c r="K120" s="53"/>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I120" s="9"/>
+      <c r="J120" s="24"/>
+      <c r="K120" s="49"/>
+    </row>
+    <row r="121" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" s="5"/>
       <c r="B121" s="5"/>
       <c r="C121" s="5"/>
@@ -5280,10 +5304,10 @@
       <c r="G121" s="7"/>
       <c r="H121" s="8"/>
       <c r="I121" s="9"/>
-      <c r="J121" s="29"/>
-      <c r="K121" s="50"/>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J121" s="26"/>
+      <c r="K121" s="46"/>
+    </row>
+    <row r="122" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A122" s="5"/>
       <c r="B122" s="5"/>
       <c r="C122" s="5"/>
@@ -5293,10 +5317,10 @@
       <c r="G122" s="7"/>
       <c r="H122" s="8"/>
       <c r="I122" s="9"/>
-      <c r="J122" s="26"/>
-      <c r="K122" s="52"/>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J122" s="23"/>
+      <c r="K122" s="48"/>
+    </row>
+    <row r="123" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A123" s="5"/>
       <c r="B123" s="5"/>
       <c r="C123" s="5"/>
@@ -5306,10 +5330,10 @@
       <c r="G123" s="7"/>
       <c r="H123" s="8"/>
       <c r="I123" s="9"/>
-      <c r="J123" s="29"/>
-      <c r="K123" s="50"/>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J123" s="26"/>
+      <c r="K123" s="46"/>
+    </row>
+    <row r="124" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A124" s="5"/>
       <c r="B124" s="5"/>
       <c r="C124" s="5"/>
@@ -5319,10 +5343,10 @@
       <c r="G124" s="7"/>
       <c r="H124" s="8"/>
       <c r="I124" s="9"/>
-      <c r="J124" s="26"/>
-      <c r="K124" s="52"/>
-    </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J124" s="23"/>
+      <c r="K124" s="48"/>
+    </row>
+    <row r="125" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A125" s="5"/>
       <c r="B125" s="5"/>
       <c r="C125" s="5"/>
@@ -5332,10 +5356,10 @@
       <c r="G125" s="7"/>
       <c r="H125" s="8"/>
       <c r="I125" s="9"/>
-      <c r="J125" s="29"/>
-      <c r="K125" s="50"/>
-    </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J125" s="26"/>
+      <c r="K125" s="46"/>
+    </row>
+    <row r="126" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A126" s="5"/>
       <c r="B126" s="5"/>
       <c r="C126" s="5"/>
@@ -5345,10 +5369,10 @@
       <c r="G126" s="7"/>
       <c r="H126" s="8"/>
       <c r="I126" s="9"/>
-      <c r="J126" s="26"/>
-      <c r="K126" s="52"/>
-    </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J126" s="23"/>
+      <c r="K126" s="48"/>
+    </row>
+    <row r="127" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A127" s="5"/>
       <c r="B127" s="5"/>
       <c r="C127" s="5"/>
@@ -5358,23 +5382,23 @@
       <c r="G127" s="7"/>
       <c r="H127" s="8"/>
       <c r="I127" s="9"/>
-      <c r="J127" s="29"/>
-      <c r="K127" s="50"/>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A128" s="22"/>
-      <c r="B128" s="22"/>
-      <c r="C128" s="22"/>
-      <c r="D128" s="23"/>
-      <c r="E128" s="23"/>
-      <c r="F128" s="23"/>
+      <c r="J127" s="26"/>
+      <c r="K127" s="46"/>
+    </row>
+    <row r="128" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A128" s="5"/>
+      <c r="B128" s="5"/>
+      <c r="C128" s="5"/>
+      <c r="D128" s="6"/>
+      <c r="E128" s="6"/>
+      <c r="F128" s="6"/>
       <c r="G128" s="19"/>
       <c r="H128" s="18"/>
-      <c r="I128" s="24"/>
-      <c r="J128" s="27"/>
-      <c r="K128" s="53"/>
-    </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I128" s="9"/>
+      <c r="J128" s="24"/>
+      <c r="K128" s="49"/>
+    </row>
+    <row r="129" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A129" s="5"/>
       <c r="B129" s="5"/>
       <c r="C129" s="5"/>
@@ -5384,10 +5408,10 @@
       <c r="G129" s="7"/>
       <c r="H129" s="8"/>
       <c r="I129" s="9"/>
-      <c r="J129" s="29"/>
-      <c r="K129" s="50"/>
-    </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J129" s="26"/>
+      <c r="K129" s="46"/>
+    </row>
+    <row r="130" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A130" s="5"/>
       <c r="B130" s="5"/>
       <c r="C130" s="5"/>
@@ -5397,21 +5421,21 @@
       <c r="G130" s="7"/>
       <c r="H130" s="8"/>
       <c r="I130" s="9"/>
-      <c r="J130" s="26"/>
-      <c r="K130" s="52"/>
-    </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A131" s="22"/>
-      <c r="B131" s="22"/>
-      <c r="C131" s="22"/>
-      <c r="D131" s="23"/>
-      <c r="E131" s="23"/>
-      <c r="F131" s="23"/>
+      <c r="J130" s="23"/>
+      <c r="K130" s="48"/>
+    </row>
+    <row r="131" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A131" s="5"/>
+      <c r="B131" s="5"/>
+      <c r="C131" s="5"/>
+      <c r="D131" s="6"/>
+      <c r="E131" s="6"/>
+      <c r="F131" s="6"/>
       <c r="G131" s="19"/>
       <c r="H131" s="18"/>
-      <c r="I131" s="24"/>
-      <c r="J131" s="31"/>
-      <c r="K131" s="54"/>
+      <c r="I131" s="9"/>
+      <c r="J131" s="28"/>
+      <c r="K131" s="50"/>
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H132"/>

</xml_diff>

<commit_message>
added stage display tv network parms
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40F3D613-8BD4-5143-8AC8-92673D0E6EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7826427-D20E-2B4F-B2F3-A253EA5A5785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1880" yWindow="2960" windowWidth="28360" windowHeight="16680" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
@@ -2400,7 +2400,7 @@
         <v>195</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
@@ -2452,7 +2452,7 @@
         <v>203</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
@@ -2506,7 +2506,7 @@
         <v>219</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
@@ -2558,7 +2558,7 @@
         <v>206</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>

</xml_diff>

<commit_message>
updated Shure and klang details
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{175679B4-B78B-5B4B-9E36-8C37992ABEA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6FF314F-24EB-D54E-8C05-752BA5BAE09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="2960" windowWidth="29920" windowHeight="16680" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="795" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="438">
   <si>
     <t>NSCU-A004</t>
   </si>
@@ -839,18 +839,6 @@
     <t>Manage via Dante Controller.</t>
   </si>
   <si>
-    <t>192.168.200.134</t>
-  </si>
-  <si>
-    <t>192.168.200.154</t>
-  </si>
-  <si>
-    <t>192.168.200.132</t>
-  </si>
-  <si>
-    <t>192.168.200.170</t>
-  </si>
-  <si>
     <t>KB0034</t>
   </si>
   <si>
@@ -1244,12 +1232,6 @@
     <t>notag45</t>
   </si>
   <si>
-    <t>pending93</t>
-  </si>
-  <si>
-    <t>pending100</t>
-  </si>
-  <si>
     <t>dante_control</t>
   </si>
   <si>
@@ -1383,6 +1365,51 @@
   </si>
   <si>
     <t>builtin AVNET</t>
+  </si>
+  <si>
+    <t>80:6d: 97:20:a7:8e</t>
+  </si>
+  <si>
+    <t>14:98:77:81:27:3f</t>
+  </si>
+  <si>
+    <t>172.31.99.182</t>
+  </si>
+  <si>
+    <t>SSID UAC</t>
+  </si>
+  <si>
+    <t>2509-1704</t>
+  </si>
+  <si>
+    <t>2509-1705</t>
+  </si>
+  <si>
+    <t>00-0E-DD-2C-03-83</t>
+  </si>
+  <si>
+    <t>00-0E-DD-2C-02-C8</t>
+  </si>
+  <si>
+    <t>192.168.200.116</t>
+  </si>
+  <si>
+    <t>192.168.200.117</t>
+  </si>
+  <si>
+    <t>IEM xmtr</t>
+  </si>
+  <si>
+    <t>unused</t>
+  </si>
+  <si>
+    <t>192.168.200.150</t>
+  </si>
+  <si>
+    <t>192.168.200.152</t>
+  </si>
+  <si>
+    <t>192.168.200.153</t>
   </si>
 </sst>
 </file>
@@ -2042,13 +2069,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}" name="Table1" displayName="Table1" ref="A1:K135" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:K135" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="CUMU-G002"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:K135" xr:uid="{157AC5DF-1534-C144-A7F4-07F88FA8E6FA}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{EF2C341F-E5C1-604C-942C-FB7E9F76F1CD}" name="AssetTag" dataDxfId="10"/>
     <tableColumn id="13" xr3:uid="{41250547-1480-7146-952C-14798A4748DA}" name="NIC" dataDxfId="9"/>
@@ -2369,7 +2390,7 @@
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.1640625" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="8.1640625" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.1640625" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="22.5" customWidth="1"/>
@@ -2416,13 +2437,13 @@
         <v>138</v>
       </c>
     </row>
-    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>236</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>100</v>
@@ -2443,7 +2464,7 @@
       </c>
       <c r="K2" s="41"/>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>189</v>
       </c>
@@ -2470,7 +2491,7 @@
       </c>
       <c r="K3" s="41"/>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>189</v>
       </c>
@@ -2481,7 +2502,7 @@
         <v>195</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
@@ -2495,7 +2516,7 @@
       </c>
       <c r="K4" s="41"/>
     </row>
-    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>207</v>
       </c>
@@ -2522,7 +2543,7 @@
       </c>
       <c r="K5" s="41"/>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>207</v>
       </c>
@@ -2533,7 +2554,7 @@
         <v>203</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
@@ -2547,7 +2568,7 @@
       </c>
       <c r="K6" s="41"/>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>214</v>
       </c>
@@ -2576,7 +2597,7 @@
       </c>
       <c r="K7" s="41"/>
     </row>
-    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>214</v>
       </c>
@@ -2587,7 +2608,7 @@
         <v>219</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
@@ -2601,7 +2622,7 @@
       </c>
       <c r="K8" s="41"/>
     </row>
-    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>213</v>
       </c>
@@ -2628,7 +2649,7 @@
       </c>
       <c r="K9" s="41"/>
     </row>
-    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>213</v>
       </c>
@@ -2639,7 +2660,7 @@
         <v>206</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
@@ -2653,24 +2674,24 @@
       </c>
       <c r="K10" s="41"/>
     </row>
-    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="29" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="F11" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>229</v>
@@ -2680,28 +2701,28 @@
       </c>
       <c r="I11" s="9"/>
       <c r="J11" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="K11" s="44"/>
     </row>
-    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>229</v>
@@ -2711,25 +2732,25 @@
       </c>
       <c r="I12" s="9"/>
       <c r="J12" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="K12" s="43"/>
     </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="7" t="s">
@@ -2740,28 +2761,28 @@
       </c>
       <c r="I13" s="9"/>
       <c r="J13" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="K13" s="43"/>
     </row>
-    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>229</v>
@@ -2771,28 +2792,28 @@
       </c>
       <c r="I14" s="9"/>
       <c r="J14" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="K14" s="43"/>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G15" s="7" t="s">
         <v>229</v>
@@ -2802,28 +2823,28 @@
       </c>
       <c r="I15" s="9"/>
       <c r="J15" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="K15" s="43"/>
     </row>
-    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>229</v>
@@ -2833,28 +2854,28 @@
       </c>
       <c r="I16" s="9"/>
       <c r="J16" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="K16" s="43"/>
     </row>
-    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="29" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="F17" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>229</v>
@@ -2864,28 +2885,28 @@
       </c>
       <c r="I17" s="9"/>
       <c r="J17" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="K17" s="44"/>
     </row>
-    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="29" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E18" s="29" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="F18" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>229</v>
@@ -2895,28 +2916,28 @@
       </c>
       <c r="I18" s="9"/>
       <c r="J18" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="K18" s="44"/>
     </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>229</v>
@@ -2926,28 +2947,28 @@
       </c>
       <c r="I19" s="9"/>
       <c r="J19" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="K19" s="43"/>
     </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="29" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E20" s="29" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="F20" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G20" s="7" t="s">
         <v>229</v>
@@ -2957,26 +2978,26 @@
       </c>
       <c r="I20" s="9"/>
       <c r="J20" s="5" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="K20" s="44"/>
     </row>
-    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="B21" s="29"/>
       <c r="C21" s="29" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E21" s="29" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="F21" s="29" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="G21" s="7"/>
       <c r="H21" s="8"/>
@@ -2984,11 +3005,13 @@
       <c r="J21" s="6"/>
       <c r="K21" s="41"/>
     </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B22" s="6"/>
+      <c r="B22" s="6" t="s">
+        <v>190</v>
+      </c>
       <c r="C22" s="20" t="s">
         <v>54</v>
       </c>
@@ -2996,7 +3019,7 @@
         <v>35</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>247</v>
+        <v>435</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
@@ -3004,7 +3027,7 @@
         <v>166</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="J22" s="6" t="s">
         <v>44</v>
@@ -3013,11 +3036,13 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B23" s="6"/>
+      <c r="B23" s="6" t="s">
+        <v>190</v>
+      </c>
       <c r="C23" s="20" t="s">
         <v>43</v>
       </c>
@@ -3025,7 +3050,7 @@
         <v>35</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>250</v>
+        <v>437</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
@@ -3033,7 +3058,7 @@
         <v>166</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="J23" s="6" t="s">
         <v>44</v>
@@ -3042,11 +3067,13 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B24" s="6"/>
+      <c r="B24" s="6" t="s">
+        <v>190</v>
+      </c>
       <c r="C24" s="20" t="s">
         <v>46</v>
       </c>
@@ -3054,7 +3081,7 @@
         <v>35</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>249</v>
+        <v>436</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
@@ -3062,7 +3089,7 @@
         <v>166</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="J24" s="6" t="s">
         <v>44</v>
@@ -3071,11 +3098,13 @@
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="6"/>
+      <c r="B25" s="6" t="s">
+        <v>190</v>
+      </c>
       <c r="C25" s="20" t="s">
         <v>48</v>
       </c>
@@ -3083,7 +3112,7 @@
         <v>35</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>248</v>
+        <v>361</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
@@ -3091,7 +3120,7 @@
         <v>166</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>44</v>
@@ -3100,7 +3129,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
         <v>137</v>
       </c>
@@ -3127,13 +3156,13 @@
         <v>74</v>
       </c>
     </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>100</v>
@@ -3145,22 +3174,22 @@
       <c r="I27" s="9"/>
       <c r="J27" s="6"/>
       <c r="K27" s="41" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
         <v>93</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="F28" s="19" t="str">
         <f>CONCATENATE("http://", E28)</f>
@@ -3180,7 +3209,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
         <v>41</v>
       </c>
@@ -3209,7 +3238,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
         <v>38</v>
       </c>
@@ -3238,7 +3267,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
         <v>6</v>
       </c>
@@ -3259,11 +3288,11 @@
       </c>
       <c r="I31" s="9"/>
       <c r="J31" s="6" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="K31" s="41"/>
     </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
         <v>198</v>
       </c>
@@ -3286,11 +3315,11 @@
       </c>
       <c r="I32" s="9"/>
       <c r="J32" s="5" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="K32" s="41"/>
     </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
         <v>220</v>
       </c>
@@ -3315,22 +3344,22 @@
       </c>
       <c r="K33" s="41"/>
     </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G34" s="7"/>
       <c r="H34" s="8"/>
@@ -3338,22 +3367,22 @@
       <c r="J34" s="6"/>
       <c r="K34" s="41"/>
     </row>
-    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="B35" s="29"/>
       <c r="C35" s="29" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E35" s="29" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="F35" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G35" s="19"/>
       <c r="H35" s="8"/>
@@ -3361,22 +3390,22 @@
       <c r="J35" s="6"/>
       <c r="K35" s="41"/>
     </row>
-    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="B36" s="29"/>
       <c r="C36" s="29" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E36" s="29" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="F36" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G36" s="7"/>
       <c r="H36" s="8"/>
@@ -3384,22 +3413,22 @@
       <c r="J36" s="6"/>
       <c r="K36" s="41"/>
     </row>
-    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="B37" s="29"/>
       <c r="C37" s="29" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E37" s="29" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="F37" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G37" s="7"/>
       <c r="H37" s="8"/>
@@ -3407,232 +3436,232 @@
       <c r="J37" s="6"/>
       <c r="K37" s="41"/>
     </row>
-    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="B38" s="29"/>
       <c r="C38" s="29" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E38" s="29" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="F38" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G38" s="7"/>
       <c r="H38" s="8"/>
       <c r="I38" s="9"/>
       <c r="J38" s="6"/>
       <c r="K38" s="41" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="B39" s="29"/>
       <c r="C39" s="29" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E39" s="29" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="F39" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G39" s="7"/>
       <c r="H39" s="8"/>
       <c r="I39" s="9"/>
       <c r="J39" s="6"/>
       <c r="K39" s="41" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="B40" s="29"/>
       <c r="C40" s="29" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E40" s="29" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="F40" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G40" s="7"/>
       <c r="H40" s="8"/>
       <c r="I40" s="9"/>
       <c r="J40" s="6"/>
       <c r="K40" s="41" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="B41" s="5"/>
       <c r="C41" s="5" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D41" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G41" s="7"/>
       <c r="H41" s="8"/>
       <c r="I41" s="9"/>
       <c r="J41" s="6"/>
       <c r="K41" s="41" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="B42" s="5"/>
       <c r="C42" s="5" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G42" s="7"/>
       <c r="H42" s="8"/>
       <c r="I42" s="9"/>
       <c r="J42" s="6"/>
       <c r="K42" s="41" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="5" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G43" s="7"/>
       <c r="H43" s="8"/>
       <c r="I43" s="9"/>
       <c r="J43" s="6"/>
       <c r="K43" s="41" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="5" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G44" s="7"/>
       <c r="H44" s="8"/>
       <c r="I44" s="9"/>
       <c r="J44" s="6"/>
       <c r="K44" s="41" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="B45" s="29"/>
       <c r="C45" s="29" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E45" s="29" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="F45" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G45" s="7"/>
       <c r="H45" s="8"/>
       <c r="I45" s="9"/>
       <c r="J45" s="6"/>
       <c r="K45" s="41" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="B46" s="29"/>
       <c r="C46" s="29" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E46" s="29" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="F46" s="29" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="G46" s="19"/>
       <c r="H46" s="8"/>
       <c r="I46" s="9"/>
       <c r="J46" s="6"/>
       <c r="K46" s="41" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
         <v>108</v>
       </c>
@@ -3662,7 +3691,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
         <v>103</v>
       </c>
@@ -3692,7 +3721,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" s="6" t="s">
         <v>86</v>
       </c>
@@ -3722,7 +3751,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
         <v>232</v>
       </c>
@@ -3751,9 +3780,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="31" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="B51" s="13"/>
       <c r="C51" s="5" t="s">
@@ -3776,7 +3805,7 @@
       <c r="J51" s="6"/>
       <c r="K51" s="41"/>
     </row>
-    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
         <v>27</v>
       </c>
@@ -3806,7 +3835,7 @@
       </c>
       <c r="K52" s="42"/>
     </row>
-    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" s="6" t="s">
         <v>2</v>
       </c>
@@ -3836,7 +3865,7 @@
       </c>
       <c r="K53" s="42"/>
     </row>
-    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" s="6" t="s">
         <v>130</v>
       </c>
@@ -3859,7 +3888,7 @@
       </c>
       <c r="K54" s="42"/>
     </row>
-    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" s="6" t="s">
         <v>7</v>
       </c>
@@ -3889,7 +3918,7 @@
       </c>
       <c r="K55" s="42"/>
     </row>
-    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
         <v>0</v>
       </c>
@@ -3919,7 +3948,7 @@
       </c>
       <c r="K56" s="41"/>
     </row>
-    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" s="6" t="s">
         <v>24</v>
       </c>
@@ -3949,7 +3978,7 @@
       </c>
       <c r="K57" s="42"/>
     </row>
-    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" s="10" t="s">
         <v>53</v>
       </c>
@@ -3979,7 +4008,7 @@
       </c>
       <c r="K58" s="41"/>
     </row>
-    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" s="6" t="s">
         <v>73</v>
       </c>
@@ -4011,7 +4040,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
         <v>116</v>
       </c>
@@ -4041,7 +4070,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" s="6" t="s">
         <v>112</v>
       </c>
@@ -4064,7 +4093,7 @@
         <v>166</v>
       </c>
       <c r="I61" s="9" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="J61" s="6" t="s">
         <v>111</v>
@@ -4073,19 +4102,19 @@
         <v>61</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" s="5" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="B62" s="5"/>
       <c r="C62" s="5" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="D62" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="F62" s="6"/>
       <c r="G62" s="19"/>
@@ -4094,13 +4123,13 @@
       </c>
       <c r="I62" s="9"/>
       <c r="J62" s="6" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="K62" s="41">
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" s="5" t="s">
         <v>3</v>
       </c>
@@ -4125,17 +4154,15 @@
       </c>
       <c r="I63" s="9"/>
       <c r="J63" s="6"/>
-      <c r="K63" s="41">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+      <c r="K63" s="41"/>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" s="17" t="s">
         <v>224</v>
       </c>
       <c r="B64" s="5"/>
       <c r="C64" s="6" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="D64" s="6" t="s">
         <v>100</v>
@@ -4154,13 +4181,13 @@
       </c>
       <c r="K64" s="41"/>
     </row>
-    <row r="65" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" s="5" t="s">
         <v>151</v>
       </c>
       <c r="B65" s="5"/>
       <c r="C65" s="6" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>100</v>
@@ -4181,7 +4208,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" s="5" t="s">
         <v>145</v>
       </c>
@@ -4209,7 +4236,7 @@
       </c>
       <c r="K66" s="41"/>
     </row>
-    <row r="67" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" s="5" t="s">
         <v>1</v>
       </c>
@@ -4227,7 +4254,7 @@
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="H67" s="18" t="s">
         <v>166</v>
@@ -4238,7 +4265,7 @@
       </c>
       <c r="K67" s="41"/>
     </row>
-    <row r="68" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68" s="5" t="s">
         <v>1</v>
       </c>
@@ -4256,7 +4283,7 @@
       </c>
       <c r="F68" s="6"/>
       <c r="G68" s="6" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="H68" s="18" t="s">
         <v>166</v>
@@ -4267,19 +4294,19 @@
       </c>
       <c r="K68" s="41"/>
     </row>
-    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69" s="5" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B69" s="5"/>
       <c r="C69" s="53" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="D69" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="F69" s="6"/>
       <c r="G69" s="19" t="s">
@@ -4290,25 +4317,25 @@
       </c>
       <c r="I69" s="9"/>
       <c r="J69" s="5" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="K69" s="44" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70" s="5" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="B70" s="5"/>
       <c r="C70" s="53" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="D70" s="54" t="s">
         <v>100</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="F70" s="6"/>
       <c r="G70" s="19" t="s">
@@ -4319,13 +4346,13 @@
       </c>
       <c r="I70" s="9"/>
       <c r="J70" s="38" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="K70" s="43" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A71" s="6" t="s">
         <v>97</v>
       </c>
@@ -4345,7 +4372,7 @@
         <v>166</v>
       </c>
       <c r="I71" s="9" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="J71" s="6" t="s">
         <v>96</v>
@@ -4354,7 +4381,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A72" s="6" t="s">
         <v>60</v>
       </c>
@@ -4379,7 +4406,7 @@
         <v>166</v>
       </c>
       <c r="I72" s="9" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="J72" s="6" t="s">
         <v>59</v>
@@ -4388,19 +4415,19 @@
         <v>56</v>
       </c>
     </row>
-    <row r="73" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B73" s="5"/>
       <c r="C73" s="5" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="D73" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="F73" s="6"/>
       <c r="G73" s="7" t="s">
@@ -4415,19 +4442,19 @@
       </c>
       <c r="K73" s="41"/>
     </row>
-    <row r="74" spans="1:11" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:11" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A74" s="22" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="B74" s="5"/>
       <c r="C74" s="5" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D74" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="F74" s="6"/>
       <c r="G74" s="7" t="s">
@@ -4442,7 +4469,7 @@
       </c>
       <c r="K74" s="41"/>
     </row>
-    <row r="75" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A75" s="6" t="s">
         <v>81</v>
       </c>
@@ -4465,7 +4492,7 @@
         <v>166</v>
       </c>
       <c r="I75" s="9" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="J75" s="6" t="s">
         <v>77</v>
@@ -4474,7 +4501,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A76" s="6" t="s">
         <v>78</v>
       </c>
@@ -4497,7 +4524,7 @@
         <v>166</v>
       </c>
       <c r="I76" s="9" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="J76" s="6" t="s">
         <v>77</v>
@@ -4506,13 +4533,13 @@
         <v>74</v>
       </c>
     </row>
-    <row r="77" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" s="5" t="s">
         <v>158</v>
       </c>
       <c r="B77" s="25"/>
       <c r="C77" s="33" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D77" s="54" t="s">
         <v>100</v>
@@ -4527,13 +4554,13 @@
       </c>
       <c r="I77" s="9"/>
       <c r="J77" s="6" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="K77" s="41">
         <v>18</v>
       </c>
     </row>
-    <row r="78" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78" s="6" t="s">
         <v>91</v>
       </c>
@@ -4560,13 +4587,13 @@
         <v>87</v>
       </c>
     </row>
-    <row r="79" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" s="5" t="s">
         <v>159</v>
       </c>
       <c r="B79" s="25"/>
       <c r="C79" s="26" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="D79" s="54" t="s">
         <v>100</v>
@@ -4575,21 +4602,21 @@
         <v>156</v>
       </c>
       <c r="F79" s="26" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="G79" s="7"/>
       <c r="H79" s="8"/>
       <c r="I79" s="9"/>
       <c r="J79" s="29" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="K79" s="43">
         <v>14</v>
       </c>
     </row>
-    <row r="80" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80" s="5" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="B80" s="25" t="s">
         <v>174</v>
@@ -4616,19 +4643,19 @@
       </c>
       <c r="K80" s="41"/>
     </row>
-    <row r="81" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" s="5" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="B81" s="27"/>
       <c r="C81" s="28" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="D81" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E81" s="35" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="F81" s="35"/>
       <c r="G81" s="7" t="s">
@@ -4643,19 +4670,19 @@
       </c>
       <c r="K81" s="41"/>
     </row>
-    <row r="82" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" s="5" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="B82" s="25"/>
       <c r="C82" s="26" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D82" s="54" t="s">
         <v>100</v>
       </c>
       <c r="E82" s="33" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="F82" s="33"/>
       <c r="G82" s="19"/>
@@ -4664,7 +4691,7 @@
       </c>
       <c r="I82" s="9"/>
       <c r="J82" s="6" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="K82" s="41"/>
     </row>
@@ -4691,7 +4718,7 @@
       </c>
       <c r="I83" s="9"/>
       <c r="J83" s="6" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="K83" s="41">
         <v>10</v>
@@ -4702,7 +4729,7 @@
         <v>168</v>
       </c>
       <c r="B84" s="25" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="C84" s="26" t="s">
         <v>184</v>
@@ -4726,19 +4753,19 @@
       </c>
       <c r="K84" s="41"/>
     </row>
-    <row r="85" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85" s="5" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="B85" s="25"/>
       <c r="C85" s="23" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="D85" s="54" t="s">
         <v>100</v>
       </c>
       <c r="E85" s="33" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="F85" s="33"/>
       <c r="G85" s="19" t="s">
@@ -4749,13 +4776,13 @@
       </c>
       <c r="I85" s="9"/>
       <c r="J85" s="6" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="K85" s="44">
         <v>4</v>
       </c>
     </row>
-    <row r="86" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86" s="30" t="s">
         <v>65</v>
       </c>
@@ -4787,7 +4814,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="87" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" s="52" t="s">
         <v>69</v>
       </c>
@@ -4819,7 +4846,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="88" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88" s="32" t="s">
         <v>18</v>
       </c>
@@ -4844,7 +4871,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="89" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" s="6" t="s">
         <v>120</v>
       </c>
@@ -4874,19 +4901,19 @@
         <v>70</v>
       </c>
     </row>
-    <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A90" s="5" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
       <c r="B90" s="25"/>
       <c r="C90" s="26" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="D90" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E90" s="33" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="F90" s="33"/>
       <c r="G90" s="19" t="s">
@@ -4897,23 +4924,23 @@
       </c>
       <c r="I90" s="9"/>
       <c r="J90" s="33" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="K90" s="47"/>
     </row>
-    <row r="91" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91" s="25" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="B91" s="5"/>
       <c r="C91" s="26" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="D91" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E91" s="33" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="F91" s="33"/>
       <c r="G91" s="19" t="s">
@@ -4924,13 +4951,13 @@
       </c>
       <c r="I91" s="9"/>
       <c r="J91" s="33" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="K91" s="47">
         <v>13</v>
       </c>
     </row>
-    <row r="92" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92" s="5" t="s">
         <v>14</v>
       </c>
@@ -4955,7 +4982,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="93" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93" s="25" t="s">
         <v>152</v>
       </c>
@@ -4980,7 +5007,7 @@
       </c>
       <c r="K93" s="47"/>
     </row>
-    <row r="94" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A94" s="5" t="s">
         <v>3</v>
       </c>
@@ -4988,7 +5015,7 @@
         <v>183</v>
       </c>
       <c r="C94" s="26" t="s">
-        <v>382</v>
+        <v>423</v>
       </c>
       <c r="D94" s="54" t="s">
         <v>100</v>
@@ -5007,7 +5034,7 @@
       </c>
       <c r="K94" s="47"/>
     </row>
-    <row r="95" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" s="6" t="s">
         <v>20</v>
       </c>
@@ -5030,7 +5057,7 @@
       </c>
       <c r="K95" s="47"/>
     </row>
-    <row r="96" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96" s="25" t="s">
         <v>245</v>
       </c>
@@ -5044,7 +5071,7 @@
       </c>
       <c r="F96" s="33"/>
       <c r="G96" s="19" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="H96" s="8" t="s">
         <v>166</v>
@@ -5055,7 +5082,7 @@
       </c>
       <c r="K96" s="47"/>
     </row>
-    <row r="97" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" s="25" t="s">
         <v>235</v>
       </c>
@@ -5074,9 +5101,9 @@
       <c r="J97" s="33"/>
       <c r="K97" s="47"/>
     </row>
-    <row r="98" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" s="25" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="B98" s="5"/>
       <c r="C98" s="26"/>
@@ -5084,7 +5111,7 @@
         <v>100</v>
       </c>
       <c r="E98" s="33" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="F98" s="33"/>
       <c r="G98" s="19"/>
@@ -5095,7 +5122,7 @@
       <c r="J98" s="33"/>
       <c r="K98" s="47"/>
     </row>
-    <row r="99" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99" s="27" t="s">
         <v>9</v>
       </c>
@@ -5116,7 +5143,7 @@
       </c>
       <c r="K99" s="45"/>
     </row>
-    <row r="100" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" s="25" t="s">
         <v>234</v>
       </c>
@@ -5135,44 +5162,48 @@
       <c r="J100" s="33"/>
       <c r="K100" s="47"/>
     </row>
-    <row r="101" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B101" s="25" t="s">
-        <v>161</v>
+        <v>420</v>
       </c>
       <c r="C101" s="26" t="s">
-        <v>383</v>
+        <v>424</v>
       </c>
       <c r="D101" s="54" t="s">
         <v>100</v>
       </c>
-      <c r="E101" s="33"/>
+      <c r="E101" s="33" t="s">
+        <v>425</v>
+      </c>
       <c r="F101" s="36"/>
       <c r="G101" s="7"/>
       <c r="H101" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I101" s="9"/>
-      <c r="J101" s="33"/>
+      <c r="J101" s="33" t="s">
+        <v>426</v>
+      </c>
       <c r="K101" s="47"/>
     </row>
     <row r="102" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A102" s="5" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
       <c r="B102" s="25" t="s">
         <v>174</v>
       </c>
       <c r="C102" s="26" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="D102" s="54" t="s">
         <v>100</v>
       </c>
       <c r="E102" s="33" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
       <c r="F102" s="36"/>
       <c r="G102" s="7"/>
@@ -5180,14 +5211,14 @@
         <v>166</v>
       </c>
       <c r="I102" s="1" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="J102" s="33" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="K102" s="47"/>
     </row>
-    <row r="103" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" s="30" t="s">
         <v>33</v>
       </c>
@@ -5208,7 +5239,7 @@
       </c>
       <c r="K103" s="47"/>
     </row>
-    <row r="104" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" s="30" t="s">
         <v>32</v>
       </c>
@@ -5229,7 +5260,7 @@
       </c>
       <c r="K104" s="47"/>
     </row>
-    <row r="105" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105" s="30" t="s">
         <v>29</v>
       </c>
@@ -5250,7 +5281,7 @@
       </c>
       <c r="K105" s="47"/>
     </row>
-    <row r="106" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106" s="30" t="s">
         <v>28</v>
       </c>
@@ -5271,7 +5302,7 @@
       </c>
       <c r="K106" s="47"/>
     </row>
-    <row r="107" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A107" s="30" t="s">
         <v>23</v>
       </c>
@@ -5294,7 +5325,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="108" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108" s="30" t="s">
         <v>31</v>
       </c>
@@ -5315,7 +5346,7 @@
       </c>
       <c r="K108" s="47"/>
     </row>
-    <row r="109" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A109" s="30" t="s">
         <v>25</v>
       </c>
@@ -5336,7 +5367,7 @@
       </c>
       <c r="K109" s="47"/>
     </row>
-    <row r="110" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110" s="30" t="s">
         <v>30</v>
       </c>
@@ -5357,7 +5388,7 @@
       </c>
       <c r="K110" s="47"/>
     </row>
-    <row r="111" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A111" s="30" t="s">
         <v>26</v>
       </c>
@@ -5378,7 +5409,7 @@
       </c>
       <c r="K111" s="47"/>
     </row>
-    <row r="112" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A112" s="6" t="s">
         <v>41</v>
       </c>
@@ -5401,7 +5432,7 @@
       </c>
       <c r="K112" s="45"/>
     </row>
-    <row r="113" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A113" s="6" t="s">
         <v>38</v>
       </c>
@@ -5424,21 +5455,21 @@
       </c>
       <c r="K113" s="47"/>
     </row>
-    <row r="114" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A114" s="55" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="B114" s="5" t="s">
         <v>161</v>
       </c>
       <c r="C114" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="D114" s="6" t="s">
         <v>391</v>
       </c>
-      <c r="D114" s="6" t="s">
-        <v>397</v>
-      </c>
       <c r="E114" s="6" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="F114" s="6"/>
       <c r="G114" s="7"/>
@@ -5449,50 +5480,50 @@
       <c r="J114" s="26"/>
       <c r="K114" s="46"/>
     </row>
-    <row r="115" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A115" s="55" t="s">
+        <v>383</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="C115" s="5" t="s">
         <v>389</v>
-      </c>
-      <c r="B115" s="5" t="s">
-        <v>390</v>
-      </c>
-      <c r="C115" s="5" t="s">
-        <v>395</v>
       </c>
       <c r="D115" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E115" s="6" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="F115" s="6"/>
       <c r="G115" s="7" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="H115" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I115" s="9"/>
       <c r="J115" s="23" t="s">
+        <v>387</v>
+      </c>
+      <c r="K115" s="48"/>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A116" s="55" t="s">
+        <v>392</v>
+      </c>
+      <c r="B116" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="C116" s="5" t="s">
         <v>393</v>
-      </c>
-      <c r="K115" s="48"/>
-    </row>
-    <row r="116" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A116" s="55" t="s">
-        <v>398</v>
-      </c>
-      <c r="B116" s="5" t="s">
-        <v>390</v>
-      </c>
-      <c r="C116" s="5" t="s">
-        <v>399</v>
       </c>
       <c r="D116" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="F116" s="6"/>
       <c r="G116" s="7"/>
@@ -5501,27 +5532,27 @@
       </c>
       <c r="I116" s="9"/>
       <c r="J116" s="26" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="K116" s="46" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="117" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A117" s="55" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="C117" s="5" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="D117" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="F117" s="6"/>
       <c r="G117" s="7"/>
@@ -5530,25 +5561,25 @@
       </c>
       <c r="I117" s="9"/>
       <c r="J117" s="23" t="s">
+        <v>396</v>
+      </c>
+      <c r="K117" s="48"/>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A118" s="55" t="s">
         <v>402</v>
       </c>
-      <c r="K117" s="48"/>
-    </row>
-    <row r="118" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A118" s="55" t="s">
-        <v>408</v>
-      </c>
       <c r="B118" s="5" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="C118" s="5" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
       <c r="D118" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
       <c r="F118" s="6"/>
       <c r="G118" s="7"/>
@@ -5557,50 +5588,50 @@
       </c>
       <c r="I118" s="9"/>
       <c r="J118" s="26" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="K118" s="46"/>
     </row>
-    <row r="119" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A119" s="55" t="s">
+        <v>402</v>
+      </c>
+      <c r="B119" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="C119" s="5" t="s">
         <v>408</v>
-      </c>
-      <c r="B119" s="5" t="s">
-        <v>413</v>
-      </c>
-      <c r="C119" s="5" t="s">
-        <v>414</v>
       </c>
       <c r="D119" s="6" t="s">
         <v>100</v>
       </c>
       <c r="E119" s="6" t="s">
-        <v>415</v>
+        <v>409</v>
       </c>
       <c r="F119" s="6"/>
       <c r="G119" s="7"/>
       <c r="H119" s="8"/>
       <c r="I119" s="9"/>
       <c r="J119" s="23" t="s">
+        <v>410</v>
+      </c>
+      <c r="K119" s="48"/>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A120" s="55" t="s">
+        <v>413</v>
+      </c>
+      <c r="B120" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="C120" s="5" t="s">
         <v>416</v>
-      </c>
-      <c r="K119" s="48"/>
-    </row>
-    <row r="120" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A120" s="55" t="s">
-        <v>419</v>
-      </c>
-      <c r="B120" s="5" t="s">
-        <v>390</v>
-      </c>
-      <c r="C120" s="5" t="s">
-        <v>422</v>
       </c>
       <c r="D120" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
       <c r="F120" s="6"/>
       <c r="G120" s="7"/>
@@ -5609,63 +5640,107 @@
       </c>
       <c r="I120" s="9"/>
       <c r="J120" s="26" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
       <c r="K120" s="46"/>
     </row>
-    <row r="121" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A121" s="55"/>
-      <c r="B121" s="5"/>
-      <c r="C121" s="5"/>
-      <c r="D121" s="6"/>
-      <c r="E121" s="6"/>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A121" s="55" t="s">
+        <v>427</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C121" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="D121" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E121" s="6" t="s">
+        <v>431</v>
+      </c>
       <c r="F121" s="6"/>
       <c r="G121" s="19"/>
-      <c r="H121" s="18"/>
+      <c r="H121" s="18" t="s">
+        <v>166</v>
+      </c>
       <c r="I121" s="9"/>
-      <c r="J121" s="24"/>
+      <c r="J121" s="24" t="s">
+        <v>433</v>
+      </c>
       <c r="K121" s="49"/>
     </row>
-    <row r="122" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A122" s="55"/>
-      <c r="B122" s="5"/>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A122" s="55" t="s">
+        <v>427</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>194</v>
+      </c>
       <c r="C122" s="5"/>
-      <c r="D122" s="6"/>
+      <c r="D122" s="54" t="s">
+        <v>100</v>
+      </c>
       <c r="E122" s="6"/>
       <c r="F122" s="6"/>
       <c r="G122" s="7"/>
       <c r="H122" s="8"/>
       <c r="I122" s="9"/>
-      <c r="J122" s="26"/>
+      <c r="J122" s="26" t="s">
+        <v>434</v>
+      </c>
       <c r="K122" s="46"/>
     </row>
-    <row r="123" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A123" s="55"/>
-      <c r="B123" s="5"/>
-      <c r="C123" s="5"/>
-      <c r="D123" s="6"/>
-      <c r="E123" s="6"/>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A123" s="55" t="s">
+        <v>428</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C123" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="D123" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E123" s="6" t="s">
+        <v>432</v>
+      </c>
       <c r="F123" s="6"/>
       <c r="G123" s="7"/>
-      <c r="H123" s="8"/>
+      <c r="H123" s="8" t="s">
+        <v>166</v>
+      </c>
       <c r="I123" s="9"/>
-      <c r="J123" s="23"/>
+      <c r="J123" s="23" t="s">
+        <v>433</v>
+      </c>
       <c r="K123" s="48"/>
     </row>
-    <row r="124" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A124" s="55"/>
-      <c r="B124" s="5"/>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A124" s="55" t="s">
+        <v>428</v>
+      </c>
+      <c r="B124" s="5" t="s">
+        <v>194</v>
+      </c>
       <c r="C124" s="5"/>
-      <c r="D124" s="6"/>
+      <c r="D124" s="54" t="s">
+        <v>100</v>
+      </c>
       <c r="E124" s="6"/>
       <c r="F124" s="6"/>
       <c r="G124" s="7"/>
       <c r="H124" s="8"/>
       <c r="I124" s="9"/>
-      <c r="J124" s="26"/>
+      <c r="J124" s="26" t="s">
+        <v>434</v>
+      </c>
       <c r="K124" s="46"/>
     </row>
-    <row r="125" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A125" s="55"/>
       <c r="B125" s="5"/>
       <c r="C125" s="5"/>
@@ -5678,7 +5753,7 @@
       <c r="J125" s="23"/>
       <c r="K125" s="48"/>
     </row>
-    <row r="126" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A126" s="55"/>
       <c r="B126" s="5"/>
       <c r="C126" s="5"/>
@@ -5691,7 +5766,7 @@
       <c r="J126" s="26"/>
       <c r="K126" s="46"/>
     </row>
-    <row r="127" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A127" s="55"/>
       <c r="B127" s="5"/>
       <c r="C127" s="5"/>
@@ -5704,7 +5779,7 @@
       <c r="J127" s="23"/>
       <c r="K127" s="48"/>
     </row>
-    <row r="128" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A128" s="5"/>
       <c r="B128" s="5"/>
       <c r="C128" s="5"/>
@@ -5717,7 +5792,7 @@
       <c r="J128" s="26"/>
       <c r="K128" s="46"/>
     </row>
-    <row r="129" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A129" s="5"/>
       <c r="B129" s="5"/>
       <c r="C129" s="5"/>
@@ -5730,7 +5805,7 @@
       <c r="J129" s="24"/>
       <c r="K129" s="49"/>
     </row>
-    <row r="130" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A130" s="5"/>
       <c r="B130" s="5"/>
       <c r="C130" s="5"/>
@@ -5743,7 +5818,7 @@
       <c r="J130" s="26"/>
       <c r="K130" s="46"/>
     </row>
-    <row r="131" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A131" s="5"/>
       <c r="B131" s="5"/>
       <c r="C131" s="5"/>
@@ -5756,7 +5831,7 @@
       <c r="J131" s="23"/>
       <c r="K131" s="48"/>
     </row>
-    <row r="132" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A132" s="5"/>
       <c r="B132" s="5"/>
       <c r="C132" s="5"/>
@@ -5769,7 +5844,7 @@
       <c r="J132" s="28"/>
       <c r="K132" s="50"/>
     </row>
-    <row r="133" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A133" s="5"/>
       <c r="B133" s="5"/>
       <c r="C133" s="5"/>
@@ -5782,7 +5857,7 @@
       <c r="J133" s="6"/>
       <c r="K133" s="41"/>
     </row>
-    <row r="134" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A134" s="5"/>
       <c r="B134" s="5"/>
       <c r="C134" s="5"/>
@@ -5795,7 +5870,7 @@
       <c r="J134" s="6"/>
       <c r="K134" s="41"/>
     </row>
-    <row r="135" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A135" s="5"/>
       <c r="B135" s="5"/>
       <c r="C135" s="5"/>

</xml_diff>

<commit_message>
normailzed AVNET and ITNET
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AA44528-389F-8B4C-8014-14DDEEE92F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3D9B7E-ACE9-B443-90B5-295B495888B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="3500" windowWidth="30240" windowHeight="16140" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="485">
   <si>
     <t>NSCU-A004</t>
   </si>
@@ -164,9 +164,6 @@
     <t>Lobby (port14 on switch 50-80m in length)</t>
   </si>
   <si>
-    <t>Wireless Access Point</t>
-  </si>
-  <si>
     <t>NAHU-B005</t>
   </si>
   <si>
@@ -1358,9 +1355,6 @@
     <t>80:6d:97:20:a7:89</t>
   </si>
   <si>
-    <t>builtin AVNET</t>
-  </si>
-  <si>
     <t>80:6d: 97:20:a7:8e</t>
   </si>
   <si>
@@ -1544,16 +1538,19 @@
     <t>192.168.0.48</t>
   </si>
   <si>
-    <t>ITNET WAP</t>
-  </si>
-  <si>
     <t>MHPR-J001</t>
   </si>
   <si>
     <t>B0:F5:30:CA:16:B0</t>
   </si>
   <si>
-    <t>ITNET Modem</t>
+    <t>ITNet WAP</t>
+  </si>
+  <si>
+    <t>ITNet Modem</t>
+  </si>
+  <si>
+    <t>builtin AVNet</t>
   </si>
 </sst>
 </file>
@@ -2565,600 +2562,600 @@
   <sheetData>
     <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>143</v>
-      </c>
       <c r="K1" s="40" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="19" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I2" s="9"/>
       <c r="J2" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="K2" s="41"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="C3" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>190</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>191</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I3" s="9"/>
       <c r="J3" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="K3" s="41"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>194</v>
-      </c>
       <c r="D4" s="6" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I4" s="9"/>
       <c r="J4" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K4" s="41"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I5" s="9"/>
       <c r="J5" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K5" s="41"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I6" s="9"/>
       <c r="J6" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="K6" s="41"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I7" s="9"/>
       <c r="J7" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K7" s="41"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
       <c r="H8" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I8" s="9"/>
       <c r="J8" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K8" s="41"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
       <c r="H9" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K9" s="41"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
       <c r="H10" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I10" s="9"/>
       <c r="J10" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K10" s="41"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="29" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E11" s="29" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F11" s="29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I11" s="9"/>
       <c r="J11" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K11" s="44"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I12" s="9"/>
       <c r="J12" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K12" s="43"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>376</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>378</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>377</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I13" s="9"/>
       <c r="J13" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K13" s="43"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I14" s="9"/>
       <c r="J14" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K14" s="43"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I15" s="9"/>
       <c r="J15" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K15" s="43"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I16" s="9"/>
       <c r="J16" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K16" s="43"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="29" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F17" s="29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I17" s="9"/>
       <c r="J17" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K17" s="44"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="29" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E18" s="29" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F18" s="29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I18" s="9"/>
       <c r="J18" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K18" s="44"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I19" s="9"/>
       <c r="J19" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K19" s="43"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="29" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E20" s="29" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F20" s="29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I20" s="9"/>
       <c r="J20" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K20" s="44"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B21" s="29"/>
       <c r="C21" s="29" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E21" s="29" t="s">
+        <v>282</v>
+      </c>
+      <c r="F21" s="29" t="s">
         <v>283</v>
-      </c>
-      <c r="F21" s="29" t="s">
-        <v>284</v>
       </c>
       <c r="G21" s="7"/>
       <c r="H21" s="8"/>
@@ -3168,165 +3165,165 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
       <c r="H22" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K22" s="41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
       <c r="H23" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K23" s="41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="6"/>
       <c r="H24" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K24" s="41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C25" s="20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
       <c r="H25" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K25" s="41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="6"/>
       <c r="H26" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I26" s="9"/>
       <c r="J26" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K26" s="42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E27" s="6"/>
       <c r="F27" s="6"/>
@@ -3335,36 +3332,36 @@
       <c r="I27" s="9"/>
       <c r="J27" s="6"/>
       <c r="K27" s="41" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F28" s="19" t="str">
         <f>CONCATENATE("http://", E28)</f>
         <v>http://192.168.201.110</v>
       </c>
       <c r="G28" s="21" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I28" s="9"/>
       <c r="J28" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K28" s="42">
         <v>4</v>
@@ -3372,60 +3369,60 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="6"/>
       <c r="H29" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I29" s="9"/>
       <c r="J29" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K29" s="41" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
       <c r="H30" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I30" s="9"/>
       <c r="J30" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K30" s="41" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
@@ -3437,67 +3434,67 @@
         <v>5</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
       <c r="H31" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I31" s="9"/>
       <c r="J31" s="6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="K31" s="41"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F32" s="6"/>
       <c r="G32" s="6"/>
       <c r="H32" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I32" s="9"/>
       <c r="J32" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="K32" s="41"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="6"/>
       <c r="H33" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I33" s="9"/>
       <c r="J33" s="6">
@@ -3507,20 +3504,20 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G34" s="7"/>
       <c r="H34" s="8"/>
@@ -3530,20 +3527,20 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B35" s="29"/>
       <c r="C35" s="29" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E35" s="29" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F35" s="29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G35" s="19"/>
       <c r="H35" s="8"/>
@@ -3553,20 +3550,20 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B36" s="29"/>
       <c r="C36" s="29" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E36" s="29" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F36" s="29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G36" s="7"/>
       <c r="H36" s="8"/>
@@ -3576,20 +3573,20 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B37" s="29"/>
       <c r="C37" s="29" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E37" s="29" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F37" s="29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G37" s="7"/>
       <c r="H37" s="8"/>
@@ -3599,242 +3596,242 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B38" s="29"/>
       <c r="C38" s="29" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E38" s="29" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F38" s="29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G38" s="7"/>
       <c r="H38" s="8"/>
       <c r="I38" s="9"/>
       <c r="J38" s="6"/>
       <c r="K38" s="41" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B39" s="29"/>
       <c r="C39" s="29" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E39" s="29" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F39" s="29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G39" s="7"/>
       <c r="H39" s="8"/>
       <c r="I39" s="9"/>
       <c r="J39" s="6"/>
       <c r="K39" s="41" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B40" s="29"/>
       <c r="C40" s="29" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E40" s="29" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F40" s="29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G40" s="7"/>
       <c r="H40" s="8"/>
       <c r="I40" s="9"/>
       <c r="J40" s="6"/>
       <c r="K40" s="41" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B41" s="5"/>
       <c r="C41" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G41" s="7"/>
       <c r="H41" s="8"/>
       <c r="I41" s="9"/>
       <c r="J41" s="6"/>
       <c r="K41" s="41" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B42" s="5"/>
       <c r="C42" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G42" s="7"/>
       <c r="H42" s="8"/>
       <c r="I42" s="9"/>
       <c r="J42" s="6"/>
       <c r="K42" s="41" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G43" s="7"/>
       <c r="H43" s="8"/>
       <c r="I43" s="9"/>
       <c r="J43" s="6"/>
       <c r="K43" s="41" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G44" s="7"/>
       <c r="H44" s="8"/>
       <c r="I44" s="9"/>
       <c r="J44" s="6"/>
       <c r="K44" s="41" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B45" s="29"/>
       <c r="C45" s="29" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E45" s="29" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F45" s="29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G45" s="7"/>
       <c r="H45" s="8"/>
       <c r="I45" s="9"/>
       <c r="J45" s="6"/>
       <c r="K45" s="41" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B46" s="29"/>
       <c r="C46" s="29" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E46" s="29" t="s">
+        <v>271</v>
+      </c>
+      <c r="F46" s="29" t="s">
         <v>272</v>
-      </c>
-      <c r="F46" s="29" t="s">
-        <v>273</v>
       </c>
       <c r="G46" s="19"/>
       <c r="H46" s="8"/>
       <c r="I46" s="9"/>
       <c r="J46" s="6"/>
       <c r="K46" s="41" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F47" s="7" t="str">
         <f>CONCATENATE("http://", E47)</f>
@@ -3842,29 +3839,29 @@
       </c>
       <c r="G47" s="7"/>
       <c r="H47" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I47" s="9"/>
       <c r="J47" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="K47" s="41" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F48" s="7" t="str">
         <f>CONCATENATE("http://", E48)</f>
@@ -3872,29 +3869,29 @@
       </c>
       <c r="G48" s="7"/>
       <c r="H48" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I48" s="9"/>
       <c r="J48" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K48" s="41" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F49" s="7" t="str">
         <f>CONCATENATE("http://", E49)</f>
@@ -3902,40 +3899,40 @@
       </c>
       <c r="G49" s="7"/>
       <c r="H49" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I49" s="9"/>
       <c r="J49" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K49" s="42" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B50" s="5"/>
       <c r="C50" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="19" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H50" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I50" s="9"/>
       <c r="J50" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="K50" s="41">
         <v>22</v>
@@ -3943,24 +3940,24 @@
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" s="31" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B51" s="13"/>
       <c r="C51" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F51" s="6"/>
       <c r="G51" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H51" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I51" s="9"/>
       <c r="J51" s="6"/>
@@ -3968,31 +3965,31 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F52" s="7" t="str">
         <f>CONCATENATE("http://", E52)</f>
         <v>http://192.168.0.23</v>
       </c>
       <c r="G52" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H52" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I52" s="9"/>
       <c r="J52" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K52" s="42"/>
     </row>
@@ -4002,50 +3999,50 @@
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F53" s="7" t="str">
         <f>CONCATENATE("http://", E53)</f>
         <v>http://192.168.0.22</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H53" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I53" s="9"/>
       <c r="J53" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K53" s="42"/>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E54" s="6"/>
       <c r="F54" s="19"/>
       <c r="G54" s="7"/>
       <c r="H54" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I54" s="9"/>
       <c r="J54" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K54" s="42"/>
     </row>
@@ -4055,27 +4052,27 @@
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F55" s="7" t="str">
         <f>CONCATENATE("http://", E55)</f>
         <v>http://192.168.0.24</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H55" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I55" s="9"/>
       <c r="J55" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K55" s="42"/>
     </row>
@@ -4085,135 +4082,135 @@
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F56" s="7" t="str">
         <f>CONCATENATE("http://", E56)</f>
         <v>http://192.168.0.25</v>
       </c>
       <c r="G56" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H56" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I56" s="9"/>
       <c r="J56" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K56" s="41"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F57" s="7" t="str">
         <f>CONCATENATE("http://", E57)</f>
         <v>http://192.168.0.26</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H57" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I57" s="9"/>
       <c r="J57" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K57" s="42"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B58" s="10"/>
       <c r="C58" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F58" s="6" t="str">
         <f>CONCATENATE("http://", E58, ":8080")</f>
         <v>http://192.168.0.197:8080</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H58" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I58" s="9"/>
       <c r="J58" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K58" s="41"/>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B59" s="6"/>
       <c r="C59" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F59" s="7" t="str">
         <f>CONCATENATE("http://", E59)</f>
         <v>http://192.168.0.193</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H59" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I59" s="9"/>
       <c r="J59" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K59" s="41" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F60" s="7" t="str">
         <f>CONCATENATE("http://", E60)</f>
@@ -4221,29 +4218,29 @@
       </c>
       <c r="G60" s="7"/>
       <c r="H60" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I60" s="9"/>
       <c r="J60" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K60" s="41" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F61" s="7" t="str">
         <f>CONCATENATE("http://", E61)</f>
@@ -4251,40 +4248,40 @@
       </c>
       <c r="G61" s="7"/>
       <c r="H61" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I61" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J61" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K61" s="41" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B62" s="5"/>
       <c r="C62" s="5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F62" s="6"/>
       <c r="G62" s="19"/>
       <c r="H62" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I62" s="9"/>
       <c r="J62" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="K62" s="41">
         <v>12</v>
@@ -4295,23 +4292,23 @@
         <v>3</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C63" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E63" s="6" t="s">
         <v>179</v>
-      </c>
-      <c r="D63" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E63" s="6" t="s">
-        <v>180</v>
       </c>
       <c r="F63" s="7"/>
       <c r="G63" s="7" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H63" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I63" s="9"/>
       <c r="J63" s="6"/>
@@ -4319,22 +4316,22 @@
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" s="17" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B64" s="5"/>
       <c r="C64" s="6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F64" s="6"/>
       <c r="G64" s="6"/>
       <c r="H64" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I64" s="9"/>
       <c r="J64" s="6" t="s">
@@ -4344,26 +4341,26 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B65" s="5"/>
       <c r="C65" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F65" s="6"/>
       <c r="G65" s="6"/>
       <c r="H65" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I65" s="9"/>
       <c r="J65" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K65" s="41">
         <v>6</v>
@@ -4371,17 +4368,17 @@
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B66" s="5"/>
       <c r="C66" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F66" s="7" t="str">
         <f>CONCATENATE("http://", E66)</f>
@@ -4389,11 +4386,11 @@
       </c>
       <c r="G66" s="7"/>
       <c r="H66" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I66" s="9"/>
       <c r="J66" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K66" s="41"/>
     </row>
@@ -4402,27 +4399,27 @@
         <v>1</v>
       </c>
       <c r="B67" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C67" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E67" s="6" t="s">
         <v>175</v>
-      </c>
-      <c r="C67" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="D67" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E67" s="6" t="s">
-        <v>176</v>
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="H67" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I67" s="9"/>
       <c r="J67" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K67" s="41"/>
     </row>
@@ -4431,218 +4428,218 @@
         <v>1</v>
       </c>
       <c r="B68" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C68" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E68" s="14" t="s">
         <v>170</v>
-      </c>
-      <c r="C68" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="D68" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E68" s="14" t="s">
-        <v>171</v>
       </c>
       <c r="F68" s="6"/>
       <c r="G68" s="6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="H68" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I68" s="9"/>
       <c r="J68" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K68" s="41"/>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B69" s="5"/>
       <c r="C69" s="53" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F69" s="6"/>
       <c r="G69" s="19" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H69" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I69" s="9"/>
       <c r="J69" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="K69" s="44" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B70" s="5"/>
       <c r="C70" s="53" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="D70" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F70" s="6"/>
       <c r="G70" s="19" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H70" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I70" s="9"/>
       <c r="J70" s="38" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="K70" s="43" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A71" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B71" s="6"/>
       <c r="C71" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F71" s="6"/>
       <c r="G71" s="6"/>
       <c r="H71" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I71" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K71" s="42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A72" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B72" s="6"/>
       <c r="C72" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F72" s="7" t="str">
         <f>CONCATENATE("http://", E72)</f>
         <v>http://192.168.0.183</v>
       </c>
       <c r="G72" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H72" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I72" s="9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K72" s="41" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="73" spans="1:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B73" s="5"/>
       <c r="C73" s="5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F73" s="6"/>
       <c r="G73" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H73" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I73" s="9"/>
       <c r="J73" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K73" s="41"/>
     </row>
     <row r="74" spans="1:11" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A74" s="22" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B74" s="5"/>
       <c r="C74" s="5" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F74" s="6"/>
       <c r="G74" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H74" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I74" s="9"/>
       <c r="J74" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K74" s="41"/>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A75" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B75" s="30"/>
       <c r="C75" s="33" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E75" s="33" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F75" s="36" t="str">
         <f>CONCATENATE("ftp://", E75)</f>
@@ -4650,31 +4647,31 @@
       </c>
       <c r="G75" s="7"/>
       <c r="H75" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I75" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K75" s="42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A76" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B76" s="30"/>
       <c r="C76" s="33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E76" s="33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F76" s="36" t="str">
         <f>CONCATENATE("ftp://", E76)</f>
@@ -4682,40 +4679,40 @@
       </c>
       <c r="G76" s="7"/>
       <c r="H76" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I76" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J76" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K76" s="42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B77" s="25"/>
       <c r="C77" s="33" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D77" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E77" s="33" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F77" s="33"/>
       <c r="G77" s="6"/>
       <c r="H77" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I77" s="9"/>
       <c r="J77" s="6" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="K77" s="41">
         <v>18</v>
@@ -4723,53 +4720,53 @@
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B78" s="30"/>
       <c r="C78" s="33" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E78" s="33" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F78" s="33"/>
       <c r="G78" s="6"/>
       <c r="H78" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I78" s="9"/>
       <c r="J78" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K78" s="41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B79" s="25"/>
       <c r="C79" s="26" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D79" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E79" s="26" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F79" s="26" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G79" s="7"/>
       <c r="H79" s="8"/>
       <c r="I79" s="9"/>
       <c r="J79" s="29" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="K79" s="43">
         <v>14</v>
@@ -4777,109 +4774,109 @@
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80" s="5" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B80" s="25" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C80" s="34" t="s">
+        <v>171</v>
+      </c>
+      <c r="D80" s="54" t="s">
+        <v>99</v>
+      </c>
+      <c r="E80" s="34" t="s">
         <v>172</v>
-      </c>
-      <c r="D80" s="54" t="s">
-        <v>100</v>
-      </c>
-      <c r="E80" s="34" t="s">
-        <v>173</v>
       </c>
       <c r="F80" s="33"/>
       <c r="G80" s="6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H80" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I80" s="9"/>
       <c r="J80" s="6" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="K80" s="41"/>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B81" s="27"/>
       <c r="C81" s="28" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E81" s="35" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F81" s="35"/>
       <c r="G81" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H81" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I81" s="9"/>
       <c r="J81" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K81" s="41"/>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B82" s="25"/>
       <c r="C82" s="26" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D82" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E82" s="33" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F82" s="33"/>
       <c r="G82" s="19"/>
       <c r="H82" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I82" s="9"/>
       <c r="J82" s="6" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="K82" s="41"/>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A83" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B83" s="25" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C83" s="26" t="s">
+        <v>183</v>
+      </c>
+      <c r="D83" s="54" t="s">
+        <v>99</v>
+      </c>
+      <c r="E83" s="33" t="s">
         <v>184</v>
-      </c>
-      <c r="D83" s="54" t="s">
-        <v>100</v>
-      </c>
-      <c r="E83" s="33" t="s">
-        <v>185</v>
       </c>
       <c r="F83" s="36"/>
       <c r="G83" s="7"/>
       <c r="H83" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I83" s="9"/>
       <c r="J83" s="6" t="s">
-        <v>420</v>
+        <v>484</v>
       </c>
       <c r="K83" s="41">
         <v>10</v>
@@ -4887,57 +4884,57 @@
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B84" s="25" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C84" s="26" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E84" s="33" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F84" s="36"/>
       <c r="G84" s="7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H84" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I84" s="9"/>
       <c r="J84" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K84" s="41"/>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B85" s="25"/>
       <c r="C85" s="23" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D85" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E85" s="33" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F85" s="33"/>
       <c r="G85" s="19" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H85" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I85" s="9"/>
       <c r="J85" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="K85" s="44">
         <v>4</v>
@@ -4945,66 +4942,66 @@
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86" s="30" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B86" s="6"/>
       <c r="C86" s="33" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E86" s="33" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F86" s="36" t="str">
         <f>CONCATENATE("http://", E86)</f>
         <v>http://192.168.0.195</v>
       </c>
       <c r="G86" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H86" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I86" s="9"/>
       <c r="J86" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K86" s="41" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" s="52" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B87" s="6"/>
       <c r="C87" s="35" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E87" s="35" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F87" s="37" t="str">
         <f>CONCATENATE("http://", E87)</f>
         <v>http://192.168.0.194</v>
       </c>
       <c r="G87" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H87" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I87" s="9"/>
       <c r="J87" s="35" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K87" s="45" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.2">
@@ -5016,13 +5013,13 @@
         <v>16</v>
       </c>
       <c r="D88" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E88" s="33"/>
       <c r="F88" s="33"/>
       <c r="G88" s="6"/>
       <c r="H88" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I88" s="9"/>
       <c r="J88" s="33" t="s">
@@ -5034,17 +5031,17 @@
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B89" s="30"/>
       <c r="C89" s="33" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E89" s="33" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F89" s="36" t="str">
         <f>CONCATENATE("http://", E89)</f>
@@ -5052,67 +5049,67 @@
       </c>
       <c r="G89" s="7"/>
       <c r="H89" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I89" s="9"/>
       <c r="J89" s="33" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K89" s="47" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A90" s="5" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B90" s="25"/>
       <c r="C90" s="26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E90" s="33" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F90" s="33"/>
       <c r="G90" s="19" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H90" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I90" s="9"/>
       <c r="J90" s="33" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="K90" s="47"/>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91" s="25" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B91" s="5"/>
       <c r="C91" s="26" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E91" s="33" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F91" s="33"/>
       <c r="G91" s="19" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H91" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I91" s="9"/>
       <c r="J91" s="33" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="K91" s="47">
         <v>13</v>
@@ -5127,13 +5124,13 @@
         <v>12</v>
       </c>
       <c r="D92" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E92" s="33"/>
       <c r="F92" s="33"/>
       <c r="G92" s="6"/>
       <c r="H92" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I92" s="9"/>
       <c r="J92" s="33" t="s">
@@ -5145,26 +5142,26 @@
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A93" s="25" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B93" s="5"/>
       <c r="C93" s="33" t="s">
+        <v>153</v>
+      </c>
+      <c r="D93" s="54" t="s">
+        <v>99</v>
+      </c>
+      <c r="E93" s="33" t="s">
         <v>154</v>
-      </c>
-      <c r="D93" s="54" t="s">
-        <v>100</v>
-      </c>
-      <c r="E93" s="33" t="s">
-        <v>155</v>
       </c>
       <c r="F93" s="33"/>
       <c r="G93" s="6"/>
       <c r="H93" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I93" s="9"/>
       <c r="J93" s="33" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K93" s="47"/>
     </row>
@@ -5173,25 +5170,25 @@
         <v>3</v>
       </c>
       <c r="B94" s="25" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C94" s="26" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D94" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E94" s="33" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F94" s="36"/>
       <c r="G94" s="7"/>
       <c r="H94" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I94" s="9"/>
       <c r="J94" s="26" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K94" s="47"/>
     </row>
@@ -5202,15 +5199,15 @@
       <c r="B95" s="30"/>
       <c r="C95" s="33"/>
       <c r="D95" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E95" s="34" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F95" s="33"/>
       <c r="G95" s="6"/>
       <c r="H95" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I95" s="9"/>
       <c r="J95" s="33" t="s">
@@ -5220,40 +5217,40 @@
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A96" s="25" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B96" s="5"/>
       <c r="C96" s="26"/>
       <c r="D96" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E96" s="34" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F96" s="33"/>
       <c r="G96" s="19" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="H96" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I96" s="9"/>
       <c r="J96" s="33" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="K96" s="47"/>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" s="25" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B97" s="5"/>
       <c r="C97" s="26"/>
       <c r="D97" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E97" s="33" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F97" s="33"/>
       <c r="G97" s="19"/>
@@ -5264,20 +5261,20 @@
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" s="25" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B98" s="5"/>
       <c r="C98" s="26"/>
       <c r="D98" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E98" s="33" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F98" s="33"/>
       <c r="G98" s="19"/>
       <c r="H98" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I98" s="9"/>
       <c r="J98" s="33"/>
@@ -5290,7 +5287,7 @@
       <c r="B99" s="5"/>
       <c r="C99" s="35"/>
       <c r="D99" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E99" s="35" t="s">
         <v>4</v>
@@ -5306,18 +5303,18 @@
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" s="25" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B100" s="5"/>
       <c r="C100" s="26"/>
       <c r="D100" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E100" s="33"/>
       <c r="F100" s="33"/>
       <c r="G100" s="19"/>
       <c r="H100" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I100" s="9"/>
       <c r="J100" s="33"/>
@@ -5328,159 +5325,159 @@
         <v>3</v>
       </c>
       <c r="B101" s="25" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C101" s="26" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D101" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E101" s="33" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="F101" s="36"/>
       <c r="G101" s="7"/>
       <c r="H101" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I101" s="9"/>
       <c r="J101" s="33" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="K101" s="47"/>
     </row>
     <row r="102" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A102" s="5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B102" s="25" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C102" s="26" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="D102" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E102" s="33" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="F102" s="36"/>
       <c r="G102" s="7"/>
       <c r="H102" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I102" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="J102" s="33" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="K102" s="47"/>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" s="30" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B103" s="6"/>
       <c r="C103" s="33"/>
       <c r="D103" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E103" s="33"/>
       <c r="F103" s="33"/>
       <c r="G103" s="6"/>
       <c r="H103" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I103" s="9"/>
       <c r="J103" s="33" t="s">
-        <v>22</v>
+        <v>482</v>
       </c>
       <c r="K103" s="47"/>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" s="30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B104" s="6"/>
       <c r="C104" s="33"/>
       <c r="D104" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E104" s="33"/>
       <c r="F104" s="33"/>
       <c r="G104" s="6"/>
       <c r="H104" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I104" s="9"/>
       <c r="J104" s="33" t="s">
-        <v>22</v>
+        <v>482</v>
       </c>
       <c r="K104" s="47"/>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A105" s="30" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B105" s="6"/>
       <c r="C105" s="33"/>
       <c r="D105" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E105" s="33"/>
       <c r="F105" s="33"/>
       <c r="G105" s="6"/>
       <c r="H105" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I105" s="9"/>
       <c r="J105" s="33" t="s">
-        <v>22</v>
+        <v>482</v>
       </c>
       <c r="K105" s="47"/>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A106" s="30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B106" s="6"/>
       <c r="C106" s="33"/>
       <c r="D106" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E106" s="33"/>
       <c r="F106" s="33"/>
       <c r="G106" s="6"/>
       <c r="H106" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I106" s="9"/>
       <c r="J106" s="33" t="s">
-        <v>22</v>
+        <v>482</v>
       </c>
       <c r="K106" s="47"/>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A107" s="30" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B107" s="6"/>
       <c r="C107" s="33"/>
       <c r="D107" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E107" s="33"/>
       <c r="F107" s="33"/>
       <c r="G107" s="6"/>
       <c r="H107" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I107" s="9"/>
       <c r="J107" s="33" t="s">
-        <v>22</v>
+        <v>482</v>
       </c>
       <c r="K107" s="47" t="s">
         <v>21</v>
@@ -5488,154 +5485,154 @@
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A108" s="30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B108" s="6"/>
       <c r="C108" s="33"/>
       <c r="D108" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E108" s="33"/>
       <c r="F108" s="33"/>
       <c r="G108" s="6"/>
       <c r="H108" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I108" s="9"/>
       <c r="J108" s="33" t="s">
-        <v>22</v>
+        <v>482</v>
       </c>
       <c r="K108" s="47"/>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A109" s="30" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B109" s="6"/>
       <c r="C109" s="33"/>
       <c r="D109" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E109" s="33"/>
       <c r="F109" s="33"/>
       <c r="G109" s="6"/>
       <c r="H109" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I109" s="9"/>
       <c r="J109" s="33" t="s">
-        <v>22</v>
+        <v>482</v>
       </c>
       <c r="K109" s="47"/>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A110" s="30" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B110" s="6"/>
       <c r="C110" s="33"/>
       <c r="D110" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E110" s="33"/>
       <c r="F110" s="33"/>
       <c r="G110" s="6"/>
       <c r="H110" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I110" s="9"/>
       <c r="J110" s="33" t="s">
-        <v>22</v>
+        <v>482</v>
       </c>
       <c r="K110" s="47"/>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A111" s="30" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B111" s="6"/>
       <c r="C111" s="33"/>
       <c r="D111" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E111" s="33"/>
       <c r="F111" s="33"/>
       <c r="G111" s="6"/>
       <c r="H111" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I111" s="9"/>
       <c r="J111" s="33" t="s">
-        <v>22</v>
+        <v>482</v>
       </c>
       <c r="K111" s="47"/>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A112" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C112" s="5"/>
       <c r="D112" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E112" s="6"/>
       <c r="F112" s="6"/>
       <c r="G112" s="7"/>
       <c r="H112" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I112" s="9"/>
       <c r="J112" s="35" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K112" s="45"/>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A113" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C113" s="5"/>
       <c r="D113" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E113" s="6"/>
       <c r="F113" s="6"/>
       <c r="G113" s="7"/>
       <c r="H113" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I113" s="9"/>
       <c r="J113" s="39" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K113" s="47"/>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A114" s="55" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C114" s="5" t="s">
+        <v>382</v>
+      </c>
+      <c r="D114" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="E114" s="6" t="s">
         <v>383</v>
-      </c>
-      <c r="D114" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="E114" s="6" t="s">
-        <v>384</v>
       </c>
       <c r="F114" s="6"/>
       <c r="G114" s="7"/>
       <c r="H114" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I114" s="9"/>
       <c r="J114" s="26"/>
@@ -5643,558 +5640,558 @@
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A115" s="55" t="s">
+        <v>380</v>
+      </c>
+      <c r="B115" s="5" t="s">
         <v>381</v>
       </c>
-      <c r="B115" s="5" t="s">
-        <v>382</v>
-      </c>
       <c r="C115" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="D115" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E115" s="6" t="s">
         <v>387</v>
-      </c>
-      <c r="D115" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E115" s="6" t="s">
-        <v>388</v>
       </c>
       <c r="F115" s="6"/>
       <c r="G115" s="7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="H115" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I115" s="9"/>
       <c r="J115" s="23" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="K115" s="48"/>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A116" s="55" t="s">
+        <v>389</v>
+      </c>
+      <c r="B116" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C116" s="5" t="s">
         <v>390</v>
       </c>
-      <c r="B116" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C116" s="5" t="s">
-        <v>391</v>
-      </c>
       <c r="D116" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F116" s="6"/>
       <c r="G116" s="7"/>
       <c r="H116" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I116" s="9"/>
       <c r="J116" s="26" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="K116" s="46" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A117" s="55" t="s">
+        <v>391</v>
+      </c>
+      <c r="B117" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C117" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="B117" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C117" s="5" t="s">
-        <v>393</v>
-      </c>
       <c r="D117" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F117" s="6"/>
       <c r="G117" s="7"/>
       <c r="H117" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I117" s="9"/>
       <c r="J117" s="23" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="K117" s="48"/>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A118" s="55" t="s">
+        <v>399</v>
+      </c>
+      <c r="B118" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="C118" s="5" t="s">
         <v>400</v>
       </c>
-      <c r="B118" s="5" t="s">
-        <v>404</v>
-      </c>
-      <c r="C118" s="5" t="s">
+      <c r="D118" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E118" s="6" t="s">
         <v>401</v>
-      </c>
-      <c r="D118" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E118" s="6" t="s">
-        <v>402</v>
       </c>
       <c r="F118" s="6"/>
       <c r="G118" s="7"/>
       <c r="H118" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I118" s="9"/>
       <c r="J118" s="26" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="K118" s="46"/>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A119" s="55" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B119" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="C119" s="5" t="s">
         <v>405</v>
       </c>
-      <c r="C119" s="5" t="s">
+      <c r="D119" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E119" s="6" t="s">
         <v>406</v>
-      </c>
-      <c r="D119" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E119" s="6" t="s">
-        <v>407</v>
       </c>
       <c r="F119" s="6"/>
       <c r="G119" s="7"/>
       <c r="H119" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I119" s="9"/>
       <c r="J119" s="23" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="K119" s="48"/>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A120" s="55" t="s">
+        <v>410</v>
+      </c>
+      <c r="B120" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C120" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D120" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E120" s="6" t="s">
         <v>411</v>
-      </c>
-      <c r="B120" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C120" s="5" t="s">
-        <v>414</v>
-      </c>
-      <c r="D120" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E120" s="6" t="s">
-        <v>412</v>
       </c>
       <c r="F120" s="6"/>
       <c r="G120" s="7"/>
       <c r="H120" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I120" s="9"/>
       <c r="J120" s="26" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="K120" s="46"/>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A121" s="55" t="s">
+        <v>423</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="C121" s="5" t="s">
         <v>425</v>
       </c>
-      <c r="B121" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="C121" s="5" t="s">
+      <c r="D121" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E121" s="6" t="s">
         <v>427</v>
-      </c>
-      <c r="D121" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E121" s="6" t="s">
-        <v>429</v>
       </c>
       <c r="F121" s="6"/>
       <c r="G121" s="19"/>
       <c r="H121" s="18" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I121" s="9"/>
       <c r="J121" s="24" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="K121" s="49"/>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A122" s="55" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C122" s="5"/>
       <c r="D122" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E122" s="6"/>
       <c r="F122" s="6"/>
       <c r="G122" s="7"/>
       <c r="H122" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I122" s="9"/>
       <c r="J122" s="26" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="K122" s="46"/>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A123" s="55" t="s">
+        <v>424</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="C123" s="5" t="s">
         <v>426</v>
       </c>
-      <c r="B123" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="C123" s="5" t="s">
+      <c r="D123" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E123" s="6" t="s">
         <v>428</v>
-      </c>
-      <c r="D123" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E123" s="6" t="s">
-        <v>430</v>
       </c>
       <c r="F123" s="6"/>
       <c r="G123" s="7"/>
       <c r="H123" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I123" s="9"/>
       <c r="J123" s="23" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="K123" s="48"/>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A124" s="55" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C124" s="5"/>
       <c r="D124" s="54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E124" s="6"/>
       <c r="F124" s="6"/>
       <c r="G124" s="7"/>
       <c r="H124" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I124" s="9"/>
       <c r="J124" s="26" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="K124" s="46"/>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A125" s="55" t="s">
+        <v>436</v>
+      </c>
+      <c r="B125" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C125" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="D125" s="54" t="s">
+        <v>99</v>
+      </c>
+      <c r="E125" s="54" t="s">
         <v>438</v>
-      </c>
-      <c r="B125" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C125" s="5" t="s">
-        <v>439</v>
-      </c>
-      <c r="D125" s="54" t="s">
-        <v>100</v>
-      </c>
-      <c r="E125" s="54" t="s">
-        <v>440</v>
       </c>
       <c r="F125" s="6"/>
       <c r="G125" s="7"/>
       <c r="H125" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I125" s="9"/>
       <c r="J125" s="23" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="K125" s="48"/>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A126" s="55" t="s">
+        <v>440</v>
+      </c>
+      <c r="B126" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C126" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="D126" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E126" s="6" t="s">
         <v>442</v>
-      </c>
-      <c r="B126" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C126" s="5" t="s">
-        <v>443</v>
-      </c>
-      <c r="D126" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E126" s="6" t="s">
-        <v>444</v>
       </c>
       <c r="F126" s="6"/>
       <c r="G126" s="7"/>
       <c r="H126" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I126" s="9"/>
       <c r="J126" s="26" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="K126" s="46"/>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A127" s="55" t="s">
+        <v>444</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C127" s="5" t="s">
         <v>446</v>
       </c>
-      <c r="B127" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C127" s="5" t="s">
-        <v>448</v>
-      </c>
       <c r="D127" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="F127" s="6"/>
       <c r="G127" s="7"/>
       <c r="H127" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I127" s="9"/>
       <c r="J127" s="23" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="K127" s="48"/>
     </row>
     <row r="128" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A128" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="B128" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C128" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="D128" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E128" s="6" t="s">
         <v>450</v>
-      </c>
-      <c r="B128" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C128" s="5" t="s">
-        <v>451</v>
-      </c>
-      <c r="D128" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E128" s="6" t="s">
-        <v>452</v>
       </c>
       <c r="F128" s="6"/>
       <c r="G128" s="7"/>
       <c r="H128" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I128" s="9"/>
       <c r="J128" s="26" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="K128" s="46"/>
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A129" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C129" s="5" t="s">
+        <v>453</v>
+      </c>
+      <c r="D129" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E129" s="6" t="s">
         <v>454</v>
-      </c>
-      <c r="B129" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C129" s="5" t="s">
-        <v>455</v>
-      </c>
-      <c r="D129" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E129" s="6" t="s">
-        <v>456</v>
       </c>
       <c r="F129" s="6"/>
       <c r="G129" s="19"/>
       <c r="H129" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I129" s="9"/>
       <c r="J129" s="24" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="K129" s="49"/>
     </row>
     <row r="130" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A130" s="56" t="s">
+        <v>456</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C130" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="D130" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E130" t="s">
         <v>458</v>
-      </c>
-      <c r="B130" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C130" s="5" t="s">
-        <v>459</v>
-      </c>
-      <c r="D130" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E130" t="s">
-        <v>460</v>
       </c>
       <c r="F130" s="6"/>
       <c r="G130" s="7"/>
       <c r="H130" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I130" s="9"/>
       <c r="J130" s="26" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="K130" s="46"/>
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A131" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C131" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="D131" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E131" s="6" t="s">
         <v>462</v>
-      </c>
-      <c r="B131" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C131" s="5" t="s">
-        <v>463</v>
-      </c>
-      <c r="D131" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E131" s="6" t="s">
-        <v>464</v>
       </c>
       <c r="F131" s="6"/>
       <c r="G131" s="7"/>
       <c r="H131" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I131" s="9"/>
       <c r="J131" s="23" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="K131" s="48"/>
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A132" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C132" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="D132" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E132" s="6" t="s">
         <v>466</v>
-      </c>
-      <c r="B132" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C132" s="5" t="s">
-        <v>467</v>
-      </c>
-      <c r="D132" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E132" s="6" t="s">
-        <v>468</v>
       </c>
       <c r="F132" s="6"/>
       <c r="G132" s="19"/>
       <c r="H132" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I132" s="9"/>
       <c r="J132" s="28" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="K132" s="50"/>
     </row>
     <row r="133" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A133" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C133" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="D133" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E133" s="6" t="s">
         <v>470</v>
-      </c>
-      <c r="B133" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C133" s="5" t="s">
-        <v>471</v>
-      </c>
-      <c r="D133" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E133" s="6" t="s">
-        <v>472</v>
       </c>
       <c r="F133" s="6"/>
       <c r="G133" s="19"/>
       <c r="H133" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I133" s="9"/>
       <c r="J133" s="6" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="K133" s="41"/>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A134" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="B134" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="C134" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D134" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E134" s="6" t="s">
         <v>474</v>
-      </c>
-      <c r="B134" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C134" s="5" t="s">
-        <v>475</v>
-      </c>
-      <c r="D134" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E134" s="6" t="s">
-        <v>476</v>
       </c>
       <c r="F134" s="6"/>
       <c r="G134" s="19"/>
       <c r="H134" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I134" s="9"/>
       <c r="J134" s="6" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="K134" s="41"/>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A135" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C135" s="5"/>
       <c r="D135" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E135" s="6" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="F135" s="6"/>
       <c r="G135" s="19"/>
       <c r="H135" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I135" s="9"/>
       <c r="J135" s="6" t="s">
@@ -6204,22 +6201,22 @@
     </row>
     <row r="136" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A136" s="57" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C136" s="57"/>
       <c r="D136" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E136" s="58" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="F136" s="58"/>
       <c r="G136" s="19"/>
       <c r="H136" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I136" s="59"/>
       <c r="J136" s="6" t="s">
@@ -6229,22 +6226,22 @@
     </row>
     <row r="137" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A137" s="57" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C137" s="57"/>
       <c r="D137" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E137" s="58" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="F137" s="58"/>
       <c r="G137" s="19"/>
       <c r="H137" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I137" s="59"/>
       <c r="J137" s="6" t="s">
@@ -6254,26 +6251,26 @@
     </row>
     <row r="138" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A138" s="61" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="B138" s="57" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C138" s="62" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="D138" s="58" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E138" s="58"/>
       <c r="F138" s="58"/>
       <c r="G138" s="19"/>
       <c r="H138" s="18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I138" s="59"/>
       <c r="J138" s="58" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="K138" s="60"/>
     </row>

</xml_diff>

<commit_message>
added grandma3 lighting network details
</commit_message>
<xml_diff>
--- a/network.xlsx
+++ b/network.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A2C339A-5777-1F49-9CEC-07B5B95411BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3C08F53-22A1-9F4C-BA6A-DE5BB5F776AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="3500" windowWidth="30240" windowHeight="16140" xr2:uid="{C276EF8E-8567-464E-98DC-2A8DA10DDBB6}"/>
   </bookViews>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="499">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="502">
   <si>
     <t>NSCU-A004</t>
   </si>
@@ -1583,9 +1583,6 @@
     <t>E8CF83FF3955</t>
   </si>
   <si>
-    <t>2607-2100</t>
-  </si>
-  <si>
     <t>192.168.0.81</t>
   </si>
   <si>
@@ -1593,6 +1590,18 @@
   </si>
   <si>
     <t>LAN2</t>
+  </si>
+  <si>
+    <t>2607-2500</t>
+  </si>
+  <si>
+    <t>e4-4f-29-00-0d-74</t>
+  </si>
+  <si>
+    <t>e4-4f-29-00-0d-73</t>
+  </si>
+  <si>
+    <t>Lighting Console - unused</t>
   </si>
 </sst>
 </file>
@@ -1888,7 +1897,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1978,12 +1987,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -6391,17 +6394,19 @@
     </row>
     <row r="142" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A142" s="55" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>497</v>
-      </c>
-      <c r="C142" s="5"/>
+        <v>496</v>
+      </c>
+      <c r="C142" s="5" t="s">
+        <v>499</v>
+      </c>
       <c r="D142" s="6" t="s">
         <v>487</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="F142" s="6"/>
       <c r="G142" s="19" t="s">
@@ -6418,24 +6423,28 @@
     </row>
     <row r="143" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A143" s="55" t="s">
-        <v>495</v>
-      </c>
-      <c r="B143" s="59" t="s">
         <v>498</v>
       </c>
-      <c r="C143" s="59"/>
-      <c r="D143" s="60"/>
-      <c r="E143" s="60"/>
-      <c r="F143" s="60"/>
+      <c r="B143" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="C143" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="D143" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="E143" s="6"/>
+      <c r="F143" s="6"/>
       <c r="G143" s="19"/>
       <c r="H143" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="I143" s="61"/>
+      <c r="I143" s="9"/>
       <c r="J143" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="K143" s="62"/>
+        <v>501</v>
+      </c>
+      <c r="K143" s="41"/>
     </row>
     <row r="144" spans="1:11" x14ac:dyDescent="0.2">
       <c r="H144"/>

</xml_diff>